<commit_message>
build: improve .gitignore and un-track temp files
Applied a standard Python .gitignore file to the repository.

Removed previously tracked temporary files (e.g., __pycache__, ~$*.xlsx) from the Git index to clean up the repository status.
</commit_message>
<xml_diff>
--- a/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
+++ b/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
@@ -14,9 +14,111 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>iteration</t>
+  </si>
+  <si>
+    <t>TC_03_04</t>
+  </si>
+  <si>
+    <t>TC_04_00</t>
+  </si>
+  <si>
+    <t>TC_04_01</t>
+  </si>
+  <si>
+    <t>TC_05_06</t>
+  </si>
+  <si>
+    <t>fomp_10_k1</t>
+  </si>
+  <si>
+    <t>fomp_10_k2</t>
+  </si>
+  <si>
+    <t>S_0_material_mc</t>
+  </si>
+  <si>
+    <t>S_0_WC_mc</t>
+  </si>
+  <si>
+    <t>S_0_DM_mc</t>
+  </si>
+  <si>
+    <t>S_0_CC_mc</t>
+  </si>
+  <si>
+    <t>S_1_material_mc</t>
+  </si>
+  <si>
+    <t>S_1_WC_mc</t>
+  </si>
+  <si>
+    <t>S_1_DM_mc</t>
+  </si>
+  <si>
+    <t>S_1_CC_mc</t>
+  </si>
+  <si>
+    <t>S_6_material_mc</t>
+  </si>
+  <si>
+    <t>S_6_WC_mc</t>
+  </si>
+  <si>
+    <t>S_6_DM_mc</t>
+  </si>
+  <si>
+    <t>S_6_CC_mc</t>
+  </si>
+  <si>
+    <t>S_9_material_mc</t>
+  </si>
+  <si>
+    <t>S_9_WC_mc</t>
+  </si>
+  <si>
+    <t>S_9_DM_mc</t>
+  </si>
+  <si>
+    <t>S_9_CC_mc</t>
+  </si>
+  <si>
+    <t>S_10_material_mc</t>
+  </si>
+  <si>
+    <t>S_10_WC_mc</t>
+  </si>
+  <si>
+    <t>S_10_DM_mc</t>
+  </si>
+  <si>
+    <t>S_10_CC_mc</t>
+  </si>
+  <si>
+    <t>S_11_material_mc</t>
+  </si>
+  <si>
+    <t>S_11_WC_mc</t>
+  </si>
+  <si>
+    <t>S_11_DM_mc</t>
+  </si>
+  <si>
+    <t>S_11_CC_mc</t>
+  </si>
+  <si>
+    <t>S_12_material_mc</t>
+  </si>
+  <si>
+    <t>S_12_WC_mc</t>
+  </si>
+  <si>
+    <t>S_12_DM_mc</t>
+  </si>
+  <si>
+    <t>S_12_CC_mc</t>
   </si>
 </sst>
 </file>
@@ -374,62 +476,1184 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:AI11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:35">
       <c r="A2">
         <v>0</v>
       </c>
+      <c r="B2">
+        <v>0.4044515164642742</v>
+      </c>
+      <c r="C2">
+        <v>0.4359011492442288</v>
+      </c>
+      <c r="D2">
+        <v>0.5920788225490751</v>
+      </c>
+      <c r="E2">
+        <v>0.2378725893416587</v>
+      </c>
+      <c r="F2">
+        <v>0.02780250391885774</v>
+      </c>
+      <c r="G2">
+        <v>0.03631416410733315</v>
+      </c>
+      <c r="H2">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="K2">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="L2">
+        <v>-11890474.67</v>
+      </c>
+      <c r="M2">
+        <v>-2834689.161328</v>
+      </c>
+      <c r="N2">
+        <v>-9055785.508672001</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>2091688.403242461</v>
+      </c>
+      <c r="Q2">
+        <v>292812.280201633</v>
+      </c>
+      <c r="R2">
+        <v>1798876.123040828</v>
+      </c>
+      <c r="S2">
+        <v>863448.9728664837</v>
+      </c>
+      <c r="T2">
+        <v>9.458744898438454E-11</v>
+      </c>
+      <c r="U2">
+        <v>1.000444171950221E-11</v>
+      </c>
+      <c r="V2">
+        <v>8.003553375601768E-11</v>
+      </c>
+      <c r="W2">
+        <v>3.637978807091713E-11</v>
+      </c>
+      <c r="X2">
+        <v>4073050.986513603</v>
+      </c>
+      <c r="Y2">
+        <v>570180.2163268673</v>
+      </c>
+      <c r="Z2">
+        <v>3502870.770186735</v>
+      </c>
+      <c r="AA2">
+        <v>1681355.448229763</v>
+      </c>
+      <c r="AB2">
+        <v>7528521.911194503</v>
+      </c>
+      <c r="AC2">
+        <v>1053906.33872858</v>
+      </c>
+      <c r="AD2">
+        <v>6474615.572465925</v>
+      </c>
+      <c r="AE2">
+        <v>3107773.846057842</v>
+      </c>
+      <c r="AF2">
+        <v>5879914.028609334</v>
+      </c>
+      <c r="AG2">
+        <v>823120.2270934064</v>
+      </c>
+      <c r="AH2">
+        <v>5056793.801515928</v>
+      </c>
+      <c r="AI2">
+        <v>2427228.512277931</v>
+      </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:35">
       <c r="A3">
         <v>1</v>
       </c>
+      <c r="B3">
+        <v>0.3533650501907114</v>
+      </c>
+      <c r="C3">
+        <v>0.418213397257845</v>
+      </c>
+      <c r="D3">
+        <v>0.570778593912088</v>
+      </c>
+      <c r="E3">
+        <v>0.223866727320552</v>
+      </c>
+      <c r="F3">
+        <v>0.01763152451303309</v>
+      </c>
+      <c r="G3">
+        <v>0.03114760930563983</v>
+      </c>
+      <c r="H3">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="K3">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="L3">
+        <v>-11890474.67</v>
+      </c>
+      <c r="M3">
+        <v>-2834689.161328</v>
+      </c>
+      <c r="N3">
+        <v>-9055785.508672001</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>1968530.458697262</v>
+      </c>
+      <c r="Q3">
+        <v>275571.5867449384</v>
+      </c>
+      <c r="R3">
+        <v>1692958.871952323</v>
+      </c>
+      <c r="S3">
+        <v>812609.3733577547</v>
+      </c>
+      <c r="T3">
+        <v>9.458744898438454E-11</v>
+      </c>
+      <c r="U3">
+        <v>1.000444171950221E-11</v>
+      </c>
+      <c r="V3">
+        <v>8.003553375601768E-11</v>
+      </c>
+      <c r="W3">
+        <v>3.637978807091713E-11</v>
+      </c>
+      <c r="X3">
+        <v>4073050.986513603</v>
+      </c>
+      <c r="Y3">
+        <v>570180.2163268673</v>
+      </c>
+      <c r="Z3">
+        <v>3502870.770186735</v>
+      </c>
+      <c r="AA3">
+        <v>1681355.448229763</v>
+      </c>
+      <c r="AB3">
+        <v>7090749.966614714</v>
+      </c>
+      <c r="AC3">
+        <v>992623.3096407818</v>
+      </c>
+      <c r="AD3">
+        <v>6098126.656973933</v>
+      </c>
+      <c r="AE3">
+        <v>2927061.587249019</v>
+      </c>
+      <c r="AF3">
+        <v>5257191.921396995</v>
+      </c>
+      <c r="AG3">
+        <v>735946.3058716153</v>
+      </c>
+      <c r="AH3">
+        <v>4521245.615525381</v>
+      </c>
+      <c r="AI3">
+        <v>2170168.826297938</v>
+      </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:35">
       <c r="A4">
         <v>2</v>
       </c>
+      <c r="B4">
+        <v>0.4784984181624737</v>
+      </c>
+      <c r="C4">
+        <v>0.5631245218631868</v>
+      </c>
+      <c r="D4">
+        <v>0.4166175163458492</v>
+      </c>
+      <c r="E4">
+        <v>0.2202218264624313</v>
+      </c>
+      <c r="F4">
+        <v>0.03205818281932218</v>
+      </c>
+      <c r="G4">
+        <v>0.03580641006815242</v>
+      </c>
+      <c r="H4">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="K4">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="L4">
+        <v>-11890474.67</v>
+      </c>
+      <c r="M4">
+        <v>-2834689.161328</v>
+      </c>
+      <c r="N4">
+        <v>-9055785.508672001</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>1936479.700444704</v>
+      </c>
+      <c r="Q4">
+        <v>271084.8498143446</v>
+      </c>
+      <c r="R4">
+        <v>1665394.85063036</v>
+      </c>
+      <c r="S4">
+        <v>799378.8203509763</v>
+      </c>
+      <c r="T4">
+        <v>9.458744898438454E-11</v>
+      </c>
+      <c r="U4">
+        <v>1.000444171950221E-11</v>
+      </c>
+      <c r="V4">
+        <v>8.003553375601768E-11</v>
+      </c>
+      <c r="W4">
+        <v>3.637978807091713E-11</v>
+      </c>
+      <c r="X4">
+        <v>4073050.986513603</v>
+      </c>
+      <c r="Y4">
+        <v>570180.2163268673</v>
+      </c>
+      <c r="Z4">
+        <v>3502870.770186735</v>
+      </c>
+      <c r="AA4">
+        <v>1681355.448229763</v>
+      </c>
+      <c r="AB4">
+        <v>8133940.781732601</v>
+      </c>
+      <c r="AC4">
+        <v>1138658.006155625</v>
+      </c>
+      <c r="AD4">
+        <v>6995282.775576978</v>
+      </c>
+      <c r="AE4">
+        <v>3357690.755912029</v>
+      </c>
+      <c r="AF4">
+        <v>6741110.639025928</v>
+      </c>
+      <c r="AG4">
+        <v>943677.8315342019</v>
+      </c>
+      <c r="AH4">
+        <v>5797432.807491727</v>
+      </c>
+      <c r="AI4">
+        <v>2782730.473194545</v>
+      </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:35">
       <c r="A5">
         <v>3</v>
       </c>
+      <c r="B5">
+        <v>0.4311242526405999</v>
+      </c>
+      <c r="C5">
+        <v>0.5191245799174347</v>
+      </c>
+      <c r="D5">
+        <v>0.4324618929214741</v>
+      </c>
+      <c r="E5">
+        <v>0.2049270997346183</v>
+      </c>
+      <c r="F5">
+        <v>0.02713418766765317</v>
+      </c>
+      <c r="G5">
+        <v>0.03620998988143376</v>
+      </c>
+      <c r="H5">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="K5">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="L5">
+        <v>-11890474.67</v>
+      </c>
+      <c r="M5">
+        <v>-2834689.161328</v>
+      </c>
+      <c r="N5">
+        <v>-9055785.508672001</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>1801988.363650203</v>
+      </c>
+      <c r="Q5">
+        <v>252257.612003437</v>
+      </c>
+      <c r="R5">
+        <v>1549730.751646766</v>
+      </c>
+      <c r="S5">
+        <v>743860.7965216924</v>
+      </c>
+      <c r="T5">
+        <v>9.458744898438454E-11</v>
+      </c>
+      <c r="U5">
+        <v>1.000444171950221E-11</v>
+      </c>
+      <c r="V5">
+        <v>8.003553375601768E-11</v>
+      </c>
+      <c r="W5">
+        <v>3.637978807091713E-11</v>
+      </c>
+      <c r="X5">
+        <v>4073050.986513603</v>
+      </c>
+      <c r="Y5">
+        <v>570180.2163268673</v>
+      </c>
+      <c r="Z5">
+        <v>3502870.770186735</v>
+      </c>
+      <c r="AA5">
+        <v>1681355.448229763</v>
+      </c>
+      <c r="AB5">
+        <v>7726211.372195898</v>
+      </c>
+      <c r="AC5">
+        <v>1081580.58588278</v>
+      </c>
+      <c r="AD5">
+        <v>6644630.786313119</v>
+      </c>
+      <c r="AE5">
+        <v>3189380.055573497</v>
+      </c>
+      <c r="AF5">
+        <v>6161123.455692711</v>
+      </c>
+      <c r="AG5">
+        <v>862486.3073476364</v>
+      </c>
+      <c r="AH5">
+        <v>5298637.148345075</v>
+      </c>
+      <c r="AI5">
+        <v>2543311.763798263</v>
+      </c>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:35">
       <c r="A6">
         <v>4</v>
       </c>
+      <c r="B6">
+        <v>0.4745448200553239</v>
+      </c>
+      <c r="C6">
+        <v>0.4971029394202924</v>
+      </c>
+      <c r="D6">
+        <v>0.5721971770724217</v>
+      </c>
+      <c r="E6">
+        <v>0.1561672667924529</v>
+      </c>
+      <c r="F6">
+        <v>0.02311293505053799</v>
+      </c>
+      <c r="G6">
+        <v>0.03335421799871998</v>
+      </c>
+      <c r="H6">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="K6">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="L6">
+        <v>-11890474.67</v>
+      </c>
+      <c r="M6">
+        <v>-2834689.161328</v>
+      </c>
+      <c r="N6">
+        <v>-9055785.508672001</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>1373227.835203282</v>
+      </c>
+      <c r="Q6">
+        <v>192236.0773425464</v>
+      </c>
+      <c r="R6">
+        <v>1180991.757860735</v>
+      </c>
+      <c r="S6">
+        <v>566868.4503771641</v>
+      </c>
+      <c r="T6">
+        <v>9.458744898438454E-11</v>
+      </c>
+      <c r="U6">
+        <v>1.000444171950221E-11</v>
+      </c>
+      <c r="V6">
+        <v>8.003553375601768E-11</v>
+      </c>
+      <c r="W6">
+        <v>3.637978807091713E-11</v>
+      </c>
+      <c r="X6">
+        <v>4073050.986513603</v>
+      </c>
+      <c r="Y6">
+        <v>570180.2163268673</v>
+      </c>
+      <c r="Z6">
+        <v>3502870.770186735</v>
+      </c>
+      <c r="AA6">
+        <v>1681355.448229763</v>
+      </c>
+      <c r="AB6">
+        <v>8051766.839898238</v>
+      </c>
+      <c r="AC6">
+        <v>1127154.60095569</v>
+      </c>
+      <c r="AD6">
+        <v>6924612.23894255</v>
+      </c>
+      <c r="AE6">
+        <v>3323769.352667995</v>
+      </c>
+      <c r="AF6">
+        <v>6624219.799284804</v>
+      </c>
+      <c r="AG6">
+        <v>927314.4605715044</v>
+      </c>
+      <c r="AH6">
+        <v>5696905.338713299</v>
+      </c>
+      <c r="AI6">
+        <v>2734477.934471445</v>
+      </c>
     </row>
-    <row r="7" spans="1:1">
+    <row r="7" spans="1:35">
       <c r="A7">
         <v>5</v>
       </c>
+      <c r="B7">
+        <v>0.4025120736132263</v>
+      </c>
+      <c r="C7">
+        <v>0.441611508003588</v>
+      </c>
+      <c r="D7">
+        <v>0.5017960914342195</v>
+      </c>
+      <c r="E7">
+        <v>0.1758284529126744</v>
+      </c>
+      <c r="F7">
+        <v>0.03037840208410895</v>
+      </c>
+      <c r="G7">
+        <v>0.03935885602922868</v>
+      </c>
+      <c r="H7">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="K7">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="L7">
+        <v>-11890474.67</v>
+      </c>
+      <c r="M7">
+        <v>-2834689.161328</v>
+      </c>
+      <c r="N7">
+        <v>-9055785.508672001</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <v>1546114.821112325</v>
+      </c>
+      <c r="Q7">
+        <v>216438.2637115773</v>
+      </c>
+      <c r="R7">
+        <v>1329676.557400748</v>
+      </c>
+      <c r="S7">
+        <v>638236.1981610783</v>
+      </c>
+      <c r="T7">
+        <v>9.458744898438454E-11</v>
+      </c>
+      <c r="U7">
+        <v>1.000444171950221E-11</v>
+      </c>
+      <c r="V7">
+        <v>8.003553375601768E-11</v>
+      </c>
+      <c r="W7">
+        <v>3.637978807091713E-11</v>
+      </c>
+      <c r="X7">
+        <v>4073050.986513603</v>
+      </c>
+      <c r="Y7">
+        <v>570180.2163268673</v>
+      </c>
+      <c r="Z7">
+        <v>3502870.770186735</v>
+      </c>
+      <c r="AA7">
+        <v>1681355.448229763</v>
+      </c>
+      <c r="AB7">
+        <v>7464726.106970938</v>
+      </c>
+      <c r="AC7">
+        <v>1044975.661076935</v>
+      </c>
+      <c r="AD7">
+        <v>6419750.445894002</v>
+      </c>
+      <c r="AE7">
+        <v>3081438.938024062</v>
+      </c>
+      <c r="AF7">
+        <v>5789165.733454103</v>
+      </c>
+      <c r="AG7">
+        <v>810416.5112090887</v>
+      </c>
+      <c r="AH7">
+        <v>4978749.222245014</v>
+      </c>
+      <c r="AI7">
+        <v>2389767.615966313</v>
+      </c>
     </row>
-    <row r="8" spans="1:1">
+    <row r="8" spans="1:35">
       <c r="A8">
         <v>6</v>
       </c>
+      <c r="B8">
+        <v>0.3482567793372362</v>
+      </c>
+      <c r="C8">
+        <v>0.4566197751584281</v>
+      </c>
+      <c r="D8">
+        <v>0.4893542101856769</v>
+      </c>
+      <c r="E8">
+        <v>0.2399113044565739</v>
+      </c>
+      <c r="F8">
+        <v>0.03308857409633047</v>
+      </c>
+      <c r="G8">
+        <v>0.0347419980722866</v>
+      </c>
+      <c r="H8">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="K8">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="L8">
+        <v>-11890474.67</v>
+      </c>
+      <c r="M8">
+        <v>-2834689.161328</v>
+      </c>
+      <c r="N8">
+        <v>-9055785.508672001</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <v>2109615.465688728</v>
+      </c>
+      <c r="Q8">
+        <v>295321.8624243346</v>
+      </c>
+      <c r="R8">
+        <v>1814293.603264394</v>
+      </c>
+      <c r="S8">
+        <v>870849.2642443714</v>
+      </c>
+      <c r="T8">
+        <v>9.458744898438454E-11</v>
+      </c>
+      <c r="U8">
+        <v>1.000444171950221E-11</v>
+      </c>
+      <c r="V8">
+        <v>8.003553375601768E-11</v>
+      </c>
+      <c r="W8">
+        <v>3.637978807091713E-11</v>
+      </c>
+      <c r="X8">
+        <v>4073050.986513603</v>
+      </c>
+      <c r="Y8">
+        <v>570180.2163268673</v>
+      </c>
+      <c r="Z8">
+        <v>3502870.770186735</v>
+      </c>
+      <c r="AA8">
+        <v>1681355.448229763</v>
+      </c>
+      <c r="AB8">
+        <v>7060355.28631501</v>
+      </c>
+      <c r="AC8">
+        <v>988368.4045444184</v>
+      </c>
+      <c r="AD8">
+        <v>6071986.881770594</v>
+      </c>
+      <c r="AE8">
+        <v>2914514.663226007</v>
+      </c>
+      <c r="AF8">
+        <v>5213956.07771486</v>
+      </c>
+      <c r="AG8">
+        <v>729893.7858314399</v>
+      </c>
+      <c r="AH8">
+        <v>4484062.29188342</v>
+      </c>
+      <c r="AI8">
+        <v>2152321.070032646</v>
+      </c>
     </row>
-    <row r="9" spans="1:1">
+    <row r="9" spans="1:35">
       <c r="A9">
         <v>7</v>
       </c>
+      <c r="B9">
+        <v>0.3446750642237112</v>
+      </c>
+      <c r="C9">
+        <v>0.5135029484273272</v>
+      </c>
+      <c r="D9">
+        <v>0.4632086468820766</v>
+      </c>
+      <c r="E9">
+        <v>0.2102341423312699</v>
+      </c>
+      <c r="F9">
+        <v>0.02484667761564068</v>
+      </c>
+      <c r="G9">
+        <v>0.03987258818255392</v>
+      </c>
+      <c r="H9">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="K9">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="L9">
+        <v>-11890474.67</v>
+      </c>
+      <c r="M9">
+        <v>-2834689.161328</v>
+      </c>
+      <c r="N9">
+        <v>-9055785.508672001</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <v>1848654.856353934</v>
+      </c>
+      <c r="Q9">
+        <v>258790.3833839208</v>
+      </c>
+      <c r="R9">
+        <v>1589864.472970013</v>
+      </c>
+      <c r="S9">
+        <v>763124.7247099706</v>
+      </c>
+      <c r="T9">
+        <v>9.458744898438454E-11</v>
+      </c>
+      <c r="U9">
+        <v>1.000444171950221E-11</v>
+      </c>
+      <c r="V9">
+        <v>8.003553375601768E-11</v>
+      </c>
+      <c r="W9">
+        <v>3.637978807091713E-11</v>
+      </c>
+      <c r="X9">
+        <v>4073050.986513603</v>
+      </c>
+      <c r="Y9">
+        <v>570180.2163268673</v>
+      </c>
+      <c r="Z9">
+        <v>3502870.770186735</v>
+      </c>
+      <c r="AA9">
+        <v>1681355.448229763</v>
+      </c>
+      <c r="AB9">
+        <v>7007655.264634792</v>
+      </c>
+      <c r="AC9">
+        <v>980991.0086201086</v>
+      </c>
+      <c r="AD9">
+        <v>6026664.256014684</v>
+      </c>
+      <c r="AE9">
+        <v>2892760.09424843</v>
+      </c>
+      <c r="AF9">
+        <v>5138991.318192999</v>
+      </c>
+      <c r="AG9">
+        <v>719399.5831018983</v>
+      </c>
+      <c r="AH9">
+        <v>4419591.7350911</v>
+      </c>
+      <c r="AI9">
+        <v>2121375.617262217</v>
+      </c>
     </row>
-    <row r="10" spans="1:1">
+    <row r="10" spans="1:35">
       <c r="A10">
         <v>8</v>
       </c>
+      <c r="B10">
+        <v>0.4883566468849144</v>
+      </c>
+      <c r="C10">
+        <v>0.4655573406319981</v>
+      </c>
+      <c r="D10">
+        <v>0.5104782786975733</v>
+      </c>
+      <c r="E10">
+        <v>0.1714768948122389</v>
+      </c>
+      <c r="F10">
+        <v>0.028151143799857</v>
+      </c>
+      <c r="G10">
+        <v>0.03982682161345685</v>
+      </c>
+      <c r="H10">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="K10">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="L10">
+        <v>-11890474.67</v>
+      </c>
+      <c r="M10">
+        <v>-2834689.161328</v>
+      </c>
+      <c r="N10">
+        <v>-9055785.508672001</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>1507850.203739184</v>
+      </c>
+      <c r="Q10">
+        <v>211081.6580877646</v>
+      </c>
+      <c r="R10">
+        <v>1296768.54565142</v>
+      </c>
+      <c r="S10">
+        <v>622440.5641092993</v>
+      </c>
+      <c r="T10">
+        <v>9.458744898438454E-11</v>
+      </c>
+      <c r="U10">
+        <v>1.000444171950221E-11</v>
+      </c>
+      <c r="V10">
+        <v>8.003553375601768E-11</v>
+      </c>
+      <c r="W10">
+        <v>3.637978807091713E-11</v>
+      </c>
+      <c r="X10">
+        <v>4073050.986513603</v>
+      </c>
+      <c r="Y10">
+        <v>570180.2163268673</v>
+      </c>
+      <c r="Z10">
+        <v>3502870.770186735</v>
+      </c>
+      <c r="AA10">
+        <v>1681355.448229763</v>
+      </c>
+      <c r="AB10">
+        <v>8178961.052044913</v>
+      </c>
+      <c r="AC10">
+        <v>1144960.32537124</v>
+      </c>
+      <c r="AD10">
+        <v>7034000.726673675</v>
+      </c>
+      <c r="AE10">
+        <v>3376275.123474278</v>
+      </c>
+      <c r="AF10">
+        <v>6805151.101059334</v>
+      </c>
+      <c r="AG10">
+        <v>952642.7584804446</v>
+      </c>
+      <c r="AH10">
+        <v>5852508.342578891</v>
+      </c>
+      <c r="AI10">
+        <v>2809166.375889684</v>
+      </c>
     </row>
-    <row r="11" spans="1:1">
+    <row r="11" spans="1:35">
       <c r="A11">
         <v>9</v>
+      </c>
+      <c r="B11">
+        <v>0.3235323294347978</v>
+      </c>
+      <c r="C11">
+        <v>0.478854718943495</v>
+      </c>
+      <c r="D11">
+        <v>0.5462647625053405</v>
+      </c>
+      <c r="E11">
+        <v>0.1868146053955859</v>
+      </c>
+      <c r="F11">
+        <v>0.0214769300792613</v>
+      </c>
+      <c r="G11">
+        <v>0.04248401400696341</v>
+      </c>
+      <c r="H11">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="K11">
+        <v>-8358971.299999999</v>
+      </c>
+      <c r="L11">
+        <v>-11890474.67</v>
+      </c>
+      <c r="M11">
+        <v>-2834689.161328</v>
+      </c>
+      <c r="N11">
+        <v>-9055785.508672001</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>1642719.51107832</v>
+      </c>
+      <c r="Q11">
+        <v>229961.8074207001</v>
+      </c>
+      <c r="R11">
+        <v>1412757.70365762</v>
+      </c>
+      <c r="S11">
+        <v>678114.61417941</v>
+      </c>
+      <c r="T11">
+        <v>9.458744898438454E-11</v>
+      </c>
+      <c r="U11">
+        <v>1.000444171950221E-11</v>
+      </c>
+      <c r="V11">
+        <v>8.003553375601768E-11</v>
+      </c>
+      <c r="W11">
+        <v>3.637978807091713E-11</v>
+      </c>
+      <c r="X11">
+        <v>4073050.986513603</v>
+      </c>
+      <c r="Y11">
+        <v>570180.2163268673</v>
+      </c>
+      <c r="Z11">
+        <v>3502870.770186735</v>
+      </c>
+      <c r="AA11">
+        <v>1681355.448229763</v>
+      </c>
+      <c r="AB11">
+        <v>6812962.399263395</v>
+      </c>
+      <c r="AC11">
+        <v>953736.2503416467</v>
+      </c>
+      <c r="AD11">
+        <v>5859226.148921748</v>
+      </c>
+      <c r="AE11">
+        <v>2812390.879373937</v>
+      </c>
+      <c r="AF11">
+        <v>4862044.490319731</v>
+      </c>
+      <c r="AG11">
+        <v>680630.217643776</v>
+      </c>
+      <c r="AH11">
+        <v>4181414.272675956</v>
+      </c>
+      <c r="AI11">
+        <v>2007051.966646175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: comprehensive tool cleanup and enhancement - Remove all Python cache files and __pycache__ directories - Fix syntax error in BioDYM_Scientific_Notebook.py - Add manuscript documentation and test workflow - Update FOMP model and data loader - Enhance test coverage and pytest configuration - Add FOMP problem summary for debugging - Clean up project structure for publication readiness
</commit_message>
<xml_diff>
--- a/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
+++ b/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
@@ -495,58 +495,58 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>0.3372686756995246</v>
+        <v>0.4805339013117069</v>
       </c>
       <c r="C2">
-        <v>0.5666524127873698</v>
+        <v>0.4977655235262918</v>
       </c>
       <c r="D2">
-        <v>0.484163440514402</v>
+        <v>0.4613753024295645</v>
       </c>
       <c r="E2">
-        <v>0.2282811485853466</v>
+        <v>0.1721741148360648</v>
       </c>
       <c r="F2">
-        <v>0.03078893776563844</v>
+        <v>0.01858716787891315</v>
       </c>
       <c r="G2">
-        <v>0.03391690306285543</v>
+        <v>0.03611711071017557</v>
       </c>
       <c r="H2">
-        <v>-2077266.141460755</v>
+        <v>-1444398.296991967</v>
       </c>
       <c r="I2">
-        <v>153681.5977402054</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>-2230947.73920096</v>
+        <v>-1444398.296991967</v>
       </c>
       <c r="K2">
-        <v>-2721850.671411103</v>
+        <v>-1444398.296991967</v>
       </c>
       <c r="L2">
-        <v>-6714704.016840388</v>
+        <v>-4455022.812136602</v>
       </c>
       <c r="M2">
-        <v>-1600917.166298643</v>
+        <v>-1062164.836799102</v>
       </c>
       <c r="N2">
-        <v>-5113786.850541744</v>
+        <v>-3392857.9753375</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>1333744.430370396</v>
+        <v>7.275957614183426E-11</v>
       </c>
       <c r="Q2">
-        <v>186724.2202518555</v>
+        <v>0.0006300929189819726</v>
       </c>
       <c r="R2">
-        <v>1147020.210118541</v>
+        <v>-0.0006300927343545482</v>
       </c>
       <c r="S2">
-        <v>550569.7008568998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -554,58 +554,58 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>0.3838640354212442</v>
+        <v>0.4615663833475386</v>
       </c>
       <c r="C3">
-        <v>0.5562909327951883</v>
+        <v>0.4926850455660361</v>
       </c>
       <c r="D3">
-        <v>0.5503007178603493</v>
+        <v>0.5241446013205513</v>
       </c>
       <c r="E3">
-        <v>0.2337072722581486</v>
+        <v>0.1978756636771389</v>
       </c>
       <c r="F3">
-        <v>0.02300692596625643</v>
+        <v>0.02908872726300061</v>
       </c>
       <c r="G3">
-        <v>0.03224205579803537</v>
+        <v>0.0341991094917957</v>
       </c>
       <c r="H3">
-        <v>-1597060.236472124</v>
+        <v>-1570060.386776366</v>
       </c>
       <c r="I3">
-        <v>157334.5290520539</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>-1754394.765524177</v>
+        <v>-1570060.386776366</v>
       </c>
       <c r="K3">
-        <v>-2256966.204039024</v>
+        <v>-1570060.386776366</v>
       </c>
       <c r="L3">
-        <v>-5743793.871253863</v>
+        <v>-3884810.171188374</v>
       </c>
       <c r="M3">
-        <v>-1369433.140330455</v>
+        <v>-926214.9567976819</v>
       </c>
       <c r="N3">
-        <v>-4374360.730923409</v>
+        <v>-2958595.214390692</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>1365446.838878277</v>
+        <v>1.01863406598568E-10</v>
       </c>
       <c r="Q3">
-        <v>191162.5574429587</v>
+        <v>0.0007241509920277167</v>
       </c>
       <c r="R3">
-        <v>1174284.281435318</v>
+        <v>-0.0007241507628350519</v>
       </c>
       <c r="S3">
-        <v>563656.4550889524</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -613,58 +613,58 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.4066935019950559</v>
+        <v>0.4086203398990257</v>
       </c>
       <c r="C4">
-        <v>0.495844394434643</v>
+        <v>0.5088803405518202</v>
       </c>
       <c r="D4">
-        <v>0.554208656656353</v>
+        <v>0.4366216082118222</v>
       </c>
       <c r="E4">
-        <v>0.2307953566712943</v>
+        <v>0.2068509131236811</v>
       </c>
       <c r="F4">
-        <v>0.03110521113283258</v>
+        <v>0.02402458001882022</v>
       </c>
       <c r="G4">
-        <v>0.04207278521886099</v>
+        <v>0.03199619666022699</v>
       </c>
       <c r="H4">
-        <v>-1851694.684968345</v>
+        <v>-1924813.991470188</v>
       </c>
       <c r="I4">
-        <v>155374.1926745406</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>-2007068.877642886</v>
+        <v>-1924813.991470188</v>
       </c>
       <c r="K4">
-        <v>-2503378.441671847</v>
+        <v>-1924813.991470188</v>
       </c>
       <c r="L4">
-        <v>-5457215.507651947</v>
+        <v>-5114820.199506885</v>
       </c>
       <c r="M4">
-        <v>-1301107.236369618</v>
+        <v>-1219473.477816031</v>
       </c>
       <c r="N4">
-        <v>-4156108.27128233</v>
+        <v>-3895346.721690853</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>1348433.821291221</v>
+        <v>5.820766091346741E-11</v>
       </c>
       <c r="Q4">
-        <v>188780.734980771</v>
+        <v>0.0007569970402983017</v>
       </c>
       <c r="R4">
-        <v>1159653.08631045</v>
+        <v>-0.0007569969311589375</v>
       </c>
       <c r="S4">
-        <v>556633.4814290161</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -672,58 +672,58 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>0.3497002531750191</v>
+        <v>0.4851670841553001</v>
       </c>
       <c r="C5">
-        <v>0.4507815967503702</v>
+        <v>0.5134711625773695</v>
       </c>
       <c r="D5">
-        <v>0.4284122670648705</v>
+        <v>0.5194834051500161</v>
       </c>
       <c r="E5">
-        <v>0.1804356558712845</v>
+        <v>0.2354256306167645</v>
       </c>
       <c r="F5">
-        <v>0.02602338097663437</v>
+        <v>0.02355135911356324</v>
       </c>
       <c r="G5">
-        <v>0.03554094446841606</v>
+        <v>0.03182237749735737</v>
       </c>
       <c r="H5">
-        <v>-2985202.473201036</v>
+        <v>-965294.8560030217</v>
       </c>
       <c r="I5">
-        <v>121471.4401755943</v>
+        <v>0</v>
       </c>
       <c r="J5">
-        <v>-3106673.913376631</v>
+        <v>-965294.8560030217</v>
       </c>
       <c r="K5">
-        <v>-3494688.399423242</v>
+        <v>-965294.8560030217</v>
       </c>
       <c r="L5">
-        <v>-6987611.554028764</v>
+        <v>-3445262.046614186</v>
       </c>
       <c r="M5">
-        <v>-1665983.677048993</v>
+        <v>-821418.0608689301</v>
       </c>
       <c r="N5">
-        <v>-5321627.876979772</v>
+        <v>-2623843.985745255</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>1054204.661882462</v>
+        <v>1.309672370553017E-10</v>
       </c>
       <c r="Q5">
-        <v>147588.6526635446</v>
+        <v>0.0008615698279754724</v>
       </c>
       <c r="R5">
-        <v>906616.0092189172</v>
+        <v>-0.0008615696424385533</v>
       </c>
       <c r="S5">
-        <v>435175.6844250802</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:19">
@@ -731,58 +731,58 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>0.3192390070649905</v>
+        <v>0.3417769136609921</v>
       </c>
       <c r="C6">
-        <v>0.425493073462273</v>
+        <v>0.5635883686426776</v>
       </c>
       <c r="D6">
-        <v>0.4667352370030868</v>
+        <v>0.4278325077228888</v>
       </c>
       <c r="E6">
-        <v>0.1822400348762307</v>
+        <v>0.2410334358517117</v>
       </c>
       <c r="F6">
-        <v>0.023892945153766</v>
+        <v>0.02387973345343592</v>
       </c>
       <c r="G6">
-        <v>0.03302867450300474</v>
+        <v>0.0332092461111876</v>
       </c>
       <c r="H6">
-        <v>-3418053.911061637</v>
+        <v>-2084687.77455934</v>
       </c>
       <c r="I6">
-        <v>122686.1696884228</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <v>-3540740.08075006</v>
+        <v>-2084687.77455934</v>
       </c>
       <c r="K6">
-        <v>-3932634.759926221</v>
+        <v>-2084687.77455934</v>
       </c>
       <c r="L6">
-        <v>-7004130.740873007</v>
+        <v>-5552842.765401455</v>
       </c>
       <c r="M6">
-        <v>-1669922.175265134</v>
+        <v>-1323906.650627238</v>
       </c>
       <c r="N6">
-        <v>-5334208.565607872</v>
+        <v>-4228936.114774216</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6">
-        <v>1064746.839644567</v>
+        <v>1.891748979687691E-10</v>
       </c>
       <c r="Q6">
-        <v>149064.5575502393</v>
+        <v>0.0008820923067105468</v>
       </c>
       <c r="R6">
-        <v>915682.2820943276</v>
+        <v>-0.0008820921066217124</v>
       </c>
       <c r="S6">
-        <v>439527.4954052771</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:19">
@@ -790,58 +790,58 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>0.3322441936597088</v>
+        <v>0.4206682045895849</v>
       </c>
       <c r="C7">
-        <v>0.5155040087545804</v>
+        <v>0.5357253308651272</v>
       </c>
       <c r="D7">
-        <v>0.5150401206425184</v>
+        <v>0.5615159167669858</v>
       </c>
       <c r="E7">
-        <v>0.1798401839905756</v>
+        <v>0.1737239968131636</v>
       </c>
       <c r="F7">
-        <v>0.02095804154070801</v>
+        <v>0.03642654882579148</v>
       </c>
       <c r="G7">
-        <v>0.0278611971021191</v>
+        <v>0.02912419163665422</v>
       </c>
       <c r="H7">
-        <v>-2711969.24924864</v>
+        <v>-1717645.650429058</v>
       </c>
       <c r="I7">
-        <v>121070.56138817</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>-2833039.81063681</v>
+        <v>-1717645.650429058</v>
       </c>
       <c r="K7">
-        <v>-3219773.775299594</v>
+        <v>-1717645.650429058</v>
       </c>
       <c r="L7">
-        <v>-6556233.327226514</v>
+        <v>-4151602.557916177</v>
       </c>
       <c r="M7">
-        <v>-1563134.645025664</v>
+        <v>-989823.4957115544</v>
       </c>
       <c r="N7">
-        <v>-4993098.682200851</v>
+        <v>-3161779.062204624</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7">
-        <v>1050725.586587548</v>
+        <v>8.003553375601768E-11</v>
       </c>
       <c r="Q7">
-        <v>147101.5821222568</v>
+        <v>0.0006357649072015192</v>
       </c>
       <c r="R7">
-        <v>903624.0044652914</v>
+        <v>-0.0006357647725963034</v>
       </c>
       <c r="S7">
-        <v>433739.52214334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:19">
@@ -849,58 +849,58 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0.3506585548435719</v>
+        <v>0.4376323891315589</v>
       </c>
       <c r="C8">
-        <v>0.5660602011195999</v>
+        <v>0.5543628796944019</v>
       </c>
       <c r="D8">
-        <v>0.5472465554672612</v>
+        <v>0.5434361555521705</v>
       </c>
       <c r="E8">
-        <v>0.2494189615319377</v>
+        <v>0.2098358334864847</v>
       </c>
       <c r="F8">
-        <v>0.02085590466066614</v>
+        <v>0.02095842079360604</v>
       </c>
       <c r="G8">
-        <v>0.02882224509989775</v>
+        <v>0.03967176459443192</v>
       </c>
       <c r="H8">
-        <v>-1826185.941497919</v>
+        <v>-1209676.095786615</v>
       </c>
       <c r="I8">
-        <v>167911.8260639043</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>-1994097.767561823</v>
+        <v>-1209676.095786615</v>
       </c>
       <c r="K8">
-        <v>-2530456.11481738</v>
+        <v>-1209676.095786615</v>
       </c>
       <c r="L8">
-        <v>-6135498.505503917</v>
+        <v>-3893075.199784152</v>
       </c>
       <c r="M8">
-        <v>-1462823.209575044</v>
+        <v>-928185.5017577792</v>
       </c>
       <c r="N8">
-        <v>-4672675.295928874</v>
+        <v>-2964889.698026373</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8">
-        <v>1457243.196967793</v>
+        <v>1.164153218269348E-10</v>
       </c>
       <c r="Q8">
-        <v>204014.047575491</v>
+        <v>0.0007679207428736845</v>
       </c>
       <c r="R8">
-        <v>1253229.149392301</v>
+        <v>-0.0007679205373278819</v>
       </c>
       <c r="S8">
-        <v>601549.9917083047</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:19">
@@ -908,58 +908,58 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0.3581447086850941</v>
+        <v>0.3928051454465791</v>
       </c>
       <c r="C9">
-        <v>0.4507639812564956</v>
+        <v>0.4420010379282018</v>
       </c>
       <c r="D9">
-        <v>0.5267130887283302</v>
+        <v>0.5269271970906302</v>
       </c>
       <c r="E9">
-        <v>0.2445397849059992</v>
+        <v>0.1934420065529116</v>
       </c>
       <c r="F9">
-        <v>0.0295114303285562</v>
+        <v>0.01956439925562062</v>
       </c>
       <c r="G9">
-        <v>0.02207322396208572</v>
+        <v>0.02260057972950804</v>
       </c>
       <c r="H9">
-        <v>-2599993.823582633</v>
+        <v>-2678702.670413176</v>
       </c>
       <c r="I9">
-        <v>164627.106041346</v>
+        <v>0</v>
       </c>
       <c r="J9">
-        <v>-2764620.929623979</v>
+        <v>-2678702.670413176</v>
       </c>
       <c r="K9">
-        <v>-3290486.942636049</v>
+        <v>-2678702.670413176</v>
       </c>
       <c r="L9">
-        <v>-6201454.607268951</v>
+        <v>-4620213.85562292</v>
       </c>
       <c r="M9">
-        <v>-1478548.438158905</v>
+        <v>-1101549.622274794</v>
       </c>
       <c r="N9">
-        <v>-4722906.169110048</v>
+        <v>-3518664.233348124</v>
       </c>
       <c r="O9">
         <v>0</v>
       </c>
       <c r="P9">
-        <v>1428736.354900604</v>
+        <v>9.458744898438454E-11</v>
       </c>
       <c r="Q9">
-        <v>200023.0896860846</v>
+        <v>0.0007079254519339884</v>
       </c>
       <c r="R9">
-        <v>1228713.26521452</v>
+        <v>-0.0007079252682160586</v>
       </c>
       <c r="S9">
-        <v>589782.3673029691</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:19">
@@ -967,58 +967,58 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0.4370906461070321</v>
+        <v>0.3099090050446594</v>
       </c>
       <c r="C10">
-        <v>0.4755354910412353</v>
+        <v>0.5746465391884354</v>
       </c>
       <c r="D10">
-        <v>0.5693959994505112</v>
+        <v>0.4534051389881684</v>
       </c>
       <c r="E10">
-        <v>0.2319968287267427</v>
+        <v>0.234981424815956</v>
       </c>
       <c r="F10">
-        <v>0.0278707908986356</v>
+        <v>0.02729056798273094</v>
       </c>
       <c r="G10">
-        <v>0.03997854961850016</v>
+        <v>0.02740878222946029</v>
       </c>
       <c r="H10">
-        <v>-1720463.35901672</v>
+        <v>-2405589.778113803</v>
       </c>
       <c r="I10">
-        <v>156183.0380227691</v>
+        <v>0</v>
       </c>
       <c r="J10">
-        <v>-1876646.397039489</v>
+        <v>-2405589.778113803</v>
       </c>
       <c r="K10">
-        <v>-2375539.644209362</v>
+        <v>-2405589.778113803</v>
       </c>
       <c r="L10">
-        <v>-4981665.249777675</v>
+        <v>-5706297.243418357</v>
       </c>
       <c r="M10">
-        <v>-1187726.725574309</v>
+        <v>-1360493.208647745</v>
       </c>
       <c r="N10">
-        <v>-3793938.524203365</v>
+        <v>-4345804.034770612</v>
       </c>
       <c r="O10">
         <v>0</v>
       </c>
       <c r="P10">
-        <v>1355453.483984046</v>
+        <v>5.820766091346741E-11</v>
       </c>
       <c r="Q10">
-        <v>189763.4877577665</v>
+        <v>0.0008599442026024917</v>
       </c>
       <c r="R10">
-        <v>1165689.99622628</v>
+        <v>-0.0008599440043326467</v>
       </c>
       <c r="S10">
-        <v>559531.1981886142</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:19">
@@ -1026,58 +1026,58 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0.3115746776882877</v>
+        <v>0.3934710553797131</v>
       </c>
       <c r="C11">
-        <v>0.5140664502274411</v>
+        <v>0.5564861446482909</v>
       </c>
       <c r="D11">
-        <v>0.445040526202587</v>
+        <v>0.4357649344778696</v>
       </c>
       <c r="E11">
-        <v>0.1908384899467563</v>
+        <v>0.2044788890349659</v>
       </c>
       <c r="F11">
-        <v>0.02257207658877994</v>
+        <v>0.02581746024631958</v>
       </c>
       <c r="G11">
-        <v>0.04112689266350959</v>
+        <v>0.03165763361570771</v>
       </c>
       <c r="H11">
-        <v>-2883914.303861379</v>
+        <v>-1712047.21699899</v>
       </c>
       <c r="I11">
-        <v>128474.7524142614</v>
+        <v>0</v>
       </c>
       <c r="J11">
-        <v>-3012389.056275641</v>
+        <v>-1712047.21699899</v>
       </c>
       <c r="K11">
-        <v>-3422774.122558909</v>
+        <v>-1712047.21699899</v>
       </c>
       <c r="L11">
-        <v>-7213443.900056209</v>
+        <v>-5270421.432187433</v>
       </c>
       <c r="M11">
-        <v>-1719826.538708136</v>
+        <v>-1256571.864263263</v>
       </c>
       <c r="N11">
-        <v>-5493617.361348074</v>
+        <v>-4013849.567924171</v>
       </c>
       <c r="O11">
         <v>0</v>
       </c>
       <c r="P11">
-        <v>1114983.758598109</v>
+        <v>8.731149137020111E-11</v>
       </c>
       <c r="Q11">
-        <v>156097.7262037352</v>
+        <v>0.0007483163226424949</v>
       </c>
       <c r="R11">
-        <v>958886.0323943736</v>
+        <v>-0.0007483161389245652</v>
       </c>
       <c r="S11">
-        <v>460265.2955492993</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Major BioDYM tool improvements and fixes
- Fix FOMP data loading error (output_carbon_id mapping)
- Implement Excel configuration sheet integration
- Complete TOC analysis (4/4 steps) with comprehensive documentation
- Remove unused config import and legacy plotting functions
- Add workflow visualization and function structure analysis
- Create essential knowledge summary for AI usage
- Phase 1 cleanup completed successfully

Resolves: FOMP KeyError, unused imports, configuration integration
Improves: Code quality, documentation, maintainability
</commit_message>
<xml_diff>
--- a/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
+++ b/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
@@ -495,58 +495,58 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>0.4805339013117069</v>
+        <v>0.3189820136316212</v>
       </c>
       <c r="C2">
-        <v>0.4977655235262918</v>
+        <v>0.4041255681762049</v>
       </c>
       <c r="D2">
-        <v>0.4613753024295645</v>
+        <v>0.5980722896549067</v>
       </c>
       <c r="E2">
-        <v>0.1721741148360648</v>
+        <v>0.1752537365478757</v>
       </c>
       <c r="F2">
-        <v>0.01858716787891315</v>
+        <v>0.02813228832197781</v>
       </c>
       <c r="G2">
-        <v>0.03611711071017557</v>
+        <v>0.03494429495283555</v>
       </c>
       <c r="H2">
-        <v>-1444398.296991967</v>
+        <v>-4434615.133244716</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2">
-        <v>-1444398.296991967</v>
+        <v>-4434615.133244716</v>
       </c>
       <c r="K2">
-        <v>-1444398.296991967</v>
+        <v>-4434615.133244716</v>
       </c>
       <c r="L2">
-        <v>-4455022.812136602</v>
+        <v>-6158226.140065538</v>
       </c>
       <c r="M2">
-        <v>-1062164.836799102</v>
+        <v>-1468241.923523984</v>
       </c>
       <c r="N2">
-        <v>-3392857.9753375</v>
+        <v>-4689984.216541552</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>7.275957614183426E-11</v>
+        <v>1866664.102434349</v>
       </c>
       <c r="Q2">
-        <v>0.0006300929189819726</v>
+        <v>261332.9743408089</v>
       </c>
       <c r="R2">
-        <v>-0.0006300927343545482</v>
+        <v>1605331.12809354</v>
       </c>
       <c r="S2">
-        <v>0</v>
+        <v>770558.9414848991</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -554,58 +554,58 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>0.4615663833475386</v>
+        <v>0.3820922173289832</v>
       </c>
       <c r="C3">
-        <v>0.4926850455660361</v>
+        <v>0.4132172696006317</v>
       </c>
       <c r="D3">
-        <v>0.5241446013205513</v>
+        <v>0.5668092944975084</v>
       </c>
       <c r="E3">
-        <v>0.1978756636771389</v>
+        <v>0.2423341874383638</v>
       </c>
       <c r="F3">
-        <v>0.02908872726300061</v>
+        <v>0.02637479104912397</v>
       </c>
       <c r="G3">
-        <v>0.0341991094917957</v>
+        <v>0.04401721005335676</v>
       </c>
       <c r="H3">
-        <v>-1570060.386776366</v>
+        <v>-3847820.30361057</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3">
-        <v>-1570060.386776366</v>
+        <v>-3847820.30361057</v>
       </c>
       <c r="K3">
-        <v>-1570060.386776366</v>
+        <v>-3847820.30361057</v>
       </c>
       <c r="L3">
-        <v>-3884810.171188374</v>
+        <v>-5635808.316612142</v>
       </c>
       <c r="M3">
-        <v>-926214.9567976819</v>
+        <v>-1343687.26564936</v>
       </c>
       <c r="N3">
-        <v>-2958595.214390692</v>
+        <v>-4292121.050962781</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>1.01863406598568E-10</v>
+        <v>2581151.976524142</v>
       </c>
       <c r="Q3">
-        <v>0.0007241509920277167</v>
+        <v>361361.2767133799</v>
       </c>
       <c r="R3">
-        <v>-0.0007241507628350519</v>
+        <v>2219790.699810762</v>
       </c>
       <c r="S3">
-        <v>0</v>
+        <v>1065499.535909166</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -613,58 +613,58 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.4086203398990257</v>
+        <v>0.4113777381307246</v>
       </c>
       <c r="C4">
-        <v>0.5088803405518202</v>
+        <v>0.5988830828792782</v>
       </c>
       <c r="D4">
-        <v>0.4366216082118222</v>
+        <v>0.5563703133695649</v>
       </c>
       <c r="E4">
-        <v>0.2068509131236811</v>
+        <v>0.2018877266431034</v>
       </c>
       <c r="F4">
-        <v>0.02402458001882022</v>
+        <v>0.02090473463144175</v>
       </c>
       <c r="G4">
-        <v>0.03199619666022699</v>
+        <v>0.02060831259693641</v>
       </c>
       <c r="H4">
-        <v>-1924813.991470188</v>
+        <v>-2056148.002720319</v>
       </c>
       <c r="I4">
         <v>0</v>
       </c>
       <c r="J4">
-        <v>-1924813.991470188</v>
+        <v>-2056148.002720319</v>
       </c>
       <c r="K4">
-        <v>-1924813.991470188</v>
+        <v>-2056148.002720319</v>
       </c>
       <c r="L4">
-        <v>-5114820.199506885</v>
+        <v>-5386640.079887125</v>
       </c>
       <c r="M4">
-        <v>-1219473.477816031</v>
+        <v>-1284280.669845732</v>
       </c>
       <c r="N4">
-        <v>-3895346.721690853</v>
+        <v>-4102359.410041395</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>5.820766091346741E-11</v>
+        <v>2150348.286262133</v>
       </c>
       <c r="Q4">
-        <v>0.0007569970402983017</v>
+        <v>301048.7600766986</v>
       </c>
       <c r="R4">
-        <v>-0.0007569969311589375</v>
+        <v>1849299.526185434</v>
       </c>
       <c r="S4">
-        <v>0</v>
+        <v>887663.7725690086</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -672,58 +672,58 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>0.4851670841553001</v>
+        <v>0.4095826441693662</v>
       </c>
       <c r="C5">
-        <v>0.5134711625773695</v>
+        <v>0.5327940438251747</v>
       </c>
       <c r="D5">
-        <v>0.5194834051500161</v>
+        <v>0.584573866959053</v>
       </c>
       <c r="E5">
-        <v>0.2354256306167645</v>
+        <v>0.1509405088905253</v>
       </c>
       <c r="F5">
-        <v>0.02355135911356324</v>
+        <v>0.02549444706087813</v>
       </c>
       <c r="G5">
-        <v>0.03182237749735737</v>
+        <v>0.0343828788296487</v>
       </c>
       <c r="H5">
-        <v>-965294.8560030217</v>
+        <v>-2626047.899247553</v>
       </c>
       <c r="I5">
         <v>0</v>
       </c>
       <c r="J5">
-        <v>-965294.8560030217</v>
+        <v>-2626047.899247553</v>
       </c>
       <c r="K5">
-        <v>-965294.8560030217</v>
+        <v>-2626047.899247553</v>
       </c>
       <c r="L5">
-        <v>-3445262.046614186</v>
+        <v>-5172948.707984486</v>
       </c>
       <c r="M5">
-        <v>-821418.0608689301</v>
+        <v>-1233332.454598885</v>
       </c>
       <c r="N5">
-        <v>-2623843.985745255</v>
+        <v>-3939616.2533856</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>1.309672370553017E-10</v>
+        <v>1607698.843397536</v>
       </c>
       <c r="Q5">
-        <v>0.0008615698279754724</v>
+        <v>225077.8380756551</v>
       </c>
       <c r="R5">
-        <v>-0.0008615696424385533</v>
+        <v>1382621.005321881</v>
       </c>
       <c r="S5">
-        <v>0</v>
+        <v>663658.0825545028</v>
       </c>
     </row>
     <row r="6" spans="1:19">
@@ -731,58 +731,58 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>0.3417769136609921</v>
+        <v>0.4137208446621933</v>
       </c>
       <c r="C6">
-        <v>0.5635883686426776</v>
+        <v>0.5880387757007446</v>
       </c>
       <c r="D6">
-        <v>0.4278325077228888</v>
+        <v>0.5208220478135364</v>
       </c>
       <c r="E6">
-        <v>0.2410334358517117</v>
+        <v>0.242814015414431</v>
       </c>
       <c r="F6">
-        <v>0.02387973345343592</v>
+        <v>0.01929851660302799</v>
       </c>
       <c r="G6">
-        <v>0.0332092461111876</v>
+        <v>0.03681780187622852</v>
       </c>
       <c r="H6">
-        <v>-2084687.77455934</v>
+        <v>-2118582.493014382</v>
       </c>
       <c r="I6">
         <v>0</v>
       </c>
       <c r="J6">
-        <v>-2084687.77455934</v>
+        <v>-2118582.493014382</v>
       </c>
       <c r="K6">
-        <v>-2084687.77455934</v>
+        <v>-2118582.493014382</v>
       </c>
       <c r="L6">
-        <v>-5552842.765401455</v>
+        <v>-5658051.980611512</v>
       </c>
       <c r="M6">
-        <v>-1323906.650627238</v>
+        <v>-1348990.591521753</v>
       </c>
       <c r="N6">
-        <v>-4228936.114774216</v>
+        <v>-4309061.389089758</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6">
-        <v>1.891748979687691E-10</v>
+        <v>2586262.724379859</v>
       </c>
       <c r="Q6">
-        <v>0.0008820923067105468</v>
+        <v>362076.7814131802</v>
       </c>
       <c r="R6">
-        <v>-0.0008820921066217124</v>
+        <v>2224185.942966679</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <v>1067609.252624006</v>
       </c>
     </row>
     <row r="7" spans="1:19">
@@ -790,58 +790,58 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>0.4206682045895849</v>
+        <v>0.3734038541509686</v>
       </c>
       <c r="C7">
-        <v>0.5357253308651272</v>
+        <v>0.5442391637733408</v>
       </c>
       <c r="D7">
-        <v>0.5615159167669858</v>
+        <v>0.4949245878926564</v>
       </c>
       <c r="E7">
-        <v>0.1737239968131636</v>
+        <v>0.1918917162570083</v>
       </c>
       <c r="F7">
-        <v>0.03642654882579148</v>
+        <v>0.02989269005169521</v>
       </c>
       <c r="G7">
-        <v>0.02912419163665422</v>
+        <v>0.03649912187188312</v>
       </c>
       <c r="H7">
-        <v>-1717645.650429058</v>
+        <v>-2929833.974261612</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
       <c r="J7">
-        <v>-1717645.650429058</v>
+        <v>-2929833.974261612</v>
       </c>
       <c r="K7">
-        <v>-1717645.650429058</v>
+        <v>-2929833.974261612</v>
       </c>
       <c r="L7">
-        <v>-4151602.557916177</v>
+        <v>-6279065.814879774</v>
       </c>
       <c r="M7">
-        <v>-989823.4957115544</v>
+        <v>-1497052.472625609</v>
       </c>
       <c r="N7">
-        <v>-3161779.062204624</v>
+        <v>-4782013.342254166</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7">
-        <v>8.003553375601768E-11</v>
+        <v>2043878.694669789</v>
       </c>
       <c r="Q7">
-        <v>0.0006357649072015192</v>
+        <v>286143.0172537704</v>
       </c>
       <c r="R7">
-        <v>-0.0006357647725963034</v>
+        <v>1757735.677416018</v>
       </c>
       <c r="S7">
-        <v>0</v>
+        <v>843713.1251596885</v>
       </c>
     </row>
     <row r="8" spans="1:19">
@@ -849,58 +849,58 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0.4376323891315589</v>
+        <v>0.4768289559439985</v>
       </c>
       <c r="C8">
-        <v>0.5543628796944019</v>
+        <v>0.5903355970262788</v>
       </c>
       <c r="D8">
-        <v>0.5434361555521705</v>
+        <v>0.411300000310463</v>
       </c>
       <c r="E8">
-        <v>0.2098358334864847</v>
+        <v>0.1592604001660433</v>
       </c>
       <c r="F8">
-        <v>0.02095842079360604</v>
+        <v>0.02743171414519905</v>
       </c>
       <c r="G8">
-        <v>0.03967176459443192</v>
+        <v>0.04217985580583343</v>
       </c>
       <c r="H8">
-        <v>-1209676.095786615</v>
+        <v>-1344948.209801378</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8">
-        <v>-1209676.095786615</v>
+        <v>-1344948.209801378</v>
       </c>
       <c r="K8">
-        <v>-1209676.095786615</v>
+        <v>-1344948.209801378</v>
       </c>
       <c r="L8">
-        <v>-3893075.199784152</v>
+        <v>-6049983.810455988</v>
       </c>
       <c r="M8">
-        <v>-928185.5017577792</v>
+        <v>-1442434.828653163</v>
       </c>
       <c r="N8">
-        <v>-2964889.698026373</v>
+        <v>-4607548.981802824</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8">
-        <v>1.164153218269348E-10</v>
+        <v>1696315.740737832</v>
       </c>
       <c r="Q8">
-        <v>0.0007679207428736845</v>
+        <v>237484.2037032965</v>
       </c>
       <c r="R8">
-        <v>-0.0007679205373278819</v>
+        <v>1458831.537034535</v>
       </c>
       <c r="S8">
-        <v>0</v>
+        <v>700239.137776577</v>
       </c>
     </row>
     <row r="9" spans="1:19">
@@ -908,58 +908,58 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0.3928051454465791</v>
+        <v>0.465382593808547</v>
       </c>
       <c r="C9">
-        <v>0.4420010379282018</v>
+        <v>0.5320124281728857</v>
       </c>
       <c r="D9">
-        <v>0.5269271970906302</v>
+        <v>0.4128404463970713</v>
       </c>
       <c r="E9">
-        <v>0.1934420065529116</v>
+        <v>0.1635618011585362</v>
       </c>
       <c r="F9">
-        <v>0.01956439925562062</v>
+        <v>0.02744600706171082</v>
       </c>
       <c r="G9">
-        <v>0.02260057972950804</v>
+        <v>0.04516089321025353</v>
       </c>
       <c r="H9">
-        <v>-2678702.670413176</v>
+        <v>-2031400.026463829</v>
       </c>
       <c r="I9">
         <v>0</v>
       </c>
       <c r="J9">
-        <v>-2678702.670413176</v>
+        <v>-2031400.026463829</v>
       </c>
       <c r="K9">
-        <v>-2678702.670413176</v>
+        <v>-2031400.026463829</v>
       </c>
       <c r="L9">
-        <v>-4620213.85562292</v>
+        <v>-6130799.186404467</v>
       </c>
       <c r="M9">
-        <v>-1101549.622274794</v>
+        <v>-1461702.799710758</v>
       </c>
       <c r="N9">
-        <v>-3518664.233348124</v>
+        <v>-4669096.386693709</v>
       </c>
       <c r="O9">
         <v>0</v>
       </c>
       <c r="P9">
-        <v>9.458744898438454E-11</v>
+        <v>1742130.859896039</v>
       </c>
       <c r="Q9">
-        <v>0.0007079254519339884</v>
+        <v>243898.3203854454</v>
       </c>
       <c r="R9">
-        <v>-0.0007079252682160586</v>
+        <v>1498232.539510593</v>
       </c>
       <c r="S9">
-        <v>0</v>
+        <v>719151.6189650847</v>
       </c>
     </row>
     <row r="10" spans="1:19">
@@ -967,58 +967,58 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0.3099090050446594</v>
+        <v>0.3638138616292734</v>
       </c>
       <c r="C10">
-        <v>0.5746465391884354</v>
+        <v>0.4314682277822169</v>
       </c>
       <c r="D10">
-        <v>0.4534051389881684</v>
+        <v>0.5393373549816289</v>
       </c>
       <c r="E10">
-        <v>0.234981424815956</v>
+        <v>0.1734681178806826</v>
       </c>
       <c r="F10">
-        <v>0.02729056798273094</v>
+        <v>0.02809913877823703</v>
       </c>
       <c r="G10">
-        <v>0.02740878222946029</v>
+        <v>0.03772673188948391</v>
       </c>
       <c r="H10">
-        <v>-2405589.778113803</v>
+        <v>-3866307.656167957</v>
       </c>
       <c r="I10">
         <v>0</v>
       </c>
       <c r="J10">
-        <v>-2405589.778113803</v>
+        <v>-3866307.656167957</v>
       </c>
       <c r="K10">
-        <v>-2405589.778113803</v>
+        <v>-3866307.656167957</v>
       </c>
       <c r="L10">
-        <v>-5706297.243418357</v>
+        <v>-6047986.078907579</v>
       </c>
       <c r="M10">
-        <v>-1360493.208647745</v>
+        <v>-1441958.530260637</v>
       </c>
       <c r="N10">
-        <v>-4345804.034770612</v>
+        <v>-4606027.548646943</v>
       </c>
       <c r="O10">
         <v>0</v>
       </c>
       <c r="P10">
-        <v>5.820766091346741E-11</v>
+        <v>1847645.105565341</v>
       </c>
       <c r="Q10">
-        <v>0.0008599442026024917</v>
+        <v>258670.3147791478</v>
       </c>
       <c r="R10">
-        <v>-0.0008599440043326467</v>
+        <v>1588974.790786193</v>
       </c>
       <c r="S10">
-        <v>0</v>
+        <v>762707.8995773728</v>
       </c>
     </row>
     <row r="11" spans="1:19">
@@ -1026,58 +1026,58 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0.3934710553797131</v>
+        <v>0.4532606597257179</v>
       </c>
       <c r="C11">
-        <v>0.5564861446482909</v>
+        <v>0.542068820607696</v>
       </c>
       <c r="D11">
-        <v>0.4357649344778696</v>
+        <v>0.4768071115727136</v>
       </c>
       <c r="E11">
-        <v>0.2044788890349659</v>
+        <v>0.1718884518436674</v>
       </c>
       <c r="F11">
-        <v>0.02581746024631958</v>
+        <v>0.01562866418085672</v>
       </c>
       <c r="G11">
-        <v>0.03165763361570771</v>
+        <v>0.04175412987884635</v>
       </c>
       <c r="H11">
-        <v>-1712047.21699899</v>
+        <v>-2069688.742325727</v>
       </c>
       <c r="I11">
         <v>0</v>
       </c>
       <c r="J11">
-        <v>-1712047.21699899</v>
+        <v>-2069688.742325727</v>
       </c>
       <c r="K11">
-        <v>-1712047.21699899</v>
+        <v>-2069688.742325727</v>
       </c>
       <c r="L11">
-        <v>-5270421.432187433</v>
+        <v>-5645032.226466933</v>
       </c>
       <c r="M11">
-        <v>-1256571.864263263</v>
+        <v>-1345886.426712885</v>
       </c>
       <c r="N11">
-        <v>-4013849.567924171</v>
+        <v>-4299145.799754048</v>
       </c>
       <c r="O11">
         <v>0</v>
       </c>
       <c r="P11">
-        <v>8.731149137020111E-11</v>
+        <v>1830819.753118003</v>
       </c>
       <c r="Q11">
-        <v>0.0007483163226424949</v>
+        <v>256314.7654365205</v>
       </c>
       <c r="R11">
-        <v>-0.0007483161389245652</v>
+        <v>1574504.987681483</v>
       </c>
       <c r="S11">
-        <v>0</v>
+        <v>755762.3940871115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Complete Case Study 1 validation with FOMP analysis and Monte Carlo simulation - All 4 workflow steps executed successfully - FOMP 2-pool model working (labile 70%, recalcitrant 30%) - Monte Carlo simulation completed with sensitivity analysis - Results exported and validated - Ready for detailed FOMP investigation
</commit_message>
<xml_diff>
--- a/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
+++ b/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
@@ -495,58 +495,58 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>0.3189820136316212</v>
+        <v>0.4406143776699539</v>
       </c>
       <c r="C2">
-        <v>0.4041255681762049</v>
+        <v>0.5374903685817231</v>
       </c>
       <c r="D2">
-        <v>0.5980722896549067</v>
+        <v>0.5219917630905634</v>
       </c>
       <c r="E2">
-        <v>0.1752537365478757</v>
+        <v>0.2270884712063693</v>
       </c>
       <c r="F2">
-        <v>0.02813228832197781</v>
+        <v>0.03429119080257903</v>
       </c>
       <c r="G2">
-        <v>0.03494429495283555</v>
+        <v>0.02888343746837711</v>
       </c>
       <c r="H2">
-        <v>-4434615.133244716</v>
+        <v>-2249351.688232171</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2">
-        <v>-4434615.133244716</v>
+        <v>-2249351.688232171</v>
       </c>
       <c r="K2">
-        <v>-4434615.133244716</v>
+        <v>-2249351.688232171</v>
       </c>
       <c r="L2">
-        <v>-6158226.140065538</v>
+        <v>-5363986.725678454</v>
       </c>
       <c r="M2">
-        <v>-1468241.923523984</v>
+        <v>-1278879.665790161</v>
       </c>
       <c r="N2">
-        <v>-4689984.216541552</v>
+        <v>-4085107.059888292</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>1866664.102434349</v>
+        <v>2418766.672982323</v>
       </c>
       <c r="Q2">
-        <v>261332.9743408089</v>
+        <v>338627.3342175253</v>
       </c>
       <c r="R2">
-        <v>1605331.12809354</v>
+        <v>2080139.338764798</v>
       </c>
       <c r="S2">
-        <v>770558.9414848991</v>
+        <v>998466.8826071031</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -554,58 +554,58 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>0.3820922173289832</v>
+        <v>0.4416769123823493</v>
       </c>
       <c r="C3">
-        <v>0.4132172696006317</v>
+        <v>0.5700953066948027</v>
       </c>
       <c r="D3">
-        <v>0.5668092944975084</v>
+        <v>0.5015559739057172</v>
       </c>
       <c r="E3">
-        <v>0.2423341874383638</v>
+        <v>0.1895634472658465</v>
       </c>
       <c r="F3">
-        <v>0.02637479104912397</v>
+        <v>0.02723013701411774</v>
       </c>
       <c r="G3">
-        <v>0.04401721005335676</v>
+        <v>0.03541052892489566</v>
       </c>
       <c r="H3">
-        <v>-3847820.30361057</v>
+        <v>-1946177.984131868</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3">
-        <v>-3847820.30361057</v>
+        <v>-1946177.984131868</v>
       </c>
       <c r="K3">
-        <v>-3847820.30361057</v>
+        <v>-1946177.984131868</v>
       </c>
       <c r="L3">
-        <v>-5635808.316612142</v>
+        <v>-5535527.515781911</v>
       </c>
       <c r="M3">
-        <v>-1343687.26564936</v>
+        <v>-1319778.355428351</v>
       </c>
       <c r="N3">
-        <v>-4292121.050962781</v>
+        <v>-4215749.160353561</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>2581151.976524142</v>
+        <v>2019079.816014066</v>
       </c>
       <c r="Q3">
-        <v>361361.2767133799</v>
+        <v>282671.1742419692</v>
       </c>
       <c r="R3">
-        <v>2219790.699810762</v>
+        <v>1736408.641772097</v>
       </c>
       <c r="S3">
-        <v>1065499.535909166</v>
+        <v>833476.1480506066</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -613,58 +613,58 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.4113777381307246</v>
+        <v>0.3482909032370926</v>
       </c>
       <c r="C4">
-        <v>0.5988830828792782</v>
+        <v>0.5121792890521085</v>
       </c>
       <c r="D4">
-        <v>0.5563703133695649</v>
+        <v>0.4738861652148029</v>
       </c>
       <c r="E4">
-        <v>0.2018877266431034</v>
+        <v>0.1959493145441827</v>
       </c>
       <c r="F4">
-        <v>0.02090473463144175</v>
+        <v>0.01900253902647948</v>
       </c>
       <c r="G4">
-        <v>0.02060831259693641</v>
+        <v>0.03993961533037704</v>
       </c>
       <c r="H4">
-        <v>-2056148.002720319</v>
+        <v>-3432700.901818266</v>
       </c>
       <c r="I4">
         <v>0</v>
       </c>
       <c r="J4">
-        <v>-2056148.002720319</v>
+        <v>-3432700.901818266</v>
       </c>
       <c r="K4">
-        <v>-2056148.002720319</v>
+        <v>-3432700.901818266</v>
       </c>
       <c r="L4">
-        <v>-5386640.079887125</v>
+        <v>-6679124.158590764</v>
       </c>
       <c r="M4">
-        <v>-1284280.669845732</v>
+        <v>-1592434.230088285</v>
       </c>
       <c r="N4">
-        <v>-4102359.410041395</v>
+        <v>-5086689.928502478</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>2150348.286262133</v>
+        <v>2087097.020361226</v>
       </c>
       <c r="Q4">
-        <v>301048.7600766986</v>
+        <v>292193.5828505718</v>
       </c>
       <c r="R4">
-        <v>1849299.526185434</v>
+        <v>1794903.437510655</v>
       </c>
       <c r="S4">
-        <v>887663.7725690086</v>
+        <v>861553.6500051145</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -672,58 +672,58 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>0.4095826441693662</v>
+        <v>0.3849930722341544</v>
       </c>
       <c r="C5">
-        <v>0.5327940438251747</v>
+        <v>0.46507882192787</v>
       </c>
       <c r="D5">
-        <v>0.584573866959053</v>
+        <v>0.5853263418681787</v>
       </c>
       <c r="E5">
-        <v>0.1509405088905253</v>
+        <v>0.173425454522583</v>
       </c>
       <c r="F5">
-        <v>0.02549444706087813</v>
+        <v>0.02671752043825982</v>
       </c>
       <c r="G5">
-        <v>0.0343828788296487</v>
+        <v>0.04337110046408311</v>
       </c>
       <c r="H5">
-        <v>-2626047.899247553</v>
+        <v>-3419240.340147</v>
       </c>
       <c r="I5">
         <v>0</v>
       </c>
       <c r="J5">
-        <v>-2626047.899247553</v>
+        <v>-3419240.340147</v>
       </c>
       <c r="K5">
-        <v>-2626047.899247553</v>
+        <v>-3419240.340147</v>
       </c>
       <c r="L5">
-        <v>-5172948.707984486</v>
+        <v>-5458156.556026433</v>
       </c>
       <c r="M5">
-        <v>-1233332.454598885</v>
+        <v>-1301331.600763529</v>
       </c>
       <c r="N5">
-        <v>-3939616.2533856</v>
+        <v>-4156824.955262903</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>1607698.843397536</v>
+        <v>1847190.68923949</v>
       </c>
       <c r="Q5">
-        <v>225077.8380756551</v>
+        <v>258606.6964935286</v>
       </c>
       <c r="R5">
-        <v>1382621.005321881</v>
+        <v>1588583.992745962</v>
       </c>
       <c r="S5">
-        <v>663658.0825545028</v>
+        <v>762520.3165180614</v>
       </c>
     </row>
     <row r="6" spans="1:19">
@@ -731,58 +731,58 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>0.4137208446621933</v>
+        <v>0.3554938174582777</v>
       </c>
       <c r="C6">
-        <v>0.5880387757007446</v>
+        <v>0.4966911458062038</v>
       </c>
       <c r="D6">
-        <v>0.5208220478135364</v>
+        <v>0.4035659599883265</v>
       </c>
       <c r="E6">
-        <v>0.242814015414431</v>
+        <v>0.2435310654778066</v>
       </c>
       <c r="F6">
-        <v>0.01929851660302799</v>
+        <v>0.02212794545319249</v>
       </c>
       <c r="G6">
-        <v>0.03681780187622852</v>
+        <v>0.03500397046869244</v>
       </c>
       <c r="H6">
-        <v>-2118582.493014382</v>
+        <v>-3469489.197860193</v>
       </c>
       <c r="I6">
         <v>0</v>
       </c>
       <c r="J6">
-        <v>-2118582.493014382</v>
+        <v>-3469489.197860193</v>
       </c>
       <c r="K6">
-        <v>-2118582.493014382</v>
+        <v>-3469489.197860193</v>
       </c>
       <c r="L6">
-        <v>-5658051.980611512</v>
+        <v>-7116209.195068485</v>
       </c>
       <c r="M6">
-        <v>-1348990.591521753</v>
+        <v>-1696643.877494116</v>
       </c>
       <c r="N6">
-        <v>-4309061.389089758</v>
+        <v>-5419565.317574369</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6">
-        <v>2586262.724379859</v>
+        <v>2593900.174167331</v>
       </c>
       <c r="Q6">
-        <v>362076.7814131802</v>
+        <v>363146.0243834264</v>
       </c>
       <c r="R6">
-        <v>2224185.942966679</v>
+        <v>2230754.149783906</v>
       </c>
       <c r="S6">
-        <v>1067609.252624006</v>
+        <v>1070761.991896274</v>
       </c>
     </row>
     <row r="7" spans="1:19">
@@ -790,58 +790,58 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>0.3734038541509686</v>
+        <v>0.4934901707451801</v>
       </c>
       <c r="C7">
-        <v>0.5442391637733408</v>
+        <v>0.5976290956689518</v>
       </c>
       <c r="D7">
-        <v>0.4949245878926564</v>
+        <v>0.482565943997122</v>
       </c>
       <c r="E7">
-        <v>0.1918917162570083</v>
+        <v>0.2052518451217042</v>
       </c>
       <c r="F7">
-        <v>0.02989269005169521</v>
+        <v>0.02878257980337836</v>
       </c>
       <c r="G7">
-        <v>0.03649912187188312</v>
+        <v>0.03600295008106412</v>
       </c>
       <c r="H7">
-        <v>-2929833.974261612</v>
+        <v>-1072897.347116125</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
       <c r="J7">
-        <v>-2929833.974261612</v>
+        <v>-1072897.347116125</v>
       </c>
       <c r="K7">
-        <v>-2929833.974261612</v>
+        <v>-1072897.347116125</v>
       </c>
       <c r="L7">
-        <v>-6279065.814879774</v>
+        <v>-5199065.634278371</v>
       </c>
       <c r="M7">
-        <v>-1497052.472625609</v>
+        <v>-1239559.242187732</v>
       </c>
       <c r="N7">
-        <v>-4782013.342254166</v>
+        <v>-3959506.39209064</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7">
-        <v>2043878.694669789</v>
+        <v>2186180.213866282</v>
       </c>
       <c r="Q7">
-        <v>286143.0172537704</v>
+        <v>306065.2299412795</v>
       </c>
       <c r="R7">
-        <v>1757735.677416018</v>
+        <v>1880114.983925002</v>
       </c>
       <c r="S7">
-        <v>843713.1251596885</v>
+        <v>902455.1922840013</v>
       </c>
     </row>
     <row r="8" spans="1:19">
@@ -849,58 +849,58 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0.4768289559439985</v>
+        <v>0.3758676462428207</v>
       </c>
       <c r="C8">
-        <v>0.5903355970262788</v>
+        <v>0.5948487194999903</v>
       </c>
       <c r="D8">
-        <v>0.411300000310463</v>
+        <v>0.4139783836281099</v>
       </c>
       <c r="E8">
-        <v>0.1592604001660433</v>
+        <v>0.19505799499053</v>
       </c>
       <c r="F8">
-        <v>0.02743171414519905</v>
+        <v>0.02086361499542019</v>
       </c>
       <c r="G8">
-        <v>0.04217985580583343</v>
+        <v>0.04235180828781281</v>
       </c>
       <c r="H8">
-        <v>-1344948.209801378</v>
+        <v>-2517486.674781696</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8">
-        <v>-1344948.209801378</v>
+        <v>-2517486.674781696</v>
       </c>
       <c r="K8">
-        <v>-1344948.209801378</v>
+        <v>-2517486.674781696</v>
       </c>
       <c r="L8">
-        <v>-6049983.810455988</v>
+        <v>-6870464.410729268</v>
       </c>
       <c r="M8">
-        <v>-1442434.828653163</v>
+        <v>-1638053.499900356</v>
       </c>
       <c r="N8">
-        <v>-4607548.981802824</v>
+        <v>-5232410.910828911</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8">
-        <v>1696315.740737832</v>
+        <v>2077603.389883643</v>
       </c>
       <c r="Q8">
-        <v>237484.2037032965</v>
+        <v>290864.47458371</v>
       </c>
       <c r="R8">
-        <v>1458831.537034535</v>
+        <v>1786738.915299932</v>
       </c>
       <c r="S8">
-        <v>700239.137776577</v>
+        <v>857634.6793439677</v>
       </c>
     </row>
     <row r="9" spans="1:19">
@@ -908,58 +908,58 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0.465382593808547</v>
+        <v>0.4140402087251303</v>
       </c>
       <c r="C9">
-        <v>0.5320124281728857</v>
+        <v>0.5595476627569642</v>
       </c>
       <c r="D9">
-        <v>0.4128404463970713</v>
+        <v>0.56490389409953</v>
       </c>
       <c r="E9">
-        <v>0.1635618011585362</v>
+        <v>0.1632465151059977</v>
       </c>
       <c r="F9">
-        <v>0.02744600706171082</v>
+        <v>0.02433062061080526</v>
       </c>
       <c r="G9">
-        <v>0.04516089321025353</v>
+        <v>0.03669850528039579</v>
       </c>
       <c r="H9">
-        <v>-2031400.026463829</v>
+        <v>-2353651.586388113</v>
       </c>
       <c r="I9">
         <v>0</v>
       </c>
       <c r="J9">
-        <v>-2031400.026463829</v>
+        <v>-2353651.586388113</v>
       </c>
       <c r="K9">
-        <v>-2031400.026463829</v>
+        <v>-2353651.586388113</v>
       </c>
       <c r="L9">
-        <v>-6130799.186404467</v>
+        <v>-5285097.91390918</v>
       </c>
       <c r="M9">
-        <v>-1461702.799710758</v>
+        <v>-1260071.025428116</v>
       </c>
       <c r="N9">
-        <v>-4669096.386693709</v>
+        <v>-4025026.888481064</v>
       </c>
       <c r="O9">
         <v>0</v>
       </c>
       <c r="P9">
-        <v>1742130.859896039</v>
+        <v>1738772.682388016</v>
       </c>
       <c r="Q9">
-        <v>243898.3203854454</v>
+        <v>243428.1755343222</v>
       </c>
       <c r="R9">
-        <v>1498232.539510593</v>
+        <v>1495344.506853694</v>
       </c>
       <c r="S9">
-        <v>719151.6189650847</v>
+        <v>717765.363289773</v>
       </c>
     </row>
     <row r="10" spans="1:19">
@@ -967,58 +967,58 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0.3638138616292734</v>
+        <v>0.3059669748381433</v>
       </c>
       <c r="C10">
-        <v>0.4314682277822169</v>
+        <v>0.534686019855571</v>
       </c>
       <c r="D10">
-        <v>0.5393373549816289</v>
+        <v>0.5608842492589936</v>
       </c>
       <c r="E10">
-        <v>0.1734681178806826</v>
+        <v>0.1964827420787403</v>
       </c>
       <c r="F10">
-        <v>0.02809913877823703</v>
+        <v>0.02553858230767935</v>
       </c>
       <c r="G10">
-        <v>0.03772673188948391</v>
+        <v>0.03198746274400022</v>
       </c>
       <c r="H10">
-        <v>-3866307.656167957</v>
+        <v>-3732212.952293914</v>
       </c>
       <c r="I10">
         <v>0</v>
       </c>
       <c r="J10">
-        <v>-3866307.656167957</v>
+        <v>-3732212.952293914</v>
       </c>
       <c r="K10">
-        <v>-3866307.656167957</v>
+        <v>-3732212.952293914</v>
       </c>
       <c r="L10">
-        <v>-6047986.078907579</v>
+        <v>-6546251.010599229</v>
       </c>
       <c r="M10">
-        <v>-1441958.530260637</v>
+        <v>-1560754.664909196</v>
       </c>
       <c r="N10">
-        <v>-4606027.548646943</v>
+        <v>-4985496.345690034</v>
       </c>
       <c r="O10">
         <v>0</v>
       </c>
       <c r="P10">
-        <v>1847645.105565341</v>
+        <v>2092778.668294232</v>
       </c>
       <c r="Q10">
-        <v>258670.3147791478</v>
+        <v>292989.0135611925</v>
       </c>
       <c r="R10">
-        <v>1588974.790786193</v>
+        <v>1799789.654733039</v>
       </c>
       <c r="S10">
-        <v>762707.8995773728</v>
+        <v>863899.0342718587</v>
       </c>
     </row>
     <row r="11" spans="1:19">
@@ -1026,58 +1026,58 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0.4532606597257179</v>
+        <v>0.3968217552240292</v>
       </c>
       <c r="C11">
-        <v>0.542068820607696</v>
+        <v>0.400830429717305</v>
       </c>
       <c r="D11">
-        <v>0.4768071115727136</v>
+        <v>0.4396194384539051</v>
       </c>
       <c r="E11">
-        <v>0.1718884518436674</v>
+        <v>0.1893219516222435</v>
       </c>
       <c r="F11">
-        <v>0.01562866418085672</v>
+        <v>0.02709741391199448</v>
       </c>
       <c r="G11">
-        <v>0.04175412987884635</v>
+        <v>0.03654053143753607</v>
       </c>
       <c r="H11">
-        <v>-2069688.742325727</v>
+        <v>-3824105.531735162</v>
       </c>
       <c r="I11">
         <v>0</v>
       </c>
       <c r="J11">
-        <v>-2069688.742325727</v>
+        <v>-3824105.531735162</v>
       </c>
       <c r="K11">
-        <v>-2069688.742325727</v>
+        <v>-3824105.531735162</v>
       </c>
       <c r="L11">
-        <v>-5645032.226466933</v>
+        <v>-6488772.953804204</v>
       </c>
       <c r="M11">
-        <v>-1345886.426712885</v>
+        <v>-1547050.768567992</v>
       </c>
       <c r="N11">
-        <v>-4299145.799754048</v>
+        <v>-4941722.185236212</v>
       </c>
       <c r="O11">
         <v>0</v>
       </c>
       <c r="P11">
-        <v>1830819.753118003</v>
+        <v>2016507.595542835</v>
       </c>
       <c r="Q11">
-        <v>256314.7654365205</v>
+        <v>282311.063375997</v>
       </c>
       <c r="R11">
-        <v>1574504.987681483</v>
+        <v>1734196.532166839</v>
       </c>
       <c r="S11">
-        <v>755762.3940871115</v>
+        <v>832414.3354400825</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix node positioning consistency across elements in enhanced Sankey
- Modified calculate_dynamic_positions to use ALL processes for positioning
- Ensures consistent node positions when switching between elements (material, WC, DM, CC)
- Only flows change when switching elements, not node positions
- Element-specific positions from Excel are now properly applied
- Fixes issue where fewer processes caused position recalculation
- Maintains Excel-defined layouts for each material level
</commit_message>
<xml_diff>
--- a/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
+++ b/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
@@ -495,58 +495,58 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>0.3776001798547601</v>
+        <v>0.440470713700875</v>
       </c>
       <c r="C2">
-        <v>0.7169709071255881</v>
+        <v>0.3562893583592965</v>
       </c>
       <c r="D2">
-        <v>-649807.917740525</v>
+        <v>-2414627.443401478</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>-649807.917740525</v>
+        <v>-2414627.443401478</v>
       </c>
       <c r="G2">
-        <v>-649807.917740525</v>
+        <v>-2414627.443401478</v>
       </c>
       <c r="H2">
-        <v>-75319.99328709877</v>
+        <v>-3012851.71200933</v>
       </c>
       <c r="I2">
-        <v>309362.0507911325</v>
+        <v>-555665.6333620335</v>
       </c>
       <c r="J2">
-        <v>-384682.0440782313</v>
+        <v>-2457186.078647296</v>
       </c>
       <c r="K2">
         <v>0</v>
       </c>
       <c r="L2">
-        <v>2081834.427663095</v>
+        <v>1034540.516317563</v>
       </c>
       <c r="M2">
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2081834.427663095</v>
+        <v>1034540.516317563</v>
       </c>
       <c r="O2">
-        <v>999280.5252782861</v>
+        <v>496579.4478324305</v>
       </c>
       <c r="P2">
-        <v>558305.5994972592</v>
+        <v>277442.6993289943</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
       <c r="R2">
-        <v>558305.5994972592</v>
+        <v>277442.6993289943</v>
       </c>
       <c r="S2">
-        <v>267986.6877586844</v>
+        <v>133172.4956779173</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -554,58 +554,58 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>0.5878014723389098</v>
+        <v>0.4408971156159481</v>
       </c>
       <c r="C3">
-        <v>0.4921810106979571</v>
+        <v>0.3948080795693732</v>
       </c>
       <c r="D3">
-        <v>-320172.5704428399</v>
+        <v>-2166466.646793793</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3">
-        <v>-320172.5704428399</v>
+        <v>-2166466.646793793</v>
       </c>
       <c r="G3">
-        <v>-320172.5704428399</v>
+        <v>-2166466.646793793</v>
       </c>
       <c r="H3">
-        <v>127389.2792449056</v>
+        <v>-2614234.873733097</v>
       </c>
       <c r="I3">
-        <v>255068.2460120126</v>
+        <v>-443042.5489044277</v>
       </c>
       <c r="J3">
-        <v>-127678.966767107</v>
+        <v>-2171192.324828668</v>
       </c>
       <c r="K3">
         <v>0</v>
       </c>
       <c r="L3">
-        <v>1429122.663876157</v>
+        <v>1146385.500720324</v>
       </c>
       <c r="M3">
         <v>0</v>
       </c>
       <c r="N3">
-        <v>1429122.663876157</v>
+        <v>1146385.500720324</v>
       </c>
       <c r="O3">
-        <v>685978.8786605555</v>
+        <v>550265.0403457554</v>
       </c>
       <c r="P3">
-        <v>383261.5961232536</v>
+        <v>307437.2465600337</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
       <c r="R3">
-        <v>383261.5961232536</v>
+        <v>307437.2465600338</v>
       </c>
       <c r="S3">
-        <v>183965.5661391617</v>
+        <v>147569.8783488162</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -613,58 +613,58 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.3697003873236006</v>
+        <v>0.4530374786246817</v>
       </c>
       <c r="C4">
-        <v>0.3272099640918237</v>
+        <v>0.4140134752942853</v>
       </c>
       <c r="D4">
-        <v>-3190850.713516199</v>
+        <v>-1943030.123937516</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>-3190850.713516199</v>
+        <v>-1943030.123937516</v>
       </c>
       <c r="G4">
-        <v>-3190850.713516199</v>
+        <v>-1943030.123937516</v>
       </c>
       <c r="H4">
-        <v>-4151449.368203746</v>
+        <v>-2273658.196798186</v>
       </c>
       <c r="I4">
-        <v>-840405.3114785966</v>
+        <v>-353074.5192926812</v>
       </c>
       <c r="J4">
-        <v>-3311044.05672515</v>
+        <v>-1920583.677505506</v>
       </c>
       <c r="K4">
         <v>0</v>
       </c>
       <c r="L4">
-        <v>950104.0579899602</v>
+        <v>1202151.29765804</v>
       </c>
       <c r="M4">
         <v>0</v>
       </c>
       <c r="N4">
-        <v>950104.05798996</v>
+        <v>1202151.29765804</v>
       </c>
       <c r="O4">
-        <v>456049.9478351807</v>
+        <v>577032.6228758591</v>
       </c>
       <c r="P4">
-        <v>254798.5606503314</v>
+        <v>322392.4976967455</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
       <c r="R4">
-        <v>254798.5606503314</v>
+        <v>322392.4976967455</v>
       </c>
       <c r="S4">
-        <v>122303.3091121591</v>
+        <v>154748.3988944379</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -672,58 +672,58 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>0.4505238705404483</v>
+        <v>0.4646829360384797</v>
       </c>
       <c r="C5">
-        <v>0.4585098478944794</v>
+        <v>0.4442838849451958</v>
       </c>
       <c r="D5">
-        <v>-1681486.291190924</v>
+        <v>-1653466.907215537</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>-1681486.291190924</v>
+        <v>-1653466.907215537</v>
       </c>
       <c r="G5">
-        <v>-1681486.291190924</v>
+        <v>-1653466.907215537</v>
       </c>
       <c r="H5">
-        <v>-1848925.662440928</v>
+        <v>-1825914.664277845</v>
       </c>
       <c r="I5">
-        <v>-231495.9543047259</v>
+        <v>-232504.2813391603</v>
       </c>
       <c r="J5">
-        <v>-1617429.708136202</v>
+        <v>-1593410.382938684</v>
       </c>
       <c r="K5">
         <v>0</v>
       </c>
       <c r="L5">
-        <v>1331353.304970426</v>
+        <v>1290046.050882235</v>
       </c>
       <c r="M5">
         <v>0</v>
       </c>
       <c r="N5">
-        <v>1331353.304970427</v>
+        <v>1290046.050882235</v>
       </c>
       <c r="O5">
-        <v>639049.5863858047</v>
+        <v>619222.1044234727</v>
       </c>
       <c r="P5">
-        <v>357041.8450176865</v>
+        <v>345964.0806427447</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
       <c r="R5">
-        <v>357041.8450176865</v>
+        <v>345964.0806427448</v>
       </c>
       <c r="S5">
-        <v>171380.0856084895</v>
+        <v>166062.7587085175</v>
       </c>
     </row>
     <row r="6" spans="1:19">
@@ -731,58 +731,58 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>0.4715852896987358</v>
+        <v>0.4935839306456321</v>
       </c>
       <c r="C6">
-        <v>0.2090483147406</v>
+        <v>0.5848351040346516</v>
       </c>
       <c r="D6">
-        <v>-3089532.297343528</v>
+        <v>-519374.4647446815</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
       <c r="F6">
-        <v>-3089532.297343528</v>
+        <v>-519374.4647446815</v>
       </c>
       <c r="G6">
-        <v>-3089532.297343528</v>
+        <v>-519374.4647446815</v>
       </c>
       <c r="H6">
-        <v>-4147249.979568586</v>
+        <v>-46252.87532518356</v>
       </c>
       <c r="I6">
-        <v>-893348.6116993213</v>
+        <v>255968.0635107075</v>
       </c>
       <c r="J6">
-        <v>-3253901.367869266</v>
+        <v>-302220.938835891</v>
       </c>
       <c r="K6">
         <v>0</v>
       </c>
       <c r="L6">
-        <v>607003.6794333959</v>
+        <v>1698157.961480572</v>
       </c>
       <c r="M6">
         <v>0</v>
       </c>
       <c r="N6">
-        <v>607003.6794333959</v>
+        <v>1698157.961480572</v>
       </c>
       <c r="O6">
-        <v>291361.76612803</v>
+        <v>815115.8215106749</v>
       </c>
       <c r="P6">
-        <v>162786.0259394017</v>
+        <v>455411.3843672512</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
       <c r="R6">
-        <v>162786.0259394017</v>
+        <v>455411.3843672512</v>
       </c>
       <c r="S6">
-        <v>78137.29245091284</v>
+        <v>218597.4644962806</v>
       </c>
     </row>
     <row r="7" spans="1:19">
@@ -790,58 +790,58 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>0.4997004058422669</v>
+        <v>0.4668787776140075</v>
       </c>
       <c r="C7">
-        <v>0.4497233192507541</v>
+        <v>0.6661833119258669</v>
       </c>
       <c r="D7">
-        <v>-1326216.102231493</v>
+        <v>-226035.3862292718</v>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
       <c r="F7">
-        <v>-1326216.102231493</v>
+        <v>-226035.3862292718</v>
       </c>
       <c r="G7">
-        <v>-1326216.102231493</v>
+        <v>-226035.3862292718</v>
       </c>
       <c r="H7">
-        <v>-1353965.493047441</v>
+        <v>467346.8094031098</v>
       </c>
       <c r="I7">
-        <v>-117499.0670585739</v>
+        <v>415558.3247529726</v>
       </c>
       <c r="J7">
-        <v>-1236466.425988866</v>
+        <v>51788.48465013769</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
       <c r="L7">
-        <v>1305840.278363127</v>
+        <v>1934364.895588377</v>
       </c>
       <c r="M7">
         <v>0</v>
       </c>
       <c r="N7">
-        <v>1305840.278363127</v>
+        <v>1934364.895588377</v>
       </c>
       <c r="O7">
-        <v>626803.3336143006</v>
+        <v>928495.1498824214</v>
       </c>
       <c r="P7">
-        <v>350199.77082307</v>
+        <v>518757.2740307731</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
       <c r="R7">
-        <v>350199.77082307</v>
+        <v>518757.2740307731</v>
       </c>
       <c r="S7">
-        <v>168095.8899950736</v>
+        <v>249003.4915347711</v>
       </c>
     </row>
     <row r="8" spans="1:19">
@@ -849,58 +849,58 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0.374617631601376</v>
+        <v>0.507124546745101</v>
       </c>
       <c r="C8">
-        <v>0.4971355256491042</v>
+        <v>0.4557932680542008</v>
       </c>
       <c r="D8">
-        <v>-2070708.667086535</v>
+        <v>-1225613.331299989</v>
       </c>
       <c r="E8">
         <v>0</v>
       </c>
       <c r="F8">
-        <v>-2070708.667086535</v>
+        <v>-1225613.331299989</v>
       </c>
       <c r="G8">
-        <v>-2070708.667086535</v>
+        <v>-1225613.331299989</v>
       </c>
       <c r="H8">
-        <v>-2356847.379375963</v>
+        <v>-1203672.118220932</v>
       </c>
       <c r="I8">
-        <v>-334960.616798249</v>
+        <v>-78895.05512663237</v>
       </c>
       <c r="J8">
-        <v>-2021886.762577714</v>
+        <v>-1124777.0630943</v>
       </c>
       <c r="K8">
         <v>0</v>
       </c>
       <c r="L8">
-        <v>1443508.85402022</v>
+        <v>1323465.300895532</v>
       </c>
       <c r="M8">
         <v>0</v>
       </c>
       <c r="N8">
-        <v>1443508.85402022</v>
+        <v>1323465.300895532</v>
       </c>
       <c r="O8">
-        <v>692884.2499297055</v>
+        <v>635263.3444298556</v>
       </c>
       <c r="P8">
-        <v>387119.6793627925</v>
+        <v>354926.4429543178</v>
       </c>
       <c r="Q8">
         <v>0</v>
       </c>
       <c r="R8">
-        <v>387119.6793627926</v>
+        <v>354926.4429543178</v>
       </c>
       <c r="S8">
-        <v>185817.4460941404</v>
+        <v>170364.6926180726</v>
       </c>
     </row>
     <row r="9" spans="1:19">
@@ -908,58 +908,58 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0.4902037994264422</v>
+        <v>0.545973976342663</v>
       </c>
       <c r="C9">
-        <v>0.1810445863301215</v>
+        <v>0.2757430781396258</v>
       </c>
       <c r="D9">
-        <v>-3111726.300444806</v>
+        <v>-2044203.089889325</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
       <c r="F9">
-        <v>-3111726.300444806</v>
+        <v>-2044203.089889325</v>
       </c>
       <c r="G9">
-        <v>-3111726.300444806</v>
+        <v>-2044203.089889325</v>
       </c>
       <c r="H9">
-        <v>-4211981.839574581</v>
+        <v>-2581311.155449423</v>
       </c>
       <c r="I9">
-        <v>-921566.5416021812</v>
+        <v>-489549.814118128</v>
       </c>
       <c r="J9">
-        <v>-3290415.297972399</v>
+        <v>-2091761.341331295</v>
       </c>
       <c r="K9">
         <v>0</v>
       </c>
       <c r="L9">
-        <v>525690.5810517775</v>
+        <v>800662.1015660189</v>
       </c>
       <c r="M9">
         <v>0</v>
       </c>
       <c r="N9">
-        <v>525690.5810517773</v>
+        <v>800662.1015660189</v>
       </c>
       <c r="O9">
-        <v>252331.4789048532</v>
+        <v>384317.8087516892</v>
       </c>
       <c r="P9">
-        <v>140979.5087948616</v>
+        <v>214721.2711393838</v>
       </c>
       <c r="Q9">
         <v>0</v>
       </c>
       <c r="R9">
-        <v>140979.5087948616</v>
+        <v>214721.2711393838</v>
       </c>
       <c r="S9">
-        <v>67670.16422153357</v>
+        <v>103066.2101469043</v>
       </c>
     </row>
     <row r="10" spans="1:19">
@@ -967,58 +967,58 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0.590682814192613</v>
+        <v>0.5406512389940892</v>
       </c>
       <c r="C10">
-        <v>0.4474701491554725</v>
+        <v>0.3572397216799597</v>
       </c>
       <c r="D10">
-        <v>-580004.5466251684</v>
+        <v>-1571186.435902989</v>
       </c>
       <c r="E10">
         <v>0</v>
       </c>
       <c r="F10">
-        <v>-580004.5466251684</v>
+        <v>-1571186.435902989</v>
       </c>
       <c r="G10">
-        <v>-580004.5466251684</v>
+        <v>-1571186.435902989</v>
       </c>
       <c r="H10">
-        <v>-295162.164811486</v>
+        <v>-1811947.827922707</v>
       </c>
       <c r="I10">
-        <v>133911.7747784042</v>
+        <v>-268912.7173241808</v>
       </c>
       <c r="J10">
-        <v>-429073.9395898897</v>
+        <v>-1543035.110598525</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>1299297.855192089</v>
+        <v>1037300.041230055</v>
       </c>
       <c r="M10">
         <v>0</v>
       </c>
       <c r="N10">
-        <v>1299297.855192089</v>
+        <v>1037300.041230055</v>
       </c>
       <c r="O10">
-        <v>623662.9704922027</v>
+        <v>497904.0197904264</v>
       </c>
       <c r="P10">
-        <v>348445.2261570125</v>
+        <v>278182.747716188</v>
       </c>
       <c r="Q10">
         <v>0</v>
       </c>
       <c r="R10">
-        <v>348445.2261570125</v>
+        <v>278182.747716188</v>
       </c>
       <c r="S10">
-        <v>167253.7085553661</v>
+        <v>133527.7189037702</v>
       </c>
     </row>
     <row r="11" spans="1:19">
@@ -1026,58 +1026,58 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0.3905171356894984</v>
+        <v>0.3504549342384379</v>
       </c>
       <c r="C11">
-        <v>0.3151353202430367</v>
+        <v>0.4209585612244957</v>
       </c>
       <c r="D11">
-        <v>-3093518.926060464</v>
+        <v>-2756412.897117089</v>
       </c>
       <c r="E11">
         <v>0</v>
       </c>
       <c r="F11">
-        <v>-3093518.926060464</v>
+        <v>-2756412.897117089</v>
       </c>
       <c r="G11">
-        <v>-3093518.926060464</v>
+        <v>-2756412.897117089</v>
       </c>
       <c r="H11">
-        <v>-4027295.280625903</v>
+        <v>-3422455.22988882</v>
       </c>
       <c r="I11">
-        <v>-816316.9968078226</v>
+        <v>-623799.6184116157</v>
       </c>
       <c r="J11">
-        <v>-3210978.283818079</v>
+        <v>-2798655.611477204</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>915043.4871685387</v>
+        <v>1222317.41437058</v>
       </c>
       <c r="M11">
         <v>0</v>
       </c>
       <c r="N11">
-        <v>915043.4871685387</v>
+        <v>1222317.41437058</v>
       </c>
       <c r="O11">
-        <v>439220.8738408986</v>
+        <v>586712.3588978784</v>
       </c>
       <c r="P11">
-        <v>245396.0295215026</v>
+        <v>327800.6395408424</v>
       </c>
       <c r="Q11">
         <v>0</v>
       </c>
       <c r="R11">
-        <v>245396.0295215026</v>
+        <v>327800.6395408424</v>
       </c>
       <c r="S11">
-        <v>117790.0941703213</v>
+        <v>157344.3069796044</v>
       </c>
     </row>
     <row r="12" spans="1:19">
@@ -1085,58 +1085,58 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>0.3139371253608201</v>
+        <v>0.5024346377785431</v>
       </c>
       <c r="C12">
-        <v>0.267512196587763</v>
+        <v>0.4701442422227763</v>
       </c>
       <c r="D12">
-        <v>-4036059.127990766</v>
+        <v>-1173686.477831411</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
       <c r="F12">
-        <v>-4036059.127990766</v>
+        <v>-1173686.477831411</v>
       </c>
       <c r="G12">
-        <v>-4036059.127990766</v>
+        <v>-1173686.477831411</v>
       </c>
       <c r="H12">
-        <v>-5424434.573601117</v>
+        <v>-1112813.107779967</v>
       </c>
       <c r="I12">
-        <v>-1171163.87006896</v>
+        <v>-50680.81258419952</v>
       </c>
       <c r="J12">
-        <v>-4253270.703532157</v>
+        <v>-1062132.295195768</v>
       </c>
       <c r="K12">
         <v>0</v>
       </c>
       <c r="L12">
-        <v>776762.4810732119</v>
+        <v>1365135.544133743</v>
       </c>
       <c r="M12">
         <v>0</v>
       </c>
       <c r="N12">
-        <v>776762.4810732119</v>
+        <v>1365135.544133743</v>
       </c>
       <c r="O12">
-        <v>372845.9909151418</v>
+        <v>655265.0611841967</v>
       </c>
       <c r="P12">
-        <v>208311.8796096398</v>
+        <v>366101.5536274666</v>
       </c>
       <c r="Q12">
         <v>0</v>
       </c>
       <c r="R12">
-        <v>208311.8796096398</v>
+        <v>366101.5536274666</v>
       </c>
       <c r="S12">
-        <v>99989.70221262706</v>
+        <v>175728.7457411839</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -1144,58 +1144,58 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>0.3092887732932001</v>
+        <v>0.4988428324318666</v>
       </c>
       <c r="C13">
-        <v>0.3817905575393291</v>
+        <v>0.3639467539397552</v>
       </c>
       <c r="D13">
-        <v>-3349239.158223306</v>
+        <v>-1878071.592542547</v>
       </c>
       <c r="E13">
         <v>0</v>
       </c>
       <c r="F13">
-        <v>-3349239.158223306</v>
+        <v>-1878071.592542547</v>
       </c>
       <c r="G13">
-        <v>-3349239.158223306</v>
+        <v>-1878071.592542547</v>
       </c>
       <c r="H13">
-        <v>-4312120.876056199</v>
+        <v>-2240543.714583392</v>
       </c>
       <c r="I13">
-        <v>-853794.7899505836</v>
+        <v>-368036.4132717596</v>
       </c>
       <c r="J13">
-        <v>-3458326.086105614</v>
+        <v>-1872507.301311633</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13">
-        <v>1108587.139230794</v>
+        <v>1056774.932787187</v>
       </c>
       <c r="M13">
         <v>0</v>
       </c>
       <c r="N13">
-        <v>1108587.139230794</v>
+        <v>1056774.932787187</v>
       </c>
       <c r="O13">
-        <v>532121.8268307814</v>
+        <v>507251.9677378498</v>
       </c>
       <c r="P13">
-        <v>297300.4957257638</v>
+        <v>283405.517049556</v>
       </c>
       <c r="Q13">
         <v>0</v>
       </c>
       <c r="R13">
-        <v>297300.4957257638</v>
+        <v>283405.517049556</v>
       </c>
       <c r="S13">
-        <v>142704.2379483666</v>
+        <v>136034.6481837869</v>
       </c>
     </row>
     <row r="14" spans="1:19">
@@ -1203,58 +1203,58 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>0.3053352839314246</v>
+        <v>0.4392692437158223</v>
       </c>
       <c r="C14">
-        <v>0.4654723702009245</v>
+        <v>0.5432554326675922</v>
       </c>
       <c r="D14">
-        <v>-2850901.026182467</v>
+        <v>-1237423.131938945</v>
       </c>
       <c r="E14">
         <v>0</v>
       </c>
       <c r="F14">
-        <v>-2850901.026182467</v>
+        <v>-1237423.131938945</v>
       </c>
       <c r="G14">
-        <v>-2850901.026182467</v>
+        <v>-1237423.131938945</v>
       </c>
       <c r="H14">
-        <v>-3504150.613640542</v>
+        <v>-1116900.804423215</v>
       </c>
       <c r="I14">
-        <v>-622955.4439198483</v>
+        <v>-18277.83708087195</v>
       </c>
       <c r="J14">
-        <v>-2881195.169720693</v>
+        <v>-1098622.967342343</v>
       </c>
       <c r="K14">
         <v>0</v>
       </c>
       <c r="L14">
-        <v>1351570.05086189</v>
+        <v>1577425.04124271</v>
       </c>
       <c r="M14">
         <v>0</v>
       </c>
       <c r="N14">
-        <v>1351570.05086189</v>
+        <v>1577425.04124271</v>
       </c>
       <c r="O14">
-        <v>648753.6244137072</v>
+        <v>757164.0197965013</v>
       </c>
       <c r="P14">
-        <v>362463.5645765696</v>
+        <v>423033.2737371379</v>
       </c>
       <c r="Q14">
         <v>0</v>
       </c>
       <c r="R14">
-        <v>362463.5645765696</v>
+        <v>423033.273737138</v>
       </c>
       <c r="S14">
-        <v>173982.5109967534</v>
+        <v>203055.9713938262</v>
       </c>
     </row>
     <row r="15" spans="1:19">
@@ -1262,58 +1262,58 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0.4378193035620743</v>
+        <v>0.5069431517968397</v>
       </c>
       <c r="C15">
-        <v>0.316307137220567</v>
+        <v>0.3875839846428868</v>
       </c>
       <c r="D15">
-        <v>-2690680.344569152</v>
+        <v>-1660263.223190929</v>
       </c>
       <c r="E15">
         <v>0</v>
       </c>
       <c r="F15">
-        <v>-2690680.344569152</v>
+        <v>-1660263.223190929</v>
       </c>
       <c r="G15">
-        <v>-2690680.344569152</v>
+        <v>-1660263.223190929</v>
       </c>
       <c r="H15">
-        <v>-3452877.568799219</v>
+        <v>-1902724.907861322</v>
       </c>
       <c r="I15">
-        <v>-678829.5740334714</v>
+        <v>-276702.6416833528</v>
       </c>
       <c r="J15">
-        <v>-2774047.994765747</v>
+        <v>-1626022.266177969</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
-        <v>918446.036564194</v>
+        <v>1125409.238814579</v>
       </c>
       <c r="M15">
         <v>0</v>
       </c>
       <c r="N15">
-        <v>918446.0365641939</v>
+        <v>1125409.238814579</v>
       </c>
       <c r="O15">
-        <v>440854.0975508131</v>
+        <v>540196.4346309979</v>
       </c>
       <c r="P15">
-        <v>246308.5239806768</v>
+        <v>301811.8402727315</v>
       </c>
       <c r="Q15">
         <v>0</v>
       </c>
       <c r="R15">
-        <v>246308.5239806768</v>
+        <v>301811.8402727315</v>
       </c>
       <c r="S15">
-        <v>118228.0915107248</v>
+        <v>144869.6833309111</v>
       </c>
     </row>
     <row r="16" spans="1:19">
@@ -1321,58 +1321,58 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>0.5125098799305293</v>
+        <v>0.3213104921765115</v>
       </c>
       <c r="C16">
-        <v>0.3575894760378063</v>
+        <v>0.3079302067463411</v>
       </c>
       <c r="D16">
-        <v>-1804198.284453959</v>
+        <v>-3717768.236404144</v>
       </c>
       <c r="E16">
         <v>0</v>
       </c>
       <c r="F16">
-        <v>-1804198.284453959</v>
+        <v>-3717768.236404144</v>
       </c>
       <c r="G16">
-        <v>-1804198.284453959</v>
+        <v>-3717768.236404144</v>
       </c>
       <c r="H16">
-        <v>-2142988.496316064</v>
+        <v>-4923809.943455936</v>
       </c>
       <c r="I16">
-        <v>-347679.633119232</v>
+        <v>-1033353.041584632</v>
       </c>
       <c r="J16">
-        <v>-1795308.863196832</v>
+        <v>-3890456.901871305</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
       <c r="L16">
-        <v>1038315.606375243</v>
+        <v>894122.3407404682</v>
       </c>
       <c r="M16">
         <v>0</v>
       </c>
       <c r="N16">
-        <v>1038315.606375243</v>
+        <v>894122.3407404682</v>
       </c>
       <c r="O16">
-        <v>498391.4910601165</v>
+        <v>429178.7235554248</v>
       </c>
       <c r="P16">
-        <v>278455.10160739</v>
+        <v>239785.4040829536</v>
       </c>
       <c r="Q16">
         <v>0</v>
       </c>
       <c r="R16">
-        <v>278455.10160739</v>
+        <v>239785.4040829536</v>
       </c>
       <c r="S16">
-        <v>133658.4487715472</v>
+        <v>115096.9939598177</v>
       </c>
     </row>
     <row r="17" spans="1:19">
@@ -1380,58 +1380,58 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0.3312975870273106</v>
+        <v>0.4498596300281296</v>
       </c>
       <c r="C17">
-        <v>0.223164914459507</v>
+        <v>0.2269289802658426</v>
       </c>
       <c r="D17">
-        <v>-4172551.803103202</v>
+        <v>-3157593.013397145</v>
       </c>
       <c r="E17">
         <v>0</v>
       </c>
       <c r="F17">
-        <v>-4172551.803103202</v>
+        <v>-3157593.013397145</v>
       </c>
       <c r="G17">
-        <v>-4172551.803103202</v>
+        <v>-3157593.013397145</v>
       </c>
       <c r="H17">
-        <v>-5671107.710456302</v>
+        <v>-4222891.188461766</v>
       </c>
       <c r="I17">
-        <v>-1250221.517034122</v>
+        <v>-903219.8724936618</v>
       </c>
       <c r="J17">
-        <v>-4420886.193422181</v>
+        <v>-3319671.315968103</v>
       </c>
       <c r="K17">
         <v>0</v>
       </c>
       <c r="L17">
-        <v>647993.3806950288</v>
+        <v>658922.9201027502</v>
       </c>
       <c r="M17">
         <v>0</v>
       </c>
       <c r="N17">
-        <v>647993.3806950288</v>
+        <v>658922.9201027503</v>
       </c>
       <c r="O17">
-        <v>311036.822733614</v>
+        <v>316283.0016493202</v>
       </c>
       <c r="P17">
-        <v>173778.6291128338</v>
+        <v>176709.7090153343</v>
       </c>
       <c r="Q17">
         <v>0</v>
       </c>
       <c r="R17">
-        <v>173778.6291128338</v>
+        <v>176709.7090153343</v>
       </c>
       <c r="S17">
-        <v>83413.74197416025</v>
+        <v>84820.66032736047</v>
       </c>
     </row>
     <row r="18" spans="1:19">
@@ -1439,58 +1439,58 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0.3159064616948757</v>
+        <v>0.5275043418514653</v>
       </c>
       <c r="C18">
-        <v>0.3637329797504892</v>
+        <v>0.3916172145025195</v>
       </c>
       <c r="D18">
-        <v>-3408588.945332417</v>
+        <v>-1462781.540131018</v>
       </c>
       <c r="E18">
         <v>0</v>
       </c>
       <c r="F18">
-        <v>-3408588.945332417</v>
+        <v>-1462781.540131018</v>
       </c>
       <c r="G18">
-        <v>-3408588.945332417</v>
+        <v>-1462781.540131018</v>
       </c>
       <c r="H18">
-        <v>-4417928.133831453</v>
+        <v>-1617034.99009451</v>
       </c>
       <c r="I18">
-        <v>-887265.1692795751</v>
+        <v>-206747.2640988243</v>
       </c>
       <c r="J18">
-        <v>-3530662.964551876</v>
+        <v>-1410287.725995686</v>
       </c>
       <c r="K18">
         <v>0</v>
       </c>
       <c r="L18">
-        <v>1056154.206809973</v>
+        <v>1137120.337121377</v>
       </c>
       <c r="M18">
         <v>0</v>
       </c>
       <c r="N18">
-        <v>1056154.206809973</v>
+        <v>1137120.337121377</v>
       </c>
       <c r="O18">
-        <v>506954.0192687869</v>
+        <v>545817.7618182609</v>
       </c>
       <c r="P18">
-        <v>283239.0509827895</v>
+        <v>304952.518356477</v>
       </c>
       <c r="Q18">
         <v>0</v>
       </c>
       <c r="R18">
-        <v>283239.0509827895</v>
+        <v>304952.518356477</v>
       </c>
       <c r="S18">
-        <v>135954.744471739</v>
+        <v>146377.208811109</v>
       </c>
     </row>
     <row r="19" spans="1:19">
@@ -1498,58 +1498,58 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>0.4979638342860216</v>
+        <v>0.3924884900515483</v>
       </c>
       <c r="C19">
-        <v>0.4026328375869891</v>
+        <v>0.5965255585436057</v>
       </c>
       <c r="D19">
-        <v>-1639759.834647078</v>
+        <v>-1290193.164844848</v>
       </c>
       <c r="E19">
         <v>0</v>
       </c>
       <c r="F19">
-        <v>-1639759.834647078</v>
+        <v>-1290193.164844848</v>
       </c>
       <c r="G19">
-        <v>-1639759.834647078</v>
+        <v>-1290193.164844848</v>
       </c>
       <c r="H19">
-        <v>-1855738.756554832</v>
+        <v>-1128883.99155638</v>
       </c>
       <c r="I19">
-        <v>-258629.9457988087</v>
+        <v>3184.627319237406</v>
       </c>
       <c r="J19">
-        <v>-1597108.810756024</v>
+        <v>-1132068.618875617</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
-        <v>1169105.879563188</v>
+        <v>1732102.979932356</v>
       </c>
       <c r="M19">
         <v>0</v>
       </c>
       <c r="N19">
-        <v>1169105.879563188</v>
+        <v>1732102.979932356</v>
       </c>
       <c r="O19">
-        <v>561170.8221903302</v>
+        <v>831409.4303675313</v>
       </c>
       <c r="P19">
-        <v>313530.3894930717</v>
+        <v>464514.7470673976</v>
       </c>
       <c r="Q19">
         <v>0</v>
       </c>
       <c r="R19">
-        <v>313530.3894930717</v>
+        <v>464514.7470673976</v>
       </c>
       <c r="S19">
-        <v>150494.5869566744</v>
+        <v>222967.0785923509</v>
       </c>
     </row>
     <row r="20" spans="1:19">
@@ -1557,58 +1557,58 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>0.4359008244682093</v>
+        <v>0.5063398733065707</v>
       </c>
       <c r="C20">
-        <v>0.3763306139131087</v>
+        <v>0.487593717618033</v>
       </c>
       <c r="D20">
-        <v>-2325563.672281628</v>
+        <v>-1030237.363446803</v>
       </c>
       <c r="E20">
         <v>0</v>
       </c>
       <c r="F20">
-        <v>-2325563.672281628</v>
+        <v>-1030237.363446803</v>
       </c>
       <c r="G20">
-        <v>-2325563.672281628</v>
+        <v>-1030237.363446803</v>
       </c>
       <c r="H20">
-        <v>-2862427.865815748</v>
+        <v>-888096.2865612095</v>
       </c>
       <c r="I20">
-        <v>-510652.1726520555</v>
+        <v>10862.32152348454</v>
       </c>
       <c r="J20">
-        <v>-2351775.693163693</v>
+        <v>-898958.6080846939</v>
       </c>
       <c r="K20">
         <v>0</v>
       </c>
       <c r="L20">
-        <v>1092733.359807951</v>
+        <v>1415802.758467647</v>
       </c>
       <c r="M20">
         <v>0</v>
       </c>
       <c r="N20">
-        <v>1092733.359807951</v>
+        <v>1415802.758467647</v>
       </c>
       <c r="O20">
-        <v>524512.0127078163</v>
+        <v>679585.3240644706</v>
       </c>
       <c r="P20">
-        <v>293048.8349273094</v>
+        <v>379689.4687362101</v>
       </c>
       <c r="Q20">
         <v>0</v>
       </c>
       <c r="R20">
-        <v>293048.8349273094</v>
+        <v>379689.4687362101</v>
       </c>
       <c r="S20">
-        <v>140663.4407651085</v>
+        <v>182250.9449933809</v>
       </c>
     </row>
     <row r="21" spans="1:19">
@@ -1616,58 +1616,58 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>0.5608061844165049</v>
+        <v>0.4481046645540333</v>
       </c>
       <c r="C21">
-        <v>0.4968802326355326</v>
+        <v>0.4288980269312649</v>
       </c>
       <c r="D21">
-        <v>-515985.0264876551</v>
+        <v>-1889745.453828607</v>
       </c>
       <c r="E21">
         <v>0</v>
       </c>
       <c r="F21">
-        <v>-515985.0264876551</v>
+        <v>-1889745.453828607</v>
       </c>
       <c r="G21">
-        <v>-515985.0264876551</v>
+        <v>-1889745.453828607</v>
       </c>
       <c r="H21">
-        <v>-145585.4425827528</v>
+        <v>-2180235.869294892</v>
       </c>
       <c r="I21">
-        <v>192131.060038563</v>
+        <v>-324005.5367452815</v>
       </c>
       <c r="J21">
-        <v>-337716.5026213155</v>
+        <v>-1856230.33254961</v>
       </c>
       <c r="K21">
         <v>0</v>
       </c>
       <c r="L21">
-        <v>1442767.571801495</v>
+        <v>1245370.864491545</v>
       </c>
       <c r="M21">
         <v>0</v>
       </c>
       <c r="N21">
-        <v>1442767.571801495</v>
+        <v>1245370.864491545</v>
       </c>
       <c r="O21">
-        <v>692528.4344647175</v>
+        <v>597778.0149559417</v>
       </c>
       <c r="P21">
-        <v>386920.8825670328</v>
+        <v>333983.1054080792</v>
       </c>
       <c r="Q21">
         <v>0</v>
       </c>
       <c r="R21">
-        <v>386920.8825670328</v>
+        <v>333983.1054080792</v>
       </c>
       <c r="S21">
-        <v>185722.0236321757</v>
+        <v>160311.890595878</v>
       </c>
     </row>
     <row r="22" spans="1:19">
@@ -1675,58 +1675,58 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0.3083584060422998</v>
+        <v>0.3867294601586262</v>
       </c>
       <c r="C22">
-        <v>0.3942331642642312</v>
+        <v>0.2922639139478632</v>
       </c>
       <c r="D22">
-        <v>-3278004.667308845</v>
+        <v>-3270414.99200086</v>
       </c>
       <c r="E22">
         <v>0</v>
       </c>
       <c r="F22">
-        <v>-3278004.667308845</v>
+        <v>-3270414.99200086</v>
       </c>
       <c r="G22">
-        <v>-3278004.667308845</v>
+        <v>-3270414.99200086</v>
       </c>
       <c r="H22">
-        <v>-4196056.966928101</v>
+        <v>-4306010.258347615</v>
       </c>
       <c r="I22">
-        <v>-820442.4349740908</v>
+        <v>-893209.6330893795</v>
       </c>
       <c r="J22">
-        <v>-3375614.531954011</v>
+        <v>-3412800.625258234</v>
       </c>
       <c r="K22">
         <v>0</v>
       </c>
       <c r="L22">
-        <v>1144716.146408537</v>
+        <v>848632.8691627758</v>
       </c>
       <c r="M22">
         <v>0</v>
       </c>
       <c r="N22">
-        <v>1144716.146408538</v>
+        <v>848632.8691627758</v>
       </c>
       <c r="O22">
-        <v>549463.7502760981</v>
+        <v>407343.7771981324</v>
       </c>
       <c r="P22">
-        <v>306989.5597279638</v>
+        <v>227586.0541430518</v>
       </c>
       <c r="Q22">
         <v>0</v>
       </c>
       <c r="R22">
-        <v>306989.5597279638</v>
+        <v>227586.0541430518</v>
       </c>
       <c r="S22">
-        <v>147354.9886694226</v>
+        <v>109241.3059886649</v>
       </c>
     </row>
     <row r="23" spans="1:19">
@@ -1734,58 +1734,58 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>0.4632434885172499</v>
+        <v>0.3006271609319814</v>
       </c>
       <c r="C23">
-        <v>0.3324843487367175</v>
+        <v>0.4519011420205494</v>
       </c>
       <c r="D23">
-        <v>-2375433.912278038</v>
+        <v>-2976434.318720251</v>
       </c>
       <c r="E23">
         <v>0</v>
       </c>
       <c r="F23">
-        <v>-2375433.912278038</v>
+        <v>-2976434.318720251</v>
       </c>
       <c r="G23">
-        <v>-2375433.912278038</v>
+        <v>-2976434.318720251</v>
       </c>
       <c r="H23">
-        <v>-2985288.975598224</v>
+        <v>-3698790.001314004</v>
       </c>
       <c r="I23">
-        <v>-559961.8733973966</v>
+        <v>-675556.9857343696</v>
       </c>
       <c r="J23">
-        <v>-2425327.102200828</v>
+        <v>-3023233.015579635</v>
       </c>
       <c r="K23">
         <v>0</v>
       </c>
       <c r="L23">
-        <v>965419.0385970515</v>
+        <v>1312163.919077761</v>
       </c>
       <c r="M23">
         <v>0</v>
       </c>
       <c r="N23">
-        <v>965419.0385970515</v>
+        <v>1312163.919077761</v>
       </c>
       <c r="O23">
-        <v>463401.1385265848</v>
+        <v>629838.6811573257</v>
       </c>
       <c r="P23">
-        <v>258905.7265783776</v>
+        <v>351895.6424895563</v>
       </c>
       <c r="Q23">
         <v>0</v>
       </c>
       <c r="R23">
-        <v>258905.7265783776</v>
+        <v>351895.6424895563</v>
       </c>
       <c r="S23">
-        <v>124274.7487576212</v>
+        <v>168909.9083949871</v>
       </c>
     </row>
     <row r="24" spans="1:19">
@@ -1793,58 +1793,58 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0.4731755041299949</v>
+        <v>0.5846405528056907</v>
       </c>
       <c r="C24">
-        <v>0.4017019801543336</v>
+        <v>0.4223941057117254</v>
       </c>
       <c r="D24">
-        <v>-1852875.783296529</v>
+        <v>-789746.2277622599</v>
       </c>
       <c r="E24">
         <v>0</v>
       </c>
       <c r="F24">
-        <v>-1852875.783296529</v>
+        <v>-789746.2277622599</v>
       </c>
       <c r="G24">
-        <v>-1852875.783296529</v>
+        <v>-789746.2277622599</v>
       </c>
       <c r="H24">
-        <v>-2159994.361641768</v>
+        <v>-623210.0702454419</v>
       </c>
       <c r="I24">
-        <v>-331595.4166752624</v>
+        <v>44250.7143810495</v>
       </c>
       <c r="J24">
-        <v>-1828398.944966506</v>
+        <v>-667460.7846264911</v>
       </c>
       <c r="K24">
         <v>0</v>
       </c>
       <c r="L24">
-        <v>1166402.992972828</v>
+        <v>1226485.736831443</v>
       </c>
       <c r="M24">
         <v>0</v>
       </c>
       <c r="N24">
-        <v>1166402.992972828</v>
+        <v>1226485.736831443</v>
       </c>
       <c r="O24">
-        <v>559873.4366269573</v>
+        <v>588713.1536790928</v>
       </c>
       <c r="P24">
-        <v>312805.5303505037</v>
+        <v>328918.498742077</v>
       </c>
       <c r="Q24">
         <v>0</v>
       </c>
       <c r="R24">
-        <v>312805.5303505037</v>
+        <v>328918.498742077</v>
       </c>
       <c r="S24">
-        <v>150146.6545682418</v>
+        <v>157880.8793961969</v>
       </c>
     </row>
     <row r="25" spans="1:19">
@@ -1852,58 +1852,58 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>0.3307860686894607</v>
+        <v>0.4381145246356116</v>
       </c>
       <c r="C25">
-        <v>0.3307804405967001</v>
+        <v>0.282684498660275</v>
       </c>
       <c r="D25">
-        <v>-3493461.615890956</v>
+        <v>-2901718.655498887</v>
       </c>
       <c r="E25">
         <v>0</v>
       </c>
       <c r="F25">
-        <v>-3493461.615890956</v>
+        <v>-2901718.655498887</v>
       </c>
       <c r="G25">
-        <v>-3493461.615890956</v>
+        <v>-2901718.655498887</v>
       </c>
       <c r="H25">
-        <v>-4577679.442547716</v>
+        <v>-3792890.570972144</v>
       </c>
       <c r="I25">
-        <v>-940396.8879098063</v>
+        <v>-775245.1382450842</v>
       </c>
       <c r="J25">
-        <v>-3637282.55463791</v>
+        <v>-3017645.432727059</v>
       </c>
       <c r="K25">
         <v>0</v>
       </c>
       <c r="L25">
-        <v>960471.4813221196</v>
+        <v>820817.5752026126</v>
       </c>
       <c r="M25">
         <v>0</v>
       </c>
       <c r="N25">
-        <v>960471.4813221198</v>
+        <v>820817.5752026126</v>
       </c>
       <c r="O25">
-        <v>461026.3110346177</v>
+        <v>393992.4360972541</v>
       </c>
       <c r="P25">
-        <v>257578.89246817</v>
+        <v>220126.5587272451</v>
       </c>
       <c r="Q25">
         <v>0</v>
       </c>
       <c r="R25">
-        <v>257578.8924681701</v>
+        <v>220126.5587272451</v>
       </c>
       <c r="S25">
-        <v>123637.8683847216</v>
+        <v>105660.7481890776</v>
       </c>
     </row>
     <row r="26" spans="1:19">
@@ -1911,58 +1911,58 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0.5314785154131337</v>
+        <v>0.4948403608465582</v>
       </c>
       <c r="C26">
-        <v>0.3715211669215683</v>
+        <v>0.2986978017126054</v>
       </c>
       <c r="D26">
-        <v>-1557172.814566911</v>
+        <v>-2325863.448790676</v>
       </c>
       <c r="E26">
         <v>0</v>
       </c>
       <c r="F26">
-        <v>-1557172.814566911</v>
+        <v>-2325863.448790676</v>
       </c>
       <c r="G26">
-        <v>-1557172.814566911</v>
+        <v>-2325863.448790676</v>
       </c>
       <c r="H26">
-        <v>-1775101.989868708</v>
+        <v>-2954785.143058513</v>
       </c>
       <c r="I26">
-        <v>-253608.0168525645</v>
+        <v>-568113.7848145892</v>
       </c>
       <c r="J26">
-        <v>-1521493.973016144</v>
+        <v>-2386671.358243924</v>
       </c>
       <c r="K26">
         <v>0</v>
       </c>
       <c r="L26">
-        <v>1078768.396619764</v>
+        <v>867314.644000837</v>
       </c>
       <c r="M26">
         <v>0</v>
       </c>
       <c r="N26">
-        <v>1078768.396619764</v>
+        <v>867314.6440008369</v>
       </c>
       <c r="O26">
-        <v>517808.8303774868</v>
+        <v>416311.0291204018</v>
       </c>
       <c r="P26">
-        <v>289303.7161795665</v>
+        <v>232596.1257232134</v>
       </c>
       <c r="Q26">
         <v>0</v>
       </c>
       <c r="R26">
-        <v>289303.7161795665</v>
+        <v>232596.1257232134</v>
       </c>
       <c r="S26">
-        <v>138865.7837661919</v>
+        <v>111646.1403471424</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update notebook and data files with latest changes
- Updated BioDYM_Scientific_Notebook.ipynb with latest enhancements
- Updated Excel data files with new visualization configurations
- Updated output results files
- Includes all Sankey diagram improvements and element-specific positioning
</commit_message>
<xml_diff>
--- a/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
+++ b/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
@@ -495,58 +495,58 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>0.440470713700875</v>
+        <v>0.34522233018487</v>
       </c>
       <c r="C2">
-        <v>0.3562893583592965</v>
+        <v>0.2555495550859855</v>
       </c>
       <c r="D2">
-        <v>-2414627.443401478</v>
+        <v>-3850510.590916542</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>-2414627.443401478</v>
+        <v>-3850510.590916542</v>
       </c>
       <c r="G2">
-        <v>-2414627.443401478</v>
+        <v>-3850510.590916542</v>
       </c>
       <c r="H2">
-        <v>-3012851.71200933</v>
+        <v>-5174661.238916159</v>
       </c>
       <c r="I2">
-        <v>-555665.6333620335</v>
+        <v>-1117074.329895339</v>
       </c>
       <c r="J2">
-        <v>-2457186.078647296</v>
+        <v>-4057586.90902082</v>
       </c>
       <c r="K2">
         <v>0</v>
       </c>
       <c r="L2">
-        <v>1034540.516317563</v>
+        <v>742027.1261561824</v>
       </c>
       <c r="M2">
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1034540.516317563</v>
+        <v>742027.1261561824</v>
       </c>
       <c r="O2">
-        <v>496579.4478324305</v>
+        <v>356173.0205549677</v>
       </c>
       <c r="P2">
-        <v>277442.6993289943</v>
+        <v>198996.5647637463</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
       <c r="R2">
-        <v>277442.6993289943</v>
+        <v>198996.5647637462</v>
       </c>
       <c r="S2">
-        <v>133172.4956779173</v>
+        <v>95518.35108659824</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -554,58 +554,58 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>0.4408971156159481</v>
+        <v>0.3828060085590773</v>
       </c>
       <c r="C3">
-        <v>0.3948080795693732</v>
+        <v>0.3845953868945471</v>
       </c>
       <c r="D3">
-        <v>-2166466.646793793</v>
+        <v>-2716899.840524348</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3">
-        <v>-2166466.646793793</v>
+        <v>-2716899.840524348</v>
       </c>
       <c r="G3">
-        <v>-2166466.646793793</v>
+        <v>-2716899.840524348</v>
       </c>
       <c r="H3">
-        <v>-2614234.873733097</v>
+        <v>-3409309.041902732</v>
       </c>
       <c r="I3">
-        <v>-443042.5489044277</v>
+        <v>-637266.2443805467</v>
       </c>
       <c r="J3">
-        <v>-2171192.324828668</v>
+        <v>-2772042.797522184</v>
       </c>
       <c r="K3">
         <v>0</v>
       </c>
       <c r="L3">
-        <v>1146385.500720324</v>
+        <v>1116731.389237846</v>
       </c>
       <c r="M3">
         <v>0</v>
       </c>
       <c r="N3">
-        <v>1146385.500720324</v>
+        <v>1116731.389237846</v>
       </c>
       <c r="O3">
-        <v>550265.0403457554</v>
+        <v>536031.0668341659</v>
       </c>
       <c r="P3">
-        <v>307437.2465600337</v>
+        <v>299484.6177300033</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
       <c r="R3">
-        <v>307437.2465600338</v>
+        <v>299484.6177300033</v>
       </c>
       <c r="S3">
-        <v>147569.8783488162</v>
+        <v>143752.6165104016</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -613,58 +613,58 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.4530374786246817</v>
+        <v>0.3745972271998492</v>
       </c>
       <c r="C4">
-        <v>0.4140134752942853</v>
+        <v>0.2841721824448926</v>
       </c>
       <c r="D4">
-        <v>-1943030.123937516</v>
+        <v>-3423211.027766681</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>-1943030.123937516</v>
+        <v>-3423211.027766681</v>
       </c>
       <c r="G4">
-        <v>-1943030.123937516</v>
+        <v>-3423211.027766681</v>
       </c>
       <c r="H4">
-        <v>-2273658.196798186</v>
+        <v>-4532941.685837532</v>
       </c>
       <c r="I4">
-        <v>-353074.5192926812</v>
+        <v>-951008.6677771308</v>
       </c>
       <c r="J4">
-        <v>-1920583.677505506</v>
+        <v>-3581933.018060402</v>
       </c>
       <c r="K4">
         <v>0</v>
       </c>
       <c r="L4">
-        <v>1202151.29765804</v>
+        <v>825137.2920691028</v>
       </c>
       <c r="M4">
         <v>0</v>
       </c>
       <c r="N4">
-        <v>1202151.29765804</v>
+        <v>825137.2920691026</v>
       </c>
       <c r="O4">
-        <v>577032.6228758591</v>
+        <v>396065.9001931692</v>
       </c>
       <c r="P4">
-        <v>322392.4976967455</v>
+        <v>221285.0188251076</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
       <c r="R4">
-        <v>322392.4976967455</v>
+        <v>221285.0188251076</v>
       </c>
       <c r="S4">
-        <v>154748.3988944379</v>
+        <v>106216.8090360517</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -672,58 +672,58 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>0.4646829360384797</v>
+        <v>0.4460138703083529</v>
       </c>
       <c r="C5">
-        <v>0.4442838849451958</v>
+        <v>0.4587748038299565</v>
       </c>
       <c r="D5">
-        <v>-1653466.907215537</v>
+        <v>-1717502.765358558</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>-1653466.907215537</v>
+        <v>-1717502.765358558</v>
       </c>
       <c r="G5">
-        <v>-1653466.907215537</v>
+        <v>-1717502.765358558</v>
       </c>
       <c r="H5">
-        <v>-1825914.664277845</v>
+        <v>-1899844.644702633</v>
       </c>
       <c r="I5">
-        <v>-232504.2813391603</v>
+        <v>-243515.0778668632</v>
       </c>
       <c r="J5">
-        <v>-1593410.382938684</v>
+        <v>-1656329.56683577</v>
       </c>
       <c r="K5">
         <v>0</v>
       </c>
       <c r="L5">
-        <v>1290046.050882235</v>
+        <v>1332122.644957319</v>
       </c>
       <c r="M5">
         <v>0</v>
       </c>
       <c r="N5">
-        <v>1290046.050882235</v>
+        <v>1332122.644957319</v>
       </c>
       <c r="O5">
-        <v>619222.1044234727</v>
+        <v>639418.8695795131</v>
       </c>
       <c r="P5">
-        <v>345964.0806427447</v>
+        <v>357248.1663355068</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
       <c r="R5">
-        <v>345964.0806427448</v>
+        <v>357248.1663355069</v>
       </c>
       <c r="S5">
-        <v>166062.7587085175</v>
+        <v>171479.1198410433</v>
       </c>
     </row>
     <row r="6" spans="1:19">
@@ -731,58 +731,58 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>0.4935839306456321</v>
+        <v>0.4088256478347204</v>
       </c>
       <c r="C6">
-        <v>0.5848351040346516</v>
+        <v>0.4431738989025407</v>
       </c>
       <c r="D6">
-        <v>-519374.4647446815</v>
+        <v>-2127424.863325496</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
       <c r="F6">
-        <v>-519374.4647446815</v>
+        <v>-2127424.863325496</v>
       </c>
       <c r="G6">
-        <v>-519374.4647446815</v>
+        <v>-2127424.863325496</v>
       </c>
       <c r="H6">
-        <v>-46252.87532518356</v>
+        <v>-2501425.089557387</v>
       </c>
       <c r="I6">
-        <v>255968.0635107075</v>
+        <v>-394065.9624614074</v>
       </c>
       <c r="J6">
-        <v>-302220.938835891</v>
+        <v>-2107359.127095981</v>
       </c>
       <c r="K6">
         <v>0</v>
       </c>
       <c r="L6">
-        <v>1698157.961480572</v>
+        <v>1286823.037040447</v>
       </c>
       <c r="M6">
         <v>0</v>
       </c>
       <c r="N6">
-        <v>1698157.961480572</v>
+        <v>1286823.037040447</v>
       </c>
       <c r="O6">
-        <v>815115.8215106749</v>
+        <v>617675.0577794146</v>
       </c>
       <c r="P6">
-        <v>455411.3843672512</v>
+        <v>345099.7339630968</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
       <c r="R6">
-        <v>455411.3843672512</v>
+        <v>345099.7339630968</v>
       </c>
       <c r="S6">
-        <v>218597.4644962806</v>
+        <v>165647.8723022865</v>
       </c>
     </row>
     <row r="7" spans="1:19">
@@ -790,58 +790,58 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>0.4668787776140075</v>
+        <v>0.3321281256066577</v>
       </c>
       <c r="C7">
-        <v>0.6661833119258669</v>
+        <v>0.3987151076406868</v>
       </c>
       <c r="D7">
-        <v>-226035.3862292718</v>
+        <v>-3050853.616639365</v>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
       <c r="F7">
-        <v>-226035.3862292718</v>
+        <v>-3050853.616639365</v>
       </c>
       <c r="G7">
-        <v>-226035.3862292718</v>
+        <v>-3050853.616639365</v>
       </c>
       <c r="H7">
-        <v>467346.8094031098</v>
+        <v>-3867631.59330558</v>
       </c>
       <c r="I7">
-        <v>415558.3247529726</v>
+        <v>-740093.2344699338</v>
       </c>
       <c r="J7">
-        <v>51788.48465013769</v>
+        <v>-3127538.358835646</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
       <c r="L7">
-        <v>1934364.895588377</v>
+        <v>1157730.152878269</v>
       </c>
       <c r="M7">
         <v>0</v>
       </c>
       <c r="N7">
-        <v>1934364.895588377</v>
+        <v>1157730.152878269</v>
       </c>
       <c r="O7">
-        <v>928495.1498824214</v>
+        <v>555710.4733815693</v>
       </c>
       <c r="P7">
-        <v>518757.2740307731</v>
+        <v>310479.651248883</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
       <c r="R7">
-        <v>518757.2740307731</v>
+        <v>310479.6512488829</v>
       </c>
       <c r="S7">
-        <v>249003.4915347711</v>
+        <v>149030.2325994639</v>
       </c>
     </row>
     <row r="8" spans="1:19">
@@ -849,58 +849,58 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0.507124546745101</v>
+        <v>0.4315364791177262</v>
       </c>
       <c r="C8">
-        <v>0.4557932680542008</v>
+        <v>0.3212372623793684</v>
       </c>
       <c r="D8">
-        <v>-1225613.331299989</v>
+        <v>-2711891.66166902</v>
       </c>
       <c r="E8">
         <v>0</v>
       </c>
       <c r="F8">
-        <v>-1225613.331299989</v>
+        <v>-2711891.66166902</v>
       </c>
       <c r="G8">
-        <v>-1225613.331299989</v>
+        <v>-2711891.66166902</v>
       </c>
       <c r="H8">
-        <v>-1203672.118220932</v>
+        <v>-3477212.124352356</v>
       </c>
       <c r="I8">
-        <v>-78895.05512663237</v>
+        <v>-682380.6519608214</v>
       </c>
       <c r="J8">
-        <v>-1124777.0630943</v>
+        <v>-2794831.472391534</v>
       </c>
       <c r="K8">
         <v>0</v>
       </c>
       <c r="L8">
-        <v>1323465.300895532</v>
+        <v>932761.4072246708</v>
       </c>
       <c r="M8">
         <v>0</v>
       </c>
       <c r="N8">
-        <v>1323465.300895532</v>
+        <v>932761.4072246706</v>
       </c>
       <c r="O8">
-        <v>635263.3444298556</v>
+        <v>447725.475467842</v>
       </c>
       <c r="P8">
-        <v>354926.4429543178</v>
+        <v>250147.6148768699</v>
       </c>
       <c r="Q8">
         <v>0</v>
       </c>
       <c r="R8">
-        <v>354926.4429543178</v>
+        <v>250147.6148768699</v>
       </c>
       <c r="S8">
-        <v>170364.6926180726</v>
+        <v>120070.8551408975</v>
       </c>
     </row>
     <row r="9" spans="1:19">
@@ -908,58 +908,58 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0.545973976342663</v>
+        <v>0.3910721015325745</v>
       </c>
       <c r="C9">
-        <v>0.2757430781396258</v>
+        <v>0.6030613867224857</v>
       </c>
       <c r="D9">
-        <v>-2044203.089889325</v>
+        <v>-1260529.759684632</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
       <c r="F9">
-        <v>-2044203.089889325</v>
+        <v>-1260529.759684632</v>
       </c>
       <c r="G9">
-        <v>-2044203.089889325</v>
+        <v>-1260529.759684632</v>
       </c>
       <c r="H9">
-        <v>-2581311.155449423</v>
+        <v>-1078948.806942713</v>
       </c>
       <c r="I9">
-        <v>-489549.814118128</v>
+        <v>18073.96650045061</v>
       </c>
       <c r="J9">
-        <v>-2091761.341331295</v>
+        <v>-1097022.773443164</v>
       </c>
       <c r="K9">
         <v>0</v>
       </c>
       <c r="L9">
-        <v>800662.1015660189</v>
+        <v>1751080.754317418</v>
       </c>
       <c r="M9">
         <v>0</v>
       </c>
       <c r="N9">
-        <v>800662.1015660189</v>
+        <v>1751080.754317418</v>
       </c>
       <c r="O9">
-        <v>384317.8087516892</v>
+        <v>840518.7620723612</v>
       </c>
       <c r="P9">
-        <v>214721.2711393838</v>
+        <v>469604.1996983973</v>
       </c>
       <c r="Q9">
         <v>0</v>
       </c>
       <c r="R9">
-        <v>214721.2711393838</v>
+        <v>469604.1996983974</v>
       </c>
       <c r="S9">
-        <v>103066.2101469043</v>
+        <v>225410.0158552308</v>
       </c>
     </row>
     <row r="10" spans="1:19">
@@ -967,58 +967,58 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0.5406512389940892</v>
+        <v>0.3105435299003277</v>
       </c>
       <c r="C10">
-        <v>0.3572397216799597</v>
+        <v>0.350018690224925</v>
       </c>
       <c r="D10">
-        <v>-1571186.435902989</v>
+        <v>-3540504.215123716</v>
       </c>
       <c r="E10">
         <v>0</v>
       </c>
       <c r="F10">
-        <v>-1571186.435902989</v>
+        <v>-3540504.215123716</v>
       </c>
       <c r="G10">
-        <v>-1571186.435902989</v>
+        <v>-3540504.215123716</v>
       </c>
       <c r="H10">
-        <v>-1811947.827922707</v>
+        <v>-4621815.170163461</v>
       </c>
       <c r="I10">
-        <v>-268912.7173241808</v>
+        <v>-942136.8439668739</v>
       </c>
       <c r="J10">
-        <v>-1543035.110598525</v>
+        <v>-3679678.326196585</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>1037300.041230055</v>
+        <v>1016332.67458111</v>
       </c>
       <c r="M10">
         <v>0</v>
       </c>
       <c r="N10">
-        <v>1037300.041230055</v>
+        <v>1016332.67458111</v>
       </c>
       <c r="O10">
-        <v>497904.0197904264</v>
+        <v>487839.6837989325</v>
       </c>
       <c r="P10">
-        <v>278182.747716188</v>
+        <v>272559.7269556183</v>
       </c>
       <c r="Q10">
         <v>0</v>
       </c>
       <c r="R10">
-        <v>278182.747716188</v>
+        <v>272559.7269556183</v>
       </c>
       <c r="S10">
-        <v>133527.7189037702</v>
+        <v>130828.6689386968</v>
       </c>
     </row>
     <row r="11" spans="1:19">
@@ -1026,58 +1026,58 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0.3504549342384379</v>
+        <v>0.5250865833279799</v>
       </c>
       <c r="C11">
-        <v>0.4209585612244957</v>
+        <v>0.5355603624448535</v>
       </c>
       <c r="D11">
-        <v>-2756412.897117089</v>
+        <v>-568942.6758180009</v>
       </c>
       <c r="E11">
         <v>0</v>
       </c>
       <c r="F11">
-        <v>-2756412.897117089</v>
+        <v>-568942.6758180009</v>
       </c>
       <c r="G11">
-        <v>-2756412.897117089</v>
+        <v>-568942.6758180009</v>
       </c>
       <c r="H11">
-        <v>-3422455.22988882</v>
+        <v>-175112.6219641669</v>
       </c>
       <c r="I11">
-        <v>-623799.6184116157</v>
+        <v>202749.8994938763</v>
       </c>
       <c r="J11">
-        <v>-2798655.611477204</v>
+        <v>-377862.5214580427</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>1222317.41437058</v>
+        <v>1555081.230700651</v>
       </c>
       <c r="M11">
         <v>0</v>
       </c>
       <c r="N11">
-        <v>1222317.41437058</v>
+        <v>1555081.230700651</v>
       </c>
       <c r="O11">
-        <v>586712.3588978784</v>
+        <v>746438.9907363126</v>
       </c>
       <c r="P11">
-        <v>327800.6395408424</v>
+        <v>417041.1187540249</v>
       </c>
       <c r="Q11">
         <v>0</v>
       </c>
       <c r="R11">
-        <v>327800.6395408424</v>
+        <v>417041.1187540249</v>
       </c>
       <c r="S11">
-        <v>157344.3069796044</v>
+        <v>200179.7370019319</v>
       </c>
     </row>
     <row r="12" spans="1:19">
@@ -1085,58 +1085,58 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>0.5024346377785431</v>
+        <v>0.3233829555814128</v>
       </c>
       <c r="C12">
-        <v>0.4701442422227763</v>
+        <v>0.3029090018680389</v>
       </c>
       <c r="D12">
-        <v>-1173686.477831411</v>
+        <v>-3732329.56883131</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
       <c r="F12">
-        <v>-1173686.477831411</v>
+        <v>-3732329.56883131</v>
       </c>
       <c r="G12">
-        <v>-1173686.477831411</v>
+        <v>-3732329.56883131</v>
       </c>
       <c r="H12">
-        <v>-1112813.107779967</v>
+        <v>-4950469.142931724</v>
       </c>
       <c r="I12">
-        <v>-50680.81258419952</v>
+        <v>-1042001.456011158</v>
       </c>
       <c r="J12">
-        <v>-1062132.295195768</v>
+        <v>-3908467.686920565</v>
       </c>
       <c r="K12">
         <v>0</v>
       </c>
       <c r="L12">
-        <v>1365135.544133743</v>
+        <v>879542.5062170455</v>
       </c>
       <c r="M12">
         <v>0</v>
       </c>
       <c r="N12">
-        <v>1365135.544133743</v>
+        <v>879542.5062170455</v>
       </c>
       <c r="O12">
-        <v>655265.0611841967</v>
+        <v>422180.4029841819</v>
       </c>
       <c r="P12">
-        <v>366101.5536274666</v>
+        <v>235875.3893642002</v>
       </c>
       <c r="Q12">
         <v>0</v>
       </c>
       <c r="R12">
-        <v>366101.5536274666</v>
+        <v>235875.3893642002</v>
       </c>
       <c r="S12">
-        <v>175728.7457411839</v>
+        <v>113220.1868948161</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -1144,58 +1144,58 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>0.4988428324318666</v>
+        <v>0.4532946828667089</v>
       </c>
       <c r="C13">
-        <v>0.3639467539397552</v>
+        <v>0.5204661465921996</v>
       </c>
       <c r="D13">
-        <v>-1878071.592542547</v>
+        <v>-1264898.414540258</v>
       </c>
       <c r="E13">
         <v>0</v>
       </c>
       <c r="F13">
-        <v>-1878071.592542547</v>
+        <v>-1264898.414540258</v>
       </c>
       <c r="G13">
-        <v>-1878071.592542547</v>
+        <v>-1264898.414540258</v>
       </c>
       <c r="H13">
-        <v>-2240543.714583392</v>
+        <v>-1182970.368868954</v>
       </c>
       <c r="I13">
-        <v>-368036.4132717596</v>
+        <v>-44434.14470334642</v>
       </c>
       <c r="J13">
-        <v>-1872507.301311633</v>
+        <v>-1138536.224165607</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13">
-        <v>1056774.932787187</v>
+        <v>1511252.871825374</v>
       </c>
       <c r="M13">
         <v>0</v>
       </c>
       <c r="N13">
-        <v>1056774.932787187</v>
+        <v>1511252.871825374</v>
       </c>
       <c r="O13">
-        <v>507251.9677378498</v>
+        <v>725401.3784761798</v>
       </c>
       <c r="P13">
-        <v>283405.517049556</v>
+        <v>405287.2454143903</v>
       </c>
       <c r="Q13">
         <v>0</v>
       </c>
       <c r="R13">
-        <v>283405.517049556</v>
+        <v>405287.2454143904</v>
       </c>
       <c r="S13">
-        <v>136034.6481837869</v>
+        <v>194537.8777989074</v>
       </c>
     </row>
     <row r="14" spans="1:19">
@@ -1203,58 +1203,58 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>0.4392692437158223</v>
+        <v>0.3016555482256449</v>
       </c>
       <c r="C14">
-        <v>0.5432554326675922</v>
+        <v>0.156872529693451</v>
       </c>
       <c r="D14">
-        <v>-1237423.131938945</v>
+        <v>-4841289.933781915</v>
       </c>
       <c r="E14">
         <v>0</v>
       </c>
       <c r="F14">
-        <v>-1237423.131938945</v>
+        <v>-4841289.933781915</v>
       </c>
       <c r="G14">
-        <v>-1237423.131938945</v>
+        <v>-4841289.933781915</v>
       </c>
       <c r="H14">
-        <v>-1116900.804423215</v>
+        <v>-6700876.53934056</v>
       </c>
       <c r="I14">
-        <v>-18277.83708087195</v>
+        <v>-1526003.170671528</v>
       </c>
       <c r="J14">
-        <v>-1098622.967342343</v>
+        <v>-5174873.368669032</v>
       </c>
       <c r="K14">
         <v>0</v>
       </c>
       <c r="L14">
-        <v>1577425.04124271</v>
+        <v>455503.3263200758</v>
       </c>
       <c r="M14">
         <v>0</v>
       </c>
       <c r="N14">
-        <v>1577425.04124271</v>
+        <v>455503.3263200758</v>
       </c>
       <c r="O14">
-        <v>757164.0197965013</v>
+        <v>218641.5966336364</v>
       </c>
       <c r="P14">
-        <v>423033.2737371379</v>
+        <v>122156.7163530839</v>
       </c>
       <c r="Q14">
         <v>0</v>
       </c>
       <c r="R14">
-        <v>423033.273737138</v>
+        <v>122156.7163530839</v>
       </c>
       <c r="S14">
-        <v>203055.9713938262</v>
+        <v>58635.22384948028</v>
       </c>
     </row>
     <row r="15" spans="1:19">
@@ -1262,58 +1262,58 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0.5069431517968397</v>
+        <v>0.3783202865060128</v>
       </c>
       <c r="C15">
-        <v>0.3875839846428868</v>
+        <v>0.4315890733362706</v>
       </c>
       <c r="D15">
-        <v>-1660263.223190929</v>
+        <v>-2455982.73806981</v>
       </c>
       <c r="E15">
         <v>0</v>
       </c>
       <c r="F15">
-        <v>-1660263.223190929</v>
+        <v>-2455982.73806981</v>
       </c>
       <c r="G15">
-        <v>-1660263.223190929</v>
+        <v>-2455982.73806981</v>
       </c>
       <c r="H15">
-        <v>-1902724.907861322</v>
+        <v>-2982510.762120486</v>
       </c>
       <c r="I15">
-        <v>-276702.6416833528</v>
+        <v>-514055.0626847941</v>
       </c>
       <c r="J15">
-        <v>-1626022.266177969</v>
+        <v>-2468455.699435693</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
-        <v>1125409.238814579</v>
+        <v>1253184.728341112</v>
       </c>
       <c r="M15">
         <v>0</v>
       </c>
       <c r="N15">
-        <v>1125409.238814579</v>
+        <v>1253184.728341112</v>
       </c>
       <c r="O15">
-        <v>540196.4346309979</v>
+        <v>601528.6696037337</v>
       </c>
       <c r="P15">
-        <v>301811.8402727315</v>
+        <v>336078.6245727899</v>
       </c>
       <c r="Q15">
         <v>0</v>
       </c>
       <c r="R15">
-        <v>301811.8402727315</v>
+        <v>336078.6245727899</v>
       </c>
       <c r="S15">
-        <v>144869.6833309111</v>
+        <v>161317.7397949391</v>
       </c>
     </row>
     <row r="16" spans="1:19">
@@ -1321,58 +1321,58 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>0.3213104921765115</v>
+        <v>0.3862821106782843</v>
       </c>
       <c r="C16">
-        <v>0.3079302067463411</v>
+        <v>0.3079012190991818</v>
       </c>
       <c r="D16">
-        <v>-3717768.236404144</v>
+        <v>-3174856.415809009</v>
       </c>
       <c r="E16">
         <v>0</v>
       </c>
       <c r="F16">
-        <v>-3717768.236404144</v>
+        <v>-3174856.415809009</v>
       </c>
       <c r="G16">
-        <v>-3717768.236404144</v>
+        <v>-3174856.415809009</v>
       </c>
       <c r="H16">
-        <v>-4923809.943455936</v>
+        <v>-4151562.726659162</v>
       </c>
       <c r="I16">
-        <v>-1033353.041584632</v>
+        <v>-849247.3889725171</v>
       </c>
       <c r="J16">
-        <v>-3890456.901871305</v>
+        <v>-3302315.337686644</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
       <c r="L16">
-        <v>894122.3407404682</v>
+        <v>894038.1706838683</v>
       </c>
       <c r="M16">
         <v>0</v>
       </c>
       <c r="N16">
-        <v>894122.3407404682</v>
+        <v>894038.1706838683</v>
       </c>
       <c r="O16">
-        <v>429178.7235554248</v>
+        <v>429138.3219282568</v>
       </c>
       <c r="P16">
-        <v>239785.4040829536</v>
+        <v>239762.8313877934</v>
       </c>
       <c r="Q16">
         <v>0</v>
       </c>
       <c r="R16">
-        <v>239785.4040829536</v>
+        <v>239762.8313877934</v>
       </c>
       <c r="S16">
-        <v>115096.9939598177</v>
+        <v>115086.1590661408</v>
       </c>
     </row>
     <row r="17" spans="1:19">
@@ -1380,58 +1380,58 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0.4498596300281296</v>
+        <v>0.5338973307135134</v>
       </c>
       <c r="C17">
-        <v>0.2269289802658426</v>
+        <v>0.4607227217342627</v>
       </c>
       <c r="D17">
-        <v>-3157593.013397145</v>
+        <v>-970518.0304279651</v>
       </c>
       <c r="E17">
         <v>0</v>
       </c>
       <c r="F17">
-        <v>-3157593.013397145</v>
+        <v>-970518.0304279651</v>
       </c>
       <c r="G17">
-        <v>-3157593.013397145</v>
+        <v>-970518.0304279651</v>
       </c>
       <c r="H17">
-        <v>-4222891.188461766</v>
+        <v>-834966.6596369415</v>
       </c>
       <c r="I17">
-        <v>-903219.8724936618</v>
+        <v>11262.01040188567</v>
       </c>
       <c r="J17">
-        <v>-3319671.315968103</v>
+        <v>-846228.670038827</v>
       </c>
       <c r="K17">
         <v>0</v>
       </c>
       <c r="L17">
-        <v>658922.9201027502</v>
+        <v>1337778.721815031</v>
       </c>
       <c r="M17">
         <v>0</v>
       </c>
       <c r="N17">
-        <v>658922.9201027503</v>
+        <v>1337778.721815031</v>
       </c>
       <c r="O17">
-        <v>316283.0016493202</v>
+        <v>642133.7864712148</v>
       </c>
       <c r="P17">
-        <v>176709.7090153343</v>
+        <v>358765.0109696848</v>
       </c>
       <c r="Q17">
         <v>0</v>
       </c>
       <c r="R17">
-        <v>176709.7090153343</v>
+        <v>358765.0109696848</v>
       </c>
       <c r="S17">
-        <v>84820.66032736047</v>
+        <v>172207.2052654487</v>
       </c>
     </row>
     <row r="18" spans="1:19">
@@ -1439,58 +1439,58 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0.5275043418514653</v>
+        <v>0.3681674312145542</v>
       </c>
       <c r="C18">
-        <v>0.3916172145025195</v>
+        <v>0.3565354152051198</v>
       </c>
       <c r="D18">
-        <v>-1462781.540131018</v>
+        <v>-3017446.028534439</v>
       </c>
       <c r="E18">
         <v>0</v>
       </c>
       <c r="F18">
-        <v>-1462781.540131018</v>
+        <v>-3017446.028534439</v>
       </c>
       <c r="G18">
-        <v>-1462781.540131018</v>
+        <v>-3017446.028534439</v>
       </c>
       <c r="H18">
-        <v>-1617034.99009451</v>
+        <v>-3870058.092415463</v>
       </c>
       <c r="I18">
-        <v>-206747.2640988243</v>
+        <v>-759928.1183724501</v>
       </c>
       <c r="J18">
-        <v>-1410287.725995686</v>
+        <v>-3110129.974043012</v>
       </c>
       <c r="K18">
         <v>0</v>
       </c>
       <c r="L18">
-        <v>1137120.337121377</v>
+        <v>1035254.979913932</v>
       </c>
       <c r="M18">
         <v>0</v>
       </c>
       <c r="N18">
-        <v>1137120.337121377</v>
+        <v>1035254.979913932</v>
       </c>
       <c r="O18">
-        <v>545817.7618182609</v>
+        <v>496922.3903586876</v>
       </c>
       <c r="P18">
-        <v>304952.518356477</v>
+        <v>277634.3039163666</v>
       </c>
       <c r="Q18">
         <v>0</v>
       </c>
       <c r="R18">
-        <v>304952.518356477</v>
+        <v>277634.3039163666</v>
       </c>
       <c r="S18">
-        <v>146377.208811109</v>
+        <v>133264.465879856</v>
       </c>
     </row>
     <row r="19" spans="1:19">
@@ -1498,58 +1498,58 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>0.3924884900515483</v>
+        <v>0.5636472996760196</v>
       </c>
       <c r="C19">
-        <v>0.5965255585436057</v>
+        <v>0.390115712399095</v>
       </c>
       <c r="D19">
-        <v>-1290193.164844848</v>
+        <v>-1170198.234201567</v>
       </c>
       <c r="E19">
         <v>0</v>
       </c>
       <c r="F19">
-        <v>-1290193.164844848</v>
+        <v>-1170198.234201567</v>
       </c>
       <c r="G19">
-        <v>-1290193.164844848</v>
+        <v>-1170198.234201567</v>
       </c>
       <c r="H19">
-        <v>-1128883.99155638</v>
+        <v>-1202618.949183644</v>
       </c>
       <c r="I19">
-        <v>3184.627319237406</v>
+        <v>-108627.832986039</v>
       </c>
       <c r="J19">
-        <v>-1132068.618875617</v>
+        <v>-1093991.116197605</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
-        <v>1732102.979932356</v>
+        <v>1132760.496657767</v>
       </c>
       <c r="M19">
         <v>0</v>
       </c>
       <c r="N19">
-        <v>1732102.979932356</v>
+        <v>1132760.496657767</v>
       </c>
       <c r="O19">
-        <v>831409.4303675313</v>
+        <v>543725.0383957283</v>
       </c>
       <c r="P19">
-        <v>464514.7470673976</v>
+        <v>303783.2979269347</v>
       </c>
       <c r="Q19">
         <v>0</v>
       </c>
       <c r="R19">
-        <v>464514.7470673976</v>
+        <v>303783.2979269347</v>
       </c>
       <c r="S19">
-        <v>222967.0785923509</v>
+        <v>145815.9830049286</v>
       </c>
     </row>
     <row r="20" spans="1:19">
@@ -1557,58 +1557,58 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>0.5063398733065707</v>
+        <v>0.3630811448260451</v>
       </c>
       <c r="C20">
-        <v>0.487593717618033</v>
+        <v>0.4159897000323737</v>
       </c>
       <c r="D20">
-        <v>-1030237.363446803</v>
+        <v>-2682423.373785645</v>
       </c>
       <c r="E20">
         <v>0</v>
       </c>
       <c r="F20">
-        <v>-1030237.363446803</v>
+        <v>-2682423.373785645</v>
       </c>
       <c r="G20">
-        <v>-1030237.363446803</v>
+        <v>-2682423.373785645</v>
       </c>
       <c r="H20">
-        <v>-888096.2865612095</v>
+        <v>-3323090.56905475</v>
       </c>
       <c r="I20">
-        <v>10862.32152348454</v>
+        <v>-602377.575668924</v>
       </c>
       <c r="J20">
-        <v>-898958.6080846939</v>
+        <v>-2720712.993385828</v>
       </c>
       <c r="K20">
         <v>0</v>
       </c>
       <c r="L20">
-        <v>1415802.758467647</v>
+        <v>1207889.56772683</v>
       </c>
       <c r="M20">
         <v>0</v>
       </c>
       <c r="N20">
-        <v>1415802.758467647</v>
+        <v>1207889.56772683</v>
       </c>
       <c r="O20">
-        <v>679585.3240644706</v>
+        <v>579786.9925088785</v>
       </c>
       <c r="P20">
-        <v>379689.4687362101</v>
+        <v>323931.3848763707</v>
       </c>
       <c r="Q20">
         <v>0</v>
       </c>
       <c r="R20">
-        <v>379689.4687362101</v>
+        <v>323931.3848763707</v>
       </c>
       <c r="S20">
-        <v>182250.9449933809</v>
+        <v>155487.0647406578</v>
       </c>
     </row>
     <row r="21" spans="1:19">
@@ -1616,58 +1616,58 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>0.4481046645540333</v>
+        <v>0.5071837494890213</v>
       </c>
       <c r="C21">
-        <v>0.4288980269312649</v>
+        <v>0.3676712185017366</v>
       </c>
       <c r="D21">
-        <v>-1889745.453828607</v>
+        <v>-1784699.501469505</v>
       </c>
       <c r="E21">
         <v>0</v>
       </c>
       <c r="F21">
-        <v>-1889745.453828607</v>
+        <v>-1784699.501469505</v>
       </c>
       <c r="G21">
-        <v>-1889745.453828607</v>
+        <v>-1784699.501469505</v>
       </c>
       <c r="H21">
-        <v>-2180235.869294892</v>
+        <v>-2103313.305998462</v>
       </c>
       <c r="I21">
-        <v>-324005.5367452815</v>
+        <v>-333617.6562357291</v>
       </c>
       <c r="J21">
-        <v>-1856230.33254961</v>
+        <v>-1769695.649762732</v>
       </c>
       <c r="K21">
         <v>0</v>
       </c>
       <c r="L21">
-        <v>1245370.864491545</v>
+        <v>1067589.48393938</v>
       </c>
       <c r="M21">
         <v>0</v>
       </c>
       <c r="N21">
-        <v>1245370.864491545</v>
+        <v>1067589.48393938</v>
       </c>
       <c r="O21">
-        <v>597778.0149559417</v>
+        <v>512442.9522909025</v>
       </c>
       <c r="P21">
-        <v>333983.1054080792</v>
+        <v>286305.7594435184</v>
       </c>
       <c r="Q21">
         <v>0</v>
       </c>
       <c r="R21">
-        <v>333983.1054080792</v>
+        <v>286305.7594435184</v>
       </c>
       <c r="S21">
-        <v>160311.890595878</v>
+        <v>137426.7645328889</v>
       </c>
     </row>
     <row r="22" spans="1:19">
@@ -1675,58 +1675,58 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0.3867294601586262</v>
+        <v>0.5740531015491221</v>
       </c>
       <c r="C22">
-        <v>0.2922639139478632</v>
+        <v>0.3843199924304567</v>
       </c>
       <c r="D22">
-        <v>-3270414.99200086</v>
+        <v>-1120019.653387767</v>
       </c>
       <c r="E22">
         <v>0</v>
       </c>
       <c r="F22">
-        <v>-3270414.99200086</v>
+        <v>-1120019.653387767</v>
       </c>
       <c r="G22">
-        <v>-3270414.99200086</v>
+        <v>-1120019.653387767</v>
       </c>
       <c r="H22">
-        <v>-4306010.258347615</v>
+        <v>-1138104.03828618</v>
       </c>
       <c r="I22">
-        <v>-893209.6330893795</v>
+        <v>-95892.14139902277</v>
       </c>
       <c r="J22">
-        <v>-3412800.625258234</v>
+        <v>-1042211.896887156</v>
       </c>
       <c r="K22">
         <v>0</v>
       </c>
       <c r="L22">
-        <v>848632.8691627758</v>
+        <v>1115931.739390365</v>
       </c>
       <c r="M22">
         <v>0</v>
       </c>
       <c r="N22">
-        <v>848632.8691627758</v>
+        <v>1115931.739390365</v>
       </c>
       <c r="O22">
-        <v>407343.7771981324</v>
+        <v>535647.2349073752</v>
       </c>
       <c r="P22">
-        <v>227586.0541430518</v>
+        <v>299270.1679247963</v>
       </c>
       <c r="Q22">
         <v>0</v>
       </c>
       <c r="R22">
-        <v>227586.0541430518</v>
+        <v>299270.1679247963</v>
       </c>
       <c r="S22">
-        <v>109241.3059886649</v>
+        <v>143649.6806039022</v>
       </c>
     </row>
     <row r="23" spans="1:19">
@@ -1734,58 +1734,58 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>0.3006271609319814</v>
+        <v>0.3096290768820745</v>
       </c>
       <c r="C23">
-        <v>0.4519011420205494</v>
+        <v>0.5930249676594933</v>
       </c>
       <c r="D23">
-        <v>-2976434.318720251</v>
+        <v>-2005041.612800343</v>
       </c>
       <c r="E23">
         <v>0</v>
       </c>
       <c r="F23">
-        <v>-2976434.318720251</v>
+        <v>-2005041.612800343</v>
       </c>
       <c r="G23">
-        <v>-2976434.318720251</v>
+        <v>-2005041.612800343</v>
       </c>
       <c r="H23">
-        <v>-3698790.001314004</v>
+        <v>-2149887.368033735</v>
       </c>
       <c r="I23">
-        <v>-675556.9857343696</v>
+        <v>-241840.7376810388</v>
       </c>
       <c r="J23">
-        <v>-3023233.015579635</v>
+        <v>-1908046.630352695</v>
       </c>
       <c r="K23">
         <v>0</v>
       </c>
       <c r="L23">
-        <v>1312163.919077761</v>
+        <v>1721938.480163564</v>
       </c>
       <c r="M23">
         <v>0</v>
       </c>
       <c r="N23">
-        <v>1312163.919077761</v>
+        <v>1721938.480163564</v>
       </c>
       <c r="O23">
-        <v>629838.6811573257</v>
+        <v>826530.4704785108</v>
       </c>
       <c r="P23">
-        <v>351895.6424895563</v>
+        <v>461788.8352169651</v>
       </c>
       <c r="Q23">
         <v>0</v>
       </c>
       <c r="R23">
-        <v>351895.6424895563</v>
+        <v>461788.8352169651</v>
       </c>
       <c r="S23">
-        <v>168909.9083949871</v>
+        <v>221658.6409041433</v>
       </c>
     </row>
     <row r="24" spans="1:19">
@@ -1793,58 +1793,58 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0.5846405528056907</v>
+        <v>0.3618943212562551</v>
       </c>
       <c r="C24">
-        <v>0.4223941057117254</v>
+        <v>0.3879163465188795</v>
       </c>
       <c r="D24">
-        <v>-789746.2277622599</v>
+        <v>-2870611.713604734</v>
       </c>
       <c r="E24">
         <v>0</v>
       </c>
       <c r="F24">
-        <v>-789746.2277622599</v>
+        <v>-2870611.713604734</v>
       </c>
       <c r="G24">
-        <v>-789746.2277622599</v>
+        <v>-2870611.713604734</v>
       </c>
       <c r="H24">
-        <v>-623210.0702454419</v>
+        <v>-3624028.604417659</v>
       </c>
       <c r="I24">
-        <v>44250.7143810495</v>
+        <v>-686943.4777100682</v>
       </c>
       <c r="J24">
-        <v>-667460.7846264911</v>
+        <v>-2937085.12670759</v>
       </c>
       <c r="K24">
         <v>0</v>
       </c>
       <c r="L24">
-        <v>1226485.736831443</v>
+        <v>1126374.302234876</v>
       </c>
       <c r="M24">
         <v>0</v>
       </c>
       <c r="N24">
-        <v>1226485.736831443</v>
+        <v>1126374.302234876</v>
       </c>
       <c r="O24">
-        <v>588713.1536790928</v>
+        <v>540659.6650727405</v>
       </c>
       <c r="P24">
-        <v>328918.498742077</v>
+        <v>302070.6506297236</v>
       </c>
       <c r="Q24">
         <v>0</v>
       </c>
       <c r="R24">
-        <v>328918.498742077</v>
+        <v>302070.6506297236</v>
       </c>
       <c r="S24">
-        <v>157880.8793961969</v>
+        <v>144993.9123022673</v>
       </c>
     </row>
     <row r="25" spans="1:19">
@@ -1852,58 +1852,58 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>0.4381145246356116</v>
+        <v>0.5358209046451742</v>
       </c>
       <c r="C25">
-        <v>0.282684498660275</v>
+        <v>0.6231394140128803</v>
       </c>
       <c r="D25">
-        <v>-2901718.655498887</v>
+        <v>76918.17781098298</v>
       </c>
       <c r="E25">
         <v>0</v>
       </c>
       <c r="F25">
-        <v>-2901718.655498887</v>
+        <v>76918.17781098298</v>
       </c>
       <c r="G25">
-        <v>-2901718.655498887</v>
+        <v>76918.17781098298</v>
       </c>
       <c r="H25">
-        <v>-3792890.570972144</v>
+        <v>847320.8666073449</v>
       </c>
       <c r="I25">
-        <v>-775245.1382450842</v>
+        <v>486500.6983519153</v>
       </c>
       <c r="J25">
-        <v>-3017645.432727059</v>
+        <v>360820.1682554288</v>
       </c>
       <c r="K25">
         <v>0</v>
       </c>
       <c r="L25">
-        <v>820817.5752026126</v>
+        <v>1809380.370155779</v>
       </c>
       <c r="M25">
         <v>0</v>
       </c>
       <c r="N25">
-        <v>820817.5752026126</v>
+        <v>1809380.370155779</v>
       </c>
       <c r="O25">
-        <v>393992.4360972541</v>
+        <v>868502.577674774</v>
       </c>
       <c r="P25">
-        <v>220126.5587272451</v>
+        <v>485238.9694661511</v>
       </c>
       <c r="Q25">
         <v>0</v>
       </c>
       <c r="R25">
-        <v>220126.5587272451</v>
+        <v>485238.9694661512</v>
       </c>
       <c r="S25">
-        <v>105660.7481890776</v>
+        <v>232914.7053437526</v>
       </c>
     </row>
     <row r="26" spans="1:19">
@@ -1911,58 +1911,58 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0.4948403608465582</v>
+        <v>0.5618065346466206</v>
       </c>
       <c r="C26">
-        <v>0.2986978017126054</v>
+        <v>0.4982304602067967</v>
       </c>
       <c r="D26">
-        <v>-2325863.448790676</v>
+        <v>-499049.0901640135</v>
       </c>
       <c r="E26">
         <v>0</v>
       </c>
       <c r="F26">
-        <v>-2325863.448790676</v>
+        <v>-499049.0901640135</v>
       </c>
       <c r="G26">
-        <v>-2325863.448790676</v>
+        <v>-499049.0901640135</v>
       </c>
       <c r="H26">
-        <v>-2954785.143058513</v>
+        <v>-119895.4953730031</v>
       </c>
       <c r="I26">
-        <v>-568113.7848145892</v>
+        <v>198872.4688767064</v>
       </c>
       <c r="J26">
-        <v>-2386671.358243924</v>
+        <v>-318767.9642497092</v>
       </c>
       <c r="K26">
         <v>0</v>
       </c>
       <c r="L26">
-        <v>867314.644000837</v>
+        <v>1446688.163578792</v>
       </c>
       <c r="M26">
         <v>0</v>
       </c>
       <c r="N26">
-        <v>867314.6440008369</v>
+        <v>1446688.163578792</v>
       </c>
       <c r="O26">
-        <v>416311.0291204018</v>
+        <v>694410.3185178199</v>
       </c>
       <c r="P26">
-        <v>232596.1257232134</v>
+        <v>387972.3054436661</v>
       </c>
       <c r="Q26">
         <v>0</v>
       </c>
       <c r="R26">
-        <v>232596.1257232134</v>
+        <v>387972.3054436661</v>
       </c>
       <c r="S26">
-        <v>111646.1403471424</v>
+        <v>186226.7066129597</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(plotting,engine): overhaul plotting suite and fix MC simulation
This commit provides a comprehensive update to the plotting suite and the Monte Carlo engine.

Plotting:

- Overhauls the enhanced Sankey to fix layout, zoom, and positioning bugs.

- Adds 'Custom' and 'Auto-Layout' modes to the enhanced Sankey.

- Stabilizes the traditional Sankey layout to prevent it from collapsing.

- Integrates a Graphviz flow chart into the notebook.

- Fixes a bug in the Monte Carlo histogram where the mean indicator was not cleared.

- Fixes the y-axis range on the process dynamics plot.

Monte Carlo Engine:

- Corrects the TC normalization logic to ensure mass balance is respected.

General:

- Restructures the main notebook for a more logical workflow.

- Fixes various module import errors.
</commit_message>
<xml_diff>
--- a/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
+++ b/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
@@ -495,58 +495,58 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>0.5449950755588977</v>
+        <v>0.3960433521366136</v>
       </c>
       <c r="C2">
-        <v>0.3719355993735756</v>
+        <v>0.3892089166004167</v>
       </c>
       <c r="D2">
-        <v>-1441556.601855356</v>
+        <v>-2576953.036216497</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>-1441556.601855356</v>
+        <v>-2576953.036216497</v>
       </c>
       <c r="G2">
-        <v>-1441556.601855356</v>
+        <v>-2576953.036216497</v>
       </c>
       <c r="H2">
-        <v>-1610149.407278767</v>
+        <v>-3204774.197456812</v>
       </c>
       <c r="I2">
-        <v>-214090.8836572845</v>
+        <v>-586394.9032031018</v>
       </c>
       <c r="J2">
-        <v>-1396058.523621483</v>
+        <v>-2618379.29425371</v>
       </c>
       <c r="K2">
         <v>0</v>
       </c>
       <c r="L2">
-        <v>1079971.764480238</v>
+        <v>1130127.476693097</v>
       </c>
       <c r="M2">
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1079971.764480238</v>
+        <v>1130127.476693098</v>
       </c>
       <c r="O2">
-        <v>518386.4469505142</v>
+        <v>542461.1888126868</v>
       </c>
       <c r="P2">
-        <v>289626.4349346366</v>
+        <v>303077.175590629</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
       <c r="R2">
-        <v>289626.4349346366</v>
+        <v>303077.175590629</v>
       </c>
       <c r="S2">
-        <v>139020.6887686256</v>
+        <v>145477.0442835019</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -554,58 +554,58 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>0.370229545831497</v>
+        <v>0.4953343596326366</v>
       </c>
       <c r="C3">
-        <v>0.4908156915791926</v>
+        <v>0.4481760908787957</v>
       </c>
       <c r="D3">
-        <v>-2147519.928847208</v>
+        <v>-1372536.763204096</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3">
-        <v>-2147519.928847208</v>
+        <v>-1372536.763204096</v>
       </c>
       <c r="G3">
-        <v>-2147519.928847208</v>
+        <v>-1372536.763204096</v>
       </c>
       <c r="H3">
-        <v>-2473593.70141829</v>
+        <v>-1421687.92506163</v>
       </c>
       <c r="I3">
-        <v>-365680.4337216622</v>
+        <v>-134351.7819391069</v>
       </c>
       <c r="J3">
-        <v>-2107913.267696628</v>
+        <v>-1287336.143122522</v>
       </c>
       <c r="K3">
         <v>0</v>
       </c>
       <c r="L3">
-        <v>1425158.251487953</v>
+        <v>1301347.664701696</v>
       </c>
       <c r="M3">
         <v>0</v>
       </c>
       <c r="N3">
-        <v>1425158.251487953</v>
+        <v>1301347.664701696</v>
       </c>
       <c r="O3">
-        <v>684075.9607142177</v>
+        <v>624646.8790568142</v>
       </c>
       <c r="P3">
-        <v>382198.4214511279</v>
+        <v>348994.9433256356</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
       <c r="R3">
-        <v>382198.4214511279</v>
+        <v>348994.9433256356</v>
       </c>
       <c r="S3">
-        <v>183455.2422965414</v>
+        <v>167517.5727963051</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -613,58 +613,58 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.4611195759782936</v>
+        <v>0.5984464829628622</v>
       </c>
       <c r="C4">
-        <v>0.2201772492623726</v>
+        <v>0.3316639504335053</v>
       </c>
       <c r="D4">
-        <v>-3106345.40224422</v>
+        <v>-1250485.547876938</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>-3106345.40224422</v>
+        <v>-1250485.547876938</v>
       </c>
       <c r="G4">
-        <v>-3106345.40224422</v>
+        <v>-1250485.547876938</v>
       </c>
       <c r="H4">
-        <v>-4157987.687183581</v>
+        <v>-1386043.223887909</v>
       </c>
       <c r="I4">
-        <v>-890827.9825031236</v>
+        <v>-179044.8499575838</v>
       </c>
       <c r="J4">
-        <v>-3267159.704680458</v>
+        <v>-1206998.373930324</v>
       </c>
       <c r="K4">
         <v>0</v>
       </c>
       <c r="L4">
-        <v>639318.2389230131</v>
+        <v>963036.8869434083</v>
       </c>
       <c r="M4">
         <v>0</v>
       </c>
       <c r="N4">
-        <v>639318.2389230131</v>
+        <v>963036.8869434083</v>
       </c>
       <c r="O4">
-        <v>306872.7546830464</v>
+        <v>462257.7057328359</v>
       </c>
       <c r="P4">
-        <v>171452.1327481898</v>
+        <v>258266.8820144639</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
       <c r="R4">
-        <v>171452.1327481898</v>
+        <v>258266.8820144639</v>
       </c>
       <c r="S4">
-        <v>82297.02371913113</v>
+        <v>123968.1033669427</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -672,58 +672,58 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>0.3086702192017908</v>
+        <v>0.4520301027710972</v>
       </c>
       <c r="C5">
-        <v>0.2643096557108147</v>
+        <v>0.3713084606476049</v>
       </c>
       <c r="D5">
-        <v>-4100421.399090122</v>
+        <v>-2222630.514781113</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>-4100421.399090122</v>
+        <v>-2222630.514781113</v>
       </c>
       <c r="G5">
-        <v>-4100421.399090122</v>
+        <v>-2222630.514781113</v>
       </c>
       <c r="H5">
-        <v>-5519781.026394817</v>
+        <v>-2721954.553451012</v>
       </c>
       <c r="I5">
-        <v>-1195358.39575637</v>
+        <v>-479453.3504282762</v>
       </c>
       <c r="J5">
-        <v>-4324422.630638447</v>
+        <v>-2242501.203022736</v>
       </c>
       <c r="K5">
         <v>0</v>
       </c>
       <c r="L5">
-        <v>767463.4149781049</v>
+        <v>1078150.771497579</v>
       </c>
       <c r="M5">
         <v>0</v>
       </c>
       <c r="N5">
-        <v>767463.4149781051</v>
+        <v>1078150.771497579</v>
       </c>
       <c r="O5">
-        <v>368382.4391894905</v>
+        <v>517512.3703188378</v>
       </c>
       <c r="P5">
-        <v>205818.0594469955</v>
+        <v>289138.0816989736</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
       <c r="R5">
-        <v>205818.0594469955</v>
+        <v>289138.0816989736</v>
       </c>
       <c r="S5">
-        <v>98792.66853455783</v>
+        <v>138786.2792155074</v>
       </c>
     </row>
     <row r="6" spans="1:19">
@@ -731,58 +731,58 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>0.5721981838119</v>
+        <v>0.3523289163944616</v>
       </c>
       <c r="C6">
-        <v>0.4396331302353784</v>
+        <v>0.3405531674562756</v>
       </c>
       <c r="D6">
-        <v>-784282.6477749911</v>
+        <v>-3251328.08604714</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
       <c r="F6">
-        <v>-784282.6477749911</v>
+        <v>-3251328.08604714</v>
       </c>
       <c r="G6">
-        <v>-784282.6477749911</v>
+        <v>-3251328.08604714</v>
       </c>
       <c r="H6">
-        <v>-595024.2082717542</v>
+        <v>-4221676.568064854</v>
       </c>
       <c r="I6">
-        <v>58840.93481610212</v>
+        <v>-851057.2607848514</v>
       </c>
       <c r="J6">
-        <v>-653865.1430878559</v>
+        <v>-3370619.307280004</v>
       </c>
       <c r="K6">
         <v>0</v>
       </c>
       <c r="L6">
-        <v>1276541.874948053</v>
+        <v>988848.0849279459</v>
       </c>
       <c r="M6">
         <v>0</v>
       </c>
       <c r="N6">
-        <v>1276541.874948053</v>
+        <v>988848.0849279461</v>
       </c>
       <c r="O6">
-        <v>612740.0999750653</v>
+        <v>474647.080765414</v>
       </c>
       <c r="P6">
-        <v>342342.5356531593</v>
+        <v>265188.9197005617</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
       <c r="R6">
-        <v>342342.5356531593</v>
+        <v>265188.9197005617</v>
       </c>
       <c r="S6">
-        <v>164324.4171135165</v>
+        <v>127290.6814562696</v>
       </c>
     </row>
     <row r="7" spans="1:19">
@@ -790,58 +790,58 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>0.4957517413628772</v>
+        <v>0.3681817590423575</v>
       </c>
       <c r="C7">
-        <v>0.3761177585437477</v>
+        <v>0.5256855429273644</v>
       </c>
       <c r="D7">
-        <v>-1826623.222054502</v>
+        <v>-1943211.377888573</v>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
       <c r="F7">
-        <v>-1826623.222054502</v>
+        <v>-1943211.377888573</v>
       </c>
       <c r="G7">
-        <v>-1826623.222054502</v>
+        <v>-1943211.377888573</v>
       </c>
       <c r="H7">
-        <v>-2152946.802805963</v>
+        <v>-2141676.733929151</v>
       </c>
       <c r="I7">
-        <v>-341595.1438554887</v>
+        <v>-270625.7310619875</v>
       </c>
       <c r="J7">
-        <v>-1811351.658950475</v>
+        <v>-1871051.002867163</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
       <c r="L7">
-        <v>1092115.301764528</v>
+        <v>1526408.185484791</v>
       </c>
       <c r="M7">
         <v>0</v>
       </c>
       <c r="N7">
-        <v>1092115.301764528</v>
+        <v>1526408.185484791</v>
       </c>
       <c r="O7">
-        <v>524215.3448469737</v>
+        <v>732675.9290326998</v>
       </c>
       <c r="P7">
-        <v>292883.0843460567</v>
+        <v>409351.5919184914</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
       <c r="R7">
-        <v>292883.0843460567</v>
+        <v>409351.5919184914</v>
       </c>
       <c r="S7">
-        <v>140583.8804861072</v>
+        <v>196488.7641208759</v>
       </c>
     </row>
     <row r="8" spans="1:19">
@@ -849,58 +849,58 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0.4904159211441496</v>
+        <v>0.4179183159149376</v>
       </c>
       <c r="C8">
-        <v>0.3969657032279209</v>
+        <v>0.5203040848975512</v>
       </c>
       <c r="D8">
-        <v>-1738839.314888539</v>
+        <v>-1561637.55331131</v>
       </c>
       <c r="E8">
         <v>0</v>
       </c>
       <c r="F8">
-        <v>-1738839.314888539</v>
+        <v>-1561637.55331131</v>
       </c>
       <c r="G8">
-        <v>-1738839.314888539</v>
+        <v>-1561637.55331131</v>
       </c>
       <c r="H8">
-        <v>-2003388.277020375</v>
+        <v>-1605267.952452058</v>
       </c>
       <c r="I8">
-        <v>-296419.7134953453</v>
+        <v>-145192.1595107507</v>
       </c>
       <c r="J8">
-        <v>-1706968.563525029</v>
+        <v>-1460075.792941306</v>
       </c>
       <c r="K8">
         <v>0</v>
       </c>
       <c r="L8">
-        <v>1152650.490233375</v>
+        <v>1510782.30096682</v>
       </c>
       <c r="M8">
         <v>0</v>
       </c>
       <c r="N8">
-        <v>1152650.490233375</v>
+        <v>1510782.30096682</v>
       </c>
       <c r="O8">
-        <v>553272.2353120201</v>
+        <v>725175.5044640737</v>
       </c>
       <c r="P8">
-        <v>309117.3891686152</v>
+        <v>405161.0478927241</v>
       </c>
       <c r="Q8">
         <v>0</v>
       </c>
       <c r="R8">
-        <v>309117.3891686152</v>
+        <v>405161.0478927241</v>
       </c>
       <c r="S8">
-        <v>148376.3468009353</v>
+        <v>194477.3029885076</v>
       </c>
     </row>
     <row r="9" spans="1:19">
@@ -908,58 +908,58 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0.4971381624946343</v>
+        <v>0.4974801446411339</v>
       </c>
       <c r="C9">
-        <v>0.5064232975367189</v>
+        <v>0.484522026734526</v>
       </c>
       <c r="D9">
-        <v>-987585.0791473668</v>
+        <v>-1123801.028338873</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
       <c r="F9">
-        <v>-987585.0791473668</v>
+        <v>-1123801.028338873</v>
       </c>
       <c r="G9">
-        <v>-987585.0791473668</v>
+        <v>-1123801.028338873</v>
       </c>
       <c r="H9">
-        <v>-805126.7171606534</v>
+        <v>-1024826.206789318</v>
       </c>
       <c r="I9">
-        <v>39240.19121779221</v>
+        <v>-23139.09751300172</v>
       </c>
       <c r="J9">
-        <v>-844366.9083784455</v>
+        <v>-1001687.109276317</v>
       </c>
       <c r="K9">
         <v>0</v>
       </c>
       <c r="L9">
-        <v>1470477.316868226</v>
+        <v>1406883.63529421</v>
       </c>
       <c r="M9">
         <v>0</v>
       </c>
       <c r="N9">
-        <v>1470477.316868226</v>
+        <v>1406883.63529421</v>
       </c>
       <c r="O9">
-        <v>705829.1120967483</v>
+        <v>675304.1449412209</v>
       </c>
       <c r="P9">
-        <v>394352.0719189945</v>
+        <v>377297.5415280868</v>
       </c>
       <c r="Q9">
         <v>0</v>
       </c>
       <c r="R9">
-        <v>394352.0719189945</v>
+        <v>377297.5415280868</v>
       </c>
       <c r="S9">
-        <v>189288.9945211174</v>
+        <v>181102.8199334816</v>
       </c>
     </row>
     <row r="10" spans="1:19">
@@ -967,58 +967,58 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0.4265534763320973</v>
+        <v>0.3467129848896737</v>
       </c>
       <c r="C10">
-        <v>0.3104245187251964</v>
+        <v>0.3343490320185892</v>
       </c>
       <c r="D10">
-        <v>-2822206.100965149</v>
+        <v>-3337668.180831301</v>
       </c>
       <c r="E10">
         <v>0</v>
       </c>
       <c r="F10">
-        <v>-2822206.100965149</v>
+        <v>-3337668.180831301</v>
       </c>
       <c r="G10">
-        <v>-2822206.100965149</v>
+        <v>-3337668.180831301</v>
       </c>
       <c r="H10">
-        <v>-3646936.459261142</v>
+        <v>-4351840.46296475</v>
       </c>
       <c r="I10">
-        <v>-727782.6212928595</v>
+        <v>-884923.2702307812</v>
       </c>
       <c r="J10">
-        <v>-2919153.837968282</v>
+        <v>-3466917.192733969</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>901364.9561650353</v>
+        <v>970833.4310281919</v>
       </c>
       <c r="M10">
         <v>0</v>
       </c>
       <c r="N10">
-        <v>901364.9561650353</v>
+        <v>970833.4310281919</v>
       </c>
       <c r="O10">
-        <v>432655.178959217</v>
+        <v>466000.0468935322</v>
       </c>
       <c r="P10">
-        <v>241727.726052852</v>
+        <v>260357.7563709554</v>
       </c>
       <c r="Q10">
         <v>0</v>
       </c>
       <c r="R10">
-        <v>241727.726052852</v>
+        <v>260357.7563709554</v>
       </c>
       <c r="S10">
-        <v>116029.308505369</v>
+        <v>124971.7230580586</v>
       </c>
     </row>
     <row r="11" spans="1:19">
@@ -1026,58 +1026,58 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0.4267266824599592</v>
+        <v>0.4276591538736274</v>
       </c>
       <c r="C11">
-        <v>0.4253246229456785</v>
+        <v>0.2700794309404495</v>
       </c>
       <c r="D11">
-        <v>-2091134.752338687</v>
+        <v>-3069157.842085347</v>
       </c>
       <c r="E11">
         <v>0</v>
       </c>
       <c r="F11">
-        <v>-2091134.752338687</v>
+        <v>-3069157.842085347</v>
       </c>
       <c r="G11">
-        <v>-2091134.752338687</v>
+        <v>-3069157.842085347</v>
       </c>
       <c r="H11">
-        <v>-2470939.779913904</v>
+        <v>-4045996.177542837</v>
       </c>
       <c r="I11">
-        <v>-394946.4235868489</v>
+        <v>-841345.0909323925</v>
       </c>
       <c r="J11">
-        <v>-2075993.356327054</v>
+        <v>-3204651.086610445</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>1234994.940772454</v>
+        <v>784216.8377370393</v>
       </c>
       <c r="M11">
         <v>0</v>
       </c>
       <c r="N11">
-        <v>1234994.940772455</v>
+        <v>784216.8377370393</v>
       </c>
       <c r="O11">
-        <v>592797.5715707781</v>
+        <v>376424.0821137789</v>
       </c>
       <c r="P11">
-        <v>331200.4939595659</v>
+        <v>210310.9862680575</v>
       </c>
       <c r="Q11">
         <v>0</v>
       </c>
       <c r="R11">
-        <v>331200.4939595659</v>
+        <v>210310.9862680575</v>
       </c>
       <c r="S11">
-        <v>158976.2371005916</v>
+        <v>100949.2734086676</v>
       </c>
     </row>
     <row r="12" spans="1:19">
@@ -1085,58 +1085,58 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>0.3632398569505588</v>
+        <v>0.3070714433698677</v>
       </c>
       <c r="C12">
-        <v>0.4310048189301092</v>
+        <v>0.290192657341922</v>
       </c>
       <c r="D12">
-        <v>-2585749.671316861</v>
+        <v>-3949426.68903621</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
       <c r="F12">
-        <v>-2585749.671316861</v>
+        <v>-3949426.68903621</v>
       </c>
       <c r="G12">
-        <v>-2585749.671316861</v>
+        <v>-3949426.68903621</v>
       </c>
       <c r="H12">
-        <v>-3167793.569380045</v>
+        <v>-5274343.968946022</v>
       </c>
       <c r="I12">
-        <v>-558496.849352608</v>
+        <v>-1125024.980329387</v>
       </c>
       <c r="J12">
-        <v>-2609296.720027437</v>
+        <v>-4149318.988616633</v>
       </c>
       <c r="K12">
         <v>0</v>
       </c>
       <c r="L12">
-        <v>1251488.256524512</v>
+        <v>842618.6595652619</v>
       </c>
       <c r="M12">
         <v>0</v>
       </c>
       <c r="N12">
-        <v>1251488.256524512</v>
+        <v>842618.6595652619</v>
       </c>
       <c r="O12">
-        <v>600714.363131766</v>
+        <v>404456.9565913258</v>
       </c>
       <c r="P12">
-        <v>335623.6653781434</v>
+        <v>225973.1656009927</v>
       </c>
       <c r="Q12">
         <v>0</v>
       </c>
       <c r="R12">
-        <v>335623.6653781434</v>
+        <v>225973.1656009927</v>
       </c>
       <c r="S12">
-        <v>161099.3593815088</v>
+        <v>108467.1194884765</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -1144,58 +1144,58 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>0.5539391967412919</v>
+        <v>0.491958970463221</v>
       </c>
       <c r="C13">
-        <v>0.3337209494577609</v>
+        <v>0.3655469159831034</v>
       </c>
       <c r="D13">
-        <v>-1609458.591334967</v>
+        <v>-1925452.458684279</v>
       </c>
       <c r="E13">
         <v>0</v>
       </c>
       <c r="F13">
-        <v>-1609458.591334967</v>
+        <v>-1925452.458684279</v>
       </c>
       <c r="G13">
-        <v>-1609458.591334967</v>
+        <v>-1925452.458684279</v>
       </c>
       <c r="H13">
-        <v>-1894239.574132644</v>
+        <v>-2306047.206227333</v>
       </c>
       <c r="I13">
-        <v>-299269.7447412377</v>
+        <v>-382923.206320744</v>
       </c>
       <c r="J13">
-        <v>-1594969.829391406</v>
+        <v>-1923123.999906589</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13">
-        <v>969009.6974770087</v>
+        <v>1061421.247440368</v>
       </c>
       <c r="M13">
         <v>0</v>
       </c>
       <c r="N13">
-        <v>969009.6974770086</v>
+        <v>1061421.247440368</v>
       </c>
       <c r="O13">
-        <v>465124.6547889639</v>
+        <v>509482.1987713766</v>
       </c>
       <c r="P13">
-        <v>259868.6681706226</v>
+        <v>284651.5640230461</v>
       </c>
       <c r="Q13">
         <v>0</v>
       </c>
       <c r="R13">
-        <v>259868.6681706226</v>
+        <v>284651.5640230461</v>
       </c>
       <c r="S13">
-        <v>124736.9607218989</v>
+        <v>136632.7507310621</v>
       </c>
     </row>
     <row r="14" spans="1:19">
@@ -1203,58 +1203,58 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>0.4244725876820558</v>
+        <v>0.407037062532454</v>
       </c>
       <c r="C14">
-        <v>0.6124402631619259</v>
+        <v>0.5630012211207192</v>
       </c>
       <c r="D14">
-        <v>-921779.5475562927</v>
+        <v>-1381463.901534106</v>
       </c>
       <c r="E14">
         <v>0</v>
       </c>
       <c r="F14">
-        <v>-921779.5475562927</v>
+        <v>-1381463.901534106</v>
       </c>
       <c r="G14">
-        <v>-921779.5475562927</v>
+        <v>-1381463.901534106</v>
       </c>
       <c r="H14">
-        <v>-585976.9622267492</v>
+        <v>-1298413.53468013</v>
       </c>
       <c r="I14">
-        <v>139889.8780493011</v>
+        <v>-52539.45815295089</v>
       </c>
       <c r="J14">
-        <v>-725866.8402760499</v>
+        <v>-1245874.076527179</v>
       </c>
       <c r="K14">
         <v>0</v>
       </c>
       <c r="L14">
-        <v>1778313.753132815</v>
+        <v>1634759.950922486</v>
       </c>
       <c r="M14">
         <v>0</v>
       </c>
       <c r="N14">
-        <v>1778313.753132815</v>
+        <v>1634759.950922485</v>
       </c>
       <c r="O14">
-        <v>853590.6015037514</v>
+        <v>784684.776442793</v>
       </c>
       <c r="P14">
-        <v>476907.5354141033</v>
+        <v>438409.3289582155</v>
       </c>
       <c r="Q14">
         <v>0</v>
       </c>
       <c r="R14">
-        <v>476907.5354141033</v>
+        <v>438409.3289582155</v>
       </c>
       <c r="S14">
-        <v>228915.6169987697</v>
+        <v>210436.4778999434</v>
       </c>
     </row>
     <row r="15" spans="1:19">
@@ -1262,58 +1262,58 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0.5980077232571478</v>
+        <v>0.3398072808900268</v>
       </c>
       <c r="C15">
-        <v>0.3211065872265928</v>
+        <v>0.3023317000812984</v>
       </c>
       <c r="D15">
-        <v>-1321193.106390207</v>
+        <v>-3598705.010859956</v>
       </c>
       <c r="E15">
         <v>0</v>
       </c>
       <c r="F15">
-        <v>-1321193.106390207</v>
+        <v>-3598705.010859956</v>
       </c>
       <c r="G15">
-        <v>-1321193.106390207</v>
+        <v>-3598705.010859956</v>
       </c>
       <c r="H15">
-        <v>-1499125.123265897</v>
+        <v>-4761074.425299866</v>
       </c>
       <c r="I15">
-        <v>-210825.5622283591</v>
+        <v>-997109.5962524704</v>
       </c>
       <c r="J15">
-        <v>-1288299.561037538</v>
+        <v>-3763964.829047395</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
-        <v>932381.9719795515</v>
+        <v>877866.2223917973</v>
       </c>
       <c r="M15">
         <v>0</v>
       </c>
       <c r="N15">
-        <v>932381.9719795515</v>
+        <v>877866.2223917973</v>
       </c>
       <c r="O15">
-        <v>447543.3465501848</v>
+        <v>421375.7867480629</v>
       </c>
       <c r="P15">
-        <v>250045.8580708618</v>
+        <v>235425.8441777306</v>
       </c>
       <c r="Q15">
         <v>0</v>
       </c>
       <c r="R15">
-        <v>250045.8580708618</v>
+        <v>235425.8441777306</v>
       </c>
       <c r="S15">
-        <v>120022.0118740137</v>
+        <v>113004.4052053107</v>
       </c>
     </row>
     <row r="16" spans="1:19">
@@ -1321,58 +1321,58 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>0.3027877469224385</v>
+        <v>0.4683024327291097</v>
       </c>
       <c r="C16">
-        <v>0.3915252888936076</v>
+        <v>0.531768375522468</v>
       </c>
       <c r="D16">
-        <v>-3341764.840877483</v>
+        <v>-1067679.137180448</v>
       </c>
       <c r="E16">
         <v>0</v>
       </c>
       <c r="F16">
-        <v>-3341764.840877483</v>
+        <v>-1067679.137180448</v>
       </c>
       <c r="G16">
-        <v>-3341764.840877483</v>
+        <v>-1067679.137180448</v>
       </c>
       <c r="H16">
-        <v>-4289961.177027685</v>
+        <v>-889045.9496918081</v>
       </c>
       <c r="I16">
-        <v>-844067.2713161093</v>
+        <v>30803.02672342329</v>
       </c>
       <c r="J16">
-        <v>-3445893.905711575</v>
+        <v>-919848.9764152311</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
       <c r="L16">
-        <v>1136853.417089456</v>
+        <v>1544070.618072142</v>
       </c>
       <c r="M16">
         <v>0</v>
       </c>
       <c r="N16">
-        <v>1136853.417089456</v>
+        <v>1544070.618072142</v>
       </c>
       <c r="O16">
-        <v>545689.6402029388</v>
+        <v>741153.8966746284</v>
       </c>
       <c r="P16">
-        <v>304880.9358394145</v>
+        <v>414088.296664666</v>
       </c>
       <c r="Q16">
         <v>0</v>
       </c>
       <c r="R16">
-        <v>304880.9358394145</v>
+        <v>414088.296664666</v>
       </c>
       <c r="S16">
-        <v>146342.8492029189</v>
+        <v>198762.3823990397</v>
       </c>
     </row>
     <row r="17" spans="1:19">
@@ -1380,58 +1380,58 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0.3776922143551654</v>
+        <v>0.352969618493466</v>
       </c>
       <c r="C17">
-        <v>0.1561051479870161</v>
+        <v>0.4326959043739886</v>
       </c>
       <c r="D17">
-        <v>-4210574.550472276</v>
+        <v>-2660859.791509783</v>
       </c>
       <c r="E17">
         <v>0</v>
       </c>
       <c r="F17">
-        <v>-4210574.550472276</v>
+        <v>-2660859.791509783</v>
       </c>
       <c r="G17">
-        <v>-4210574.550472276</v>
+        <v>-2660859.791509783</v>
       </c>
       <c r="H17">
-        <v>-5804604.844135172</v>
+        <v>-3272633.718287089</v>
       </c>
       <c r="I17">
-        <v>-1312664.749460524</v>
+        <v>-582720.763799594</v>
       </c>
       <c r="J17">
-        <v>-4491940.094674647</v>
+        <v>-2689912.954487495</v>
       </c>
       <c r="K17">
         <v>0</v>
       </c>
       <c r="L17">
-        <v>453275.1164446992</v>
+        <v>1256398.58114466</v>
       </c>
       <c r="M17">
         <v>0</v>
       </c>
       <c r="N17">
-        <v>453275.1164446992</v>
+        <v>1256398.581144659</v>
       </c>
       <c r="O17">
-        <v>217572.0558934556</v>
+        <v>603071.3189494367</v>
       </c>
       <c r="P17">
-        <v>121559.1558392662</v>
+        <v>336940.514448535</v>
       </c>
       <c r="Q17">
         <v>0</v>
       </c>
       <c r="R17">
-        <v>121559.1558392662</v>
+        <v>336940.514448535</v>
       </c>
       <c r="S17">
-        <v>58348.39480284776</v>
+        <v>161731.4469352968</v>
       </c>
     </row>
     <row r="18" spans="1:19">
@@ -1439,58 +1439,58 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0.3686043768904699</v>
+        <v>0.3848249279142985</v>
       </c>
       <c r="C18">
-        <v>0.5330402156818004</v>
+        <v>0.3645135666526405</v>
       </c>
       <c r="D18">
-        <v>-1892976.05220962</v>
+        <v>-2827544.684172722</v>
       </c>
       <c r="E18">
         <v>0</v>
       </c>
       <c r="F18">
-        <v>-1892976.05220962</v>
+        <v>-2827544.684172722</v>
       </c>
       <c r="G18">
-        <v>-1892976.05220962</v>
+        <v>-2827544.684172722</v>
       </c>
       <c r="H18">
-        <v>-2061508.735618612</v>
+        <v>-3590479.581227965</v>
       </c>
       <c r="I18">
-        <v>-248154.4676347551</v>
+        <v>-689628.8389785311</v>
       </c>
       <c r="J18">
-        <v>-1813354.267983857</v>
+        <v>-2900850.742249433</v>
       </c>
       <c r="K18">
         <v>0</v>
       </c>
       <c r="L18">
-        <v>1547763.600038172</v>
+        <v>1058420.759986023</v>
       </c>
       <c r="M18">
         <v>0</v>
       </c>
       <c r="N18">
-        <v>1547763.600038172</v>
+        <v>1058420.759986023</v>
       </c>
       <c r="O18">
-        <v>742926.5280183227</v>
+        <v>508041.9647932911</v>
       </c>
       <c r="P18">
-        <v>415078.6792249116</v>
+        <v>283846.8943890338</v>
       </c>
       <c r="Q18">
         <v>0</v>
       </c>
       <c r="R18">
-        <v>415078.6792249116</v>
+        <v>283846.8943890337</v>
       </c>
       <c r="S18">
-        <v>199237.7660279576</v>
+        <v>136246.5093067363</v>
       </c>
     </row>
     <row r="19" spans="1:19">
@@ -1498,58 +1498,58 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>0.4975333812459932</v>
+        <v>0.3051651044829288</v>
       </c>
       <c r="C19">
-        <v>0.4143865387966191</v>
+        <v>0.4096254725664755</v>
       </c>
       <c r="D19">
-        <v>-1568721.172352021</v>
+        <v>-3206955.172481899</v>
       </c>
       <c r="E19">
         <v>0</v>
       </c>
       <c r="F19">
-        <v>-1568721.172352021</v>
+        <v>-3206955.172481899</v>
       </c>
       <c r="G19">
-        <v>-1568721.172352021</v>
+        <v>-3206955.172481899</v>
       </c>
       <c r="H19">
-        <v>-1740769.19466952</v>
+        <v>-4076763.247691954</v>
       </c>
       <c r="I19">
-        <v>-225853.0117527757</v>
+        <v>-784973.3981741692</v>
       </c>
       <c r="J19">
-        <v>-1514916.182916744</v>
+        <v>-3291789.849517783</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
-        <v>1203234.544460866</v>
+        <v>1189410.062195561</v>
       </c>
       <c r="M19">
         <v>0</v>
       </c>
       <c r="N19">
-        <v>1203234.544460866</v>
+        <v>1189410.062195561</v>
       </c>
       <c r="O19">
-        <v>577552.5813412154</v>
+        <v>570916.8298538695</v>
       </c>
       <c r="P19">
-        <v>322683.0024302723</v>
+        <v>318975.5578053248</v>
       </c>
       <c r="Q19">
         <v>0</v>
       </c>
       <c r="R19">
-        <v>322683.0024302723</v>
+        <v>318975.5578053248</v>
       </c>
       <c r="S19">
-        <v>154887.8411665306</v>
+        <v>153108.2677465559</v>
       </c>
     </row>
     <row r="20" spans="1:19">
@@ -1557,58 +1557,58 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>0.4174200993992755</v>
+        <v>0.533319049537044</v>
       </c>
       <c r="C20">
-        <v>0.3635115590863472</v>
+        <v>0.243044035624014</v>
       </c>
       <c r="D20">
-        <v>-2561445.397934068</v>
+        <v>-2357626.417146617</v>
       </c>
       <c r="E20">
         <v>0</v>
       </c>
       <c r="F20">
-        <v>-2561445.397934068</v>
+        <v>-2357626.417146617</v>
       </c>
       <c r="G20">
-        <v>-2561445.397934068</v>
+        <v>-2357626.417146617</v>
       </c>
       <c r="H20">
-        <v>-3213145.056027305</v>
+        <v>-3065871.159610982</v>
       </c>
       <c r="I20">
-        <v>-600122.3336761077</v>
+        <v>-620006.5686167397</v>
       </c>
       <c r="J20">
-        <v>-2613022.722351198</v>
+        <v>-2445864.590994242</v>
       </c>
       <c r="K20">
         <v>0</v>
       </c>
       <c r="L20">
-        <v>1055511.27812622</v>
+        <v>705715.4422468342</v>
       </c>
       <c r="M20">
         <v>0</v>
       </c>
       <c r="N20">
-        <v>1055511.278126221</v>
+        <v>705715.4422468342</v>
       </c>
       <c r="O20">
-        <v>506645.4135005859</v>
+        <v>338743.4122784804</v>
       </c>
       <c r="P20">
-        <v>283066.6306022604</v>
+        <v>189258.5105821173</v>
       </c>
       <c r="Q20">
         <v>0</v>
       </c>
       <c r="R20">
-        <v>283066.6306022604</v>
+        <v>189258.5105821173</v>
       </c>
       <c r="S20">
-        <v>135871.982689085</v>
+        <v>90844.0850794163</v>
       </c>
     </row>
     <row r="21" spans="1:19">
@@ -1616,58 +1616,58 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>0.5389652497230566</v>
+        <v>0.5125242500923018</v>
       </c>
       <c r="C21">
-        <v>0.3291893115269993</v>
+        <v>0.2616404202269187</v>
       </c>
       <c r="D21">
-        <v>-1763401.595581684</v>
+        <v>-2413361.234176673</v>
       </c>
       <c r="E21">
         <v>0</v>
       </c>
       <c r="F21">
-        <v>-1763401.595581684</v>
+        <v>-2413361.234176673</v>
       </c>
       <c r="G21">
-        <v>-1763401.595581684</v>
+        <v>-2413361.234176673</v>
       </c>
       <c r="H21">
-        <v>-2118586.767538194</v>
+        <v>-3123131.479234727</v>
       </c>
       <c r="I21">
-        <v>-354827.3524120017</v>
+        <v>-625168.7164987884</v>
       </c>
       <c r="J21">
-        <v>-1763759.415126191</v>
+        <v>-2497962.762735938</v>
       </c>
       <c r="K21">
         <v>0</v>
       </c>
       <c r="L21">
-        <v>955851.3952862186</v>
+        <v>759712.8824659943</v>
       </c>
       <c r="M21">
         <v>0</v>
       </c>
       <c r="N21">
-        <v>955851.3952862184</v>
+        <v>759712.8824659943</v>
       </c>
       <c r="O21">
-        <v>458808.669737385</v>
+        <v>364662.1835836772</v>
       </c>
       <c r="P21">
-        <v>256339.8794757206</v>
+        <v>203739.5244573256</v>
       </c>
       <c r="Q21">
         <v>0</v>
       </c>
       <c r="R21">
-        <v>256339.8794757206</v>
+        <v>203739.5244573256</v>
       </c>
       <c r="S21">
-        <v>123043.142148346</v>
+        <v>97794.97173951629</v>
       </c>
     </row>
     <row r="22" spans="1:19">
@@ -1675,58 +1675,58 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0.4981064980218969</v>
+        <v>0.5072192823199134</v>
       </c>
       <c r="C22">
-        <v>0.4267737825966952</v>
+        <v>0.4633485986088892</v>
       </c>
       <c r="D22">
-        <v>-1485270.659973612</v>
+        <v>-1176844.573371003</v>
       </c>
       <c r="E22">
         <v>0</v>
       </c>
       <c r="F22">
-        <v>-1485270.659973612</v>
+        <v>-1176844.573371003</v>
       </c>
       <c r="G22">
-        <v>-1485270.659973612</v>
+        <v>-1176844.573371003</v>
       </c>
       <c r="H22">
-        <v>-1607393.791156176</v>
+        <v>-1125352.670121981</v>
       </c>
       <c r="I22">
-        <v>-188398.5318188959</v>
+        <v>-56772.91572494575</v>
       </c>
       <c r="J22">
-        <v>-1418995.259337279</v>
+        <v>-1068579.754397035</v>
       </c>
       <c r="K22">
         <v>0</v>
       </c>
       <c r="L22">
-        <v>1239202.796938839</v>
+        <v>1345403.355989266</v>
       </c>
       <c r="M22">
         <v>0</v>
       </c>
       <c r="N22">
-        <v>1239202.796938839</v>
+        <v>1345403.355989266</v>
       </c>
       <c r="O22">
-        <v>594817.3425306428</v>
+        <v>645793.6108748474</v>
       </c>
       <c r="P22">
-        <v>332328.9552955658</v>
+        <v>360809.7825889013</v>
       </c>
       <c r="Q22">
         <v>0</v>
       </c>
       <c r="R22">
-        <v>332328.9552955658</v>
+        <v>360809.7825889013</v>
       </c>
       <c r="S22">
-        <v>159517.8985418716</v>
+        <v>173188.6956426727</v>
       </c>
     </row>
     <row r="23" spans="1:19">
@@ -1734,58 +1734,58 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>0.3316582514423185</v>
+        <v>0.4051684913538617</v>
       </c>
       <c r="C23">
-        <v>0.4349465393458142</v>
+        <v>0.3668482636862165</v>
       </c>
       <c r="D23">
-        <v>-2824709.210912099</v>
+        <v>-2642667.935405116</v>
       </c>
       <c r="E23">
         <v>0</v>
       </c>
       <c r="F23">
-        <v>-2824709.210912099</v>
+        <v>-2642667.935405116</v>
       </c>
       <c r="G23">
-        <v>-2824709.210912099</v>
+        <v>-2642667.935405116</v>
       </c>
       <c r="H23">
-        <v>-3503041.195891079</v>
+        <v>-3324731.298660469</v>
       </c>
       <c r="I23">
-        <v>-636626.9407866879</v>
+        <v>-625203.372204633</v>
       </c>
       <c r="J23">
-        <v>-2866414.255104391</v>
+        <v>-2699527.926455836</v>
       </c>
       <c r="K23">
         <v>0</v>
       </c>
       <c r="L23">
-        <v>1262933.643197921</v>
+        <v>1065199.909062166</v>
       </c>
       <c r="M23">
         <v>0</v>
       </c>
       <c r="N23">
-        <v>1262933.643197921</v>
+        <v>1065199.909062166</v>
       </c>
       <c r="O23">
-        <v>606208.1487350023</v>
+        <v>511295.9563498397</v>
       </c>
       <c r="P23">
-        <v>338693.0850127049</v>
+        <v>285664.9241222081</v>
       </c>
       <c r="Q23">
         <v>0</v>
       </c>
       <c r="R23">
-        <v>338693.085012705</v>
+        <v>285664.924122208</v>
       </c>
       <c r="S23">
-        <v>162572.6808060984</v>
+        <v>137119.1635786598</v>
       </c>
     </row>
     <row r="24" spans="1:19">
@@ -1793,58 +1793,58 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0.3853632325194833</v>
+        <v>0.4146177695208894</v>
       </c>
       <c r="C24">
-        <v>0.2818449184538908</v>
+        <v>0.2901743485880965</v>
       </c>
       <c r="D24">
-        <v>-3347996.583903342</v>
+        <v>-3050566.297544352</v>
       </c>
       <c r="E24">
         <v>0</v>
       </c>
       <c r="F24">
-        <v>-3347996.583903342</v>
+        <v>-3050566.297544352</v>
       </c>
       <c r="G24">
-        <v>-3347996.583903342</v>
+        <v>-3050566.297544352</v>
       </c>
       <c r="H24">
-        <v>-4428706.485389816</v>
+        <v>-3995754.162596117</v>
       </c>
       <c r="I24">
-        <v>-927219.4204669525</v>
+        <v>-820192.445716145</v>
       </c>
       <c r="J24">
-        <v>-3501487.064922864</v>
+        <v>-3175561.716879972</v>
       </c>
       <c r="K24">
         <v>0</v>
       </c>
       <c r="L24">
-        <v>818379.725966243</v>
+        <v>842565.4973048931</v>
       </c>
       <c r="M24">
         <v>0</v>
       </c>
       <c r="N24">
-        <v>818379.7259662427</v>
+        <v>842565.4973048931</v>
       </c>
       <c r="O24">
-        <v>392822.2684637968</v>
+        <v>404431.4387063488</v>
       </c>
       <c r="P24">
-        <v>219472.7772058574</v>
+        <v>225958.908565346</v>
       </c>
       <c r="Q24">
         <v>0</v>
       </c>
       <c r="R24">
-        <v>219472.7772058574</v>
+        <v>225958.908565346</v>
       </c>
       <c r="S24">
-        <v>105346.9330588115</v>
+        <v>108460.2761113661</v>
       </c>
     </row>
     <row r="25" spans="1:19">
@@ -1852,58 +1852,58 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>0.5934960030551359</v>
+        <v>0.422727857061722</v>
       </c>
       <c r="C25">
-        <v>0.3534358405219293</v>
+        <v>0.5099555116669187</v>
       </c>
       <c r="D25">
-        <v>-1153613.475576132</v>
+        <v>-1587148.885008235</v>
       </c>
       <c r="E25">
         <v>0</v>
       </c>
       <c r="F25">
-        <v>-1153613.475576132</v>
+        <v>-1587148.885008235</v>
       </c>
       <c r="G25">
-        <v>-1153613.475576132</v>
+        <v>-1587148.885008235</v>
       </c>
       <c r="H25">
-        <v>-1222462.846090724</v>
+        <v>-1653811.8511676</v>
       </c>
       <c r="I25">
-        <v>-130104.5248023151</v>
+        <v>-161490.4271164532</v>
       </c>
       <c r="J25">
-        <v>-1092358.321288409</v>
+        <v>-1492321.424051146</v>
       </c>
       <c r="K25">
         <v>0</v>
       </c>
       <c r="L25">
-        <v>1026254.891873472</v>
+        <v>1480733.639557258</v>
       </c>
       <c r="M25">
         <v>0</v>
       </c>
       <c r="N25">
-        <v>1026254.891873472</v>
+        <v>1480733.639557258</v>
       </c>
       <c r="O25">
-        <v>492602.3480992667</v>
+        <v>710752.1469874837</v>
       </c>
       <c r="P25">
-        <v>275220.6635796576</v>
+        <v>397102.6088067744</v>
       </c>
       <c r="Q25">
         <v>0</v>
       </c>
       <c r="R25">
-        <v>275220.6635796576</v>
+        <v>397102.6088067744</v>
       </c>
       <c r="S25">
-        <v>132105.9185182356</v>
+        <v>190609.2522272518</v>
       </c>
     </row>
     <row r="26" spans="1:19">
@@ -1911,58 +1911,58 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0.3664197696903931</v>
+        <v>0.4514005906228594</v>
       </c>
       <c r="C26">
-        <v>0.3734406063096361</v>
+        <v>0.2645228041110123</v>
       </c>
       <c r="D26">
-        <v>-2924705.560838273</v>
+        <v>-2905988.814329171</v>
       </c>
       <c r="E26">
         <v>0</v>
       </c>
       <c r="F26">
-        <v>-2924705.560838273</v>
+        <v>-2905988.814329171</v>
       </c>
       <c r="G26">
-        <v>-2924705.560838273</v>
+        <v>-2905988.814329171</v>
       </c>
       <c r="H26">
-        <v>-3718117.866344525</v>
+        <v>-3820471.417441091</v>
       </c>
       <c r="I26">
-        <v>-715984.8352072628</v>
+        <v>-790112.3390597637</v>
       </c>
       <c r="J26">
-        <v>-3002133.031137263</v>
+        <v>-3030359.078381327</v>
       </c>
       <c r="K26">
         <v>0</v>
       </c>
       <c r="L26">
-        <v>1084341.781760191</v>
+        <v>768082.3238812733</v>
       </c>
       <c r="M26">
         <v>0</v>
       </c>
       <c r="N26">
-        <v>1084341.781760191</v>
+        <v>768082.3238812733</v>
       </c>
       <c r="O26">
-        <v>520484.0552448917</v>
+        <v>368679.5154630112</v>
       </c>
       <c r="P26">
-        <v>290798.3845790837</v>
+        <v>205984.0382115053</v>
       </c>
       <c r="Q26">
         <v>0</v>
       </c>
       <c r="R26">
-        <v>290798.3845790837</v>
+        <v>205984.0382115053</v>
       </c>
       <c r="S26">
-        <v>139583.2245979602</v>
+        <v>98872.33834152254</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor(data_loader): enhance dynamic TC handling and warnings
- Removed the obsolete `read_excel_data.py` script.
- Improved `load_tc_parameters` function to handle missing static TC definitions with warnings.
- Added checks to ensure `Process_ID` is an integer and to handle dynamic TC values more robustly.
- Updated interpolation logic to handle cases with all NaN values, setting them to zero.
- Enhanced warnings for years outside the defined time range during dynamic TC loading.
- Updated plotting functions to include interactive elements for better user experience.
</commit_message>
<xml_diff>
--- a/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
+++ b/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
@@ -495,58 +495,58 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>0.3960433521366136</v>
+        <v>0.3300650954079945</v>
       </c>
       <c r="C2">
-        <v>0.3892089166004167</v>
+        <v>0.3300347479000214</v>
       </c>
       <c r="D2">
-        <v>-2576953.036216497</v>
+        <v>-3852952.853344902</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>-2576953.036216497</v>
+        <v>-3852952.853344902</v>
       </c>
       <c r="G2">
-        <v>-2576953.036216497</v>
+        <v>-3852952.853344902</v>
       </c>
       <c r="H2">
-        <v>-3204774.197456812</v>
+        <v>-5324747.412744758</v>
       </c>
       <c r="I2">
-        <v>-586394.9032031018</v>
+        <v>-1150715.1574829</v>
       </c>
       <c r="J2">
-        <v>-2618379.29425371</v>
+        <v>-4174032.255261858</v>
       </c>
       <c r="K2">
         <v>0</v>
       </c>
       <c r="L2">
-        <v>1130127.476693097</v>
+        <v>958306.2487959826</v>
       </c>
       <c r="M2">
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1130127.476693098</v>
+        <v>958306.2487959825</v>
       </c>
       <c r="O2">
-        <v>542461.1888126868</v>
+        <v>459986.9994220718</v>
       </c>
       <c r="P2">
-        <v>303077.175590629</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
       <c r="R2">
-        <v>303077.175590629</v>
+        <v>0</v>
       </c>
       <c r="S2">
-        <v>145477.0442835019</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -554,58 +554,58 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>0.4953343596326366</v>
+        <v>0.535772198783161</v>
       </c>
       <c r="C3">
-        <v>0.4481760908787957</v>
+        <v>0.2552318785963185</v>
       </c>
       <c r="D3">
-        <v>-1372536.763204096</v>
+        <v>-2529416.36917831</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3">
-        <v>-1372536.763204096</v>
+        <v>-2529416.36917831</v>
       </c>
       <c r="G3">
-        <v>-1372536.763204096</v>
+        <v>-2529416.36917831</v>
       </c>
       <c r="H3">
-        <v>-1421687.92506163</v>
+        <v>-3477400.804963621</v>
       </c>
       <c r="I3">
-        <v>-134351.7819391069</v>
+        <v>-737199.7421825835</v>
       </c>
       <c r="J3">
-        <v>-1287336.143122522</v>
+        <v>-2740201.062781036</v>
       </c>
       <c r="K3">
         <v>0</v>
       </c>
       <c r="L3">
-        <v>1301347.664701696</v>
+        <v>741104.7039958478</v>
       </c>
       <c r="M3">
         <v>0</v>
       </c>
       <c r="N3">
-        <v>1301347.664701696</v>
+        <v>741104.7039958478</v>
       </c>
       <c r="O3">
-        <v>624646.8790568142</v>
+        <v>355730.2579180071</v>
       </c>
       <c r="P3">
-        <v>348994.9433256356</v>
+        <v>0</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
       <c r="R3">
-        <v>348994.9433256356</v>
+        <v>0</v>
       </c>
       <c r="S3">
-        <v>167517.5727963051</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -613,58 +613,58 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.5984464829628622</v>
+        <v>0.5896335647893132</v>
       </c>
       <c r="C4">
-        <v>0.3316639504335053</v>
+        <v>0.5280671019942949</v>
       </c>
       <c r="D4">
-        <v>-1250485.547876938</v>
+        <v>-634958.2927012753</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>-1250485.547876938</v>
+        <v>-634958.2927012753</v>
       </c>
       <c r="G4">
-        <v>-1250485.547876938</v>
+        <v>-634958.2927012753</v>
       </c>
       <c r="H4">
-        <v>-1386043.223887909</v>
+        <v>-653605.0703298808</v>
       </c>
       <c r="I4">
-        <v>-179044.8499575838</v>
+        <v>34266.40874902662</v>
       </c>
       <c r="J4">
-        <v>-1206998.373930324</v>
+        <v>-687871.4790789078</v>
       </c>
       <c r="K4">
         <v>0</v>
       </c>
       <c r="L4">
-        <v>963036.8869434083</v>
+        <v>1533323.405625209</v>
       </c>
       <c r="M4">
         <v>0</v>
       </c>
       <c r="N4">
-        <v>963036.8869434083</v>
+        <v>1533323.405625209</v>
       </c>
       <c r="O4">
-        <v>462257.7057328359</v>
+        <v>735995.2347001006</v>
       </c>
       <c r="P4">
-        <v>258266.8820144639</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
       <c r="R4">
-        <v>258266.8820144639</v>
+        <v>0</v>
       </c>
       <c r="S4">
-        <v>123968.1033669427</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -672,58 +672,58 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>0.4520301027710972</v>
+        <v>0.4093599894573831</v>
       </c>
       <c r="C5">
-        <v>0.3713084606476049</v>
+        <v>0.4731179237872294</v>
       </c>
       <c r="D5">
-        <v>-2222630.514781113</v>
+        <v>-2432729.22192007</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>-2222630.514781113</v>
+        <v>-2432729.22192007</v>
       </c>
       <c r="G5">
-        <v>-2222630.514781113</v>
+        <v>-2432729.22192007</v>
       </c>
       <c r="H5">
-        <v>-2721954.553451012</v>
+        <v>-3236873.173442998</v>
       </c>
       <c r="I5">
-        <v>-479453.3504282762</v>
+        <v>-601416.5196933598</v>
       </c>
       <c r="J5">
-        <v>-2242501.203022736</v>
+        <v>-2635456.653749638</v>
       </c>
       <c r="K5">
         <v>0</v>
       </c>
       <c r="L5">
-        <v>1078150.771497579</v>
+        <v>1373770.08229458</v>
       </c>
       <c r="M5">
         <v>0</v>
       </c>
       <c r="N5">
-        <v>1078150.771497579</v>
+        <v>1373770.08229458</v>
       </c>
       <c r="O5">
-        <v>517512.3703188378</v>
+        <v>659409.6395013983</v>
       </c>
       <c r="P5">
-        <v>289138.0816989736</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
       <c r="R5">
-        <v>289138.0816989736</v>
+        <v>0</v>
       </c>
       <c r="S5">
-        <v>138786.2792155074</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:19">
@@ -731,58 +731,58 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>0.3523289163944616</v>
+        <v>0.5808678480067124</v>
       </c>
       <c r="C6">
-        <v>0.3405531674562756</v>
+        <v>0.4199853283774986</v>
       </c>
       <c r="D6">
-        <v>-3251328.08604714</v>
+        <v>-1280353.300105714</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
       <c r="F6">
-        <v>-3251328.08604714</v>
+        <v>-1280353.300105714</v>
       </c>
       <c r="G6">
-        <v>-3251328.08604714</v>
+        <v>-1280353.300105714</v>
       </c>
       <c r="H6">
-        <v>-4221676.568064854</v>
+        <v>-1622755.878132736</v>
       </c>
       <c r="I6">
-        <v>-851057.2607848514</v>
+        <v>-235706.4741156322</v>
       </c>
       <c r="J6">
-        <v>-3370619.307280004</v>
+        <v>-1387049.404017104</v>
       </c>
       <c r="K6">
         <v>0</v>
       </c>
       <c r="L6">
-        <v>988848.0849279459</v>
+        <v>1219491.484298837</v>
       </c>
       <c r="M6">
         <v>0</v>
       </c>
       <c r="N6">
-        <v>988848.0849279461</v>
+        <v>1219491.484298837</v>
       </c>
       <c r="O6">
-        <v>474647.080765414</v>
+        <v>585355.9124634417</v>
       </c>
       <c r="P6">
-        <v>265188.9197005617</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
       <c r="R6">
-        <v>265188.9197005617</v>
+        <v>0</v>
       </c>
       <c r="S6">
-        <v>127290.6814562696</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:19">
@@ -790,58 +790,58 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>0.3681817590423575</v>
+        <v>0.3705541202939737</v>
       </c>
       <c r="C7">
-        <v>0.5256855429273644</v>
+        <v>0.4317885854590039</v>
       </c>
       <c r="D7">
-        <v>-1943211.377888573</v>
+        <v>-2975880.071387835</v>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
       <c r="F7">
-        <v>-1943211.377888573</v>
+        <v>-2975880.071387835</v>
       </c>
       <c r="G7">
-        <v>-1943211.377888573</v>
+        <v>-2975880.071387835</v>
       </c>
       <c r="H7">
-        <v>-2141676.733929151</v>
+        <v>-4029030.597618576</v>
       </c>
       <c r="I7">
-        <v>-270625.7310619875</v>
+        <v>-805160.5232699048</v>
       </c>
       <c r="J7">
-        <v>-1871051.002867163</v>
+        <v>-3223870.074348671</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
       <c r="L7">
-        <v>1526408.185484791</v>
+        <v>1253764.042231975</v>
       </c>
       <c r="M7">
         <v>0</v>
       </c>
       <c r="N7">
-        <v>1526408.185484791</v>
+        <v>1253764.042231975</v>
       </c>
       <c r="O7">
-        <v>732675.9290326998</v>
+        <v>601806.740271348</v>
       </c>
       <c r="P7">
-        <v>409351.5919184914</v>
+        <v>0</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
       <c r="R7">
-        <v>409351.5919184914</v>
+        <v>0</v>
       </c>
       <c r="S7">
-        <v>196488.7641208759</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:19">
@@ -849,58 +849,58 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0.4179183159149376</v>
+        <v>0.3534558264935208</v>
       </c>
       <c r="C8">
-        <v>0.5203040848975512</v>
+        <v>0.4164929836432453</v>
       </c>
       <c r="D8">
-        <v>-1561637.55331131</v>
+        <v>-3199770.32111614</v>
       </c>
       <c r="E8">
         <v>0</v>
       </c>
       <c r="F8">
-        <v>-1561637.55331131</v>
+        <v>-3199770.32111614</v>
       </c>
       <c r="G8">
-        <v>-1561637.55331131</v>
+        <v>-3199770.32111614</v>
       </c>
       <c r="H8">
-        <v>-1605267.952452058</v>
+        <v>-4354740.180671622</v>
       </c>
       <c r="I8">
-        <v>-145192.1595107507</v>
+        <v>-888322.3356382377</v>
       </c>
       <c r="J8">
-        <v>-1460075.792941306</v>
+        <v>-3466417.845033383</v>
       </c>
       <c r="K8">
         <v>0</v>
       </c>
       <c r="L8">
-        <v>1510782.30096682</v>
+        <v>1209350.928484397</v>
       </c>
       <c r="M8">
         <v>0</v>
       </c>
       <c r="N8">
-        <v>1510782.30096682</v>
+        <v>1209350.928484397</v>
       </c>
       <c r="O8">
-        <v>725175.5044640737</v>
+        <v>580488.4456725108</v>
       </c>
       <c r="P8">
-        <v>405161.0478927241</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>0</v>
       </c>
       <c r="R8">
-        <v>405161.0478927241</v>
+        <v>0</v>
       </c>
       <c r="S8">
-        <v>194477.3029885076</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:19">
@@ -908,58 +908,58 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0.4974801446411339</v>
+        <v>0.4789835713222546</v>
       </c>
       <c r="C9">
-        <v>0.484522026734526</v>
+        <v>0.4931469555338494</v>
       </c>
       <c r="D9">
-        <v>-1123801.028338873</v>
+        <v>-1744725.546290438</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
       <c r="F9">
-        <v>-1123801.028338873</v>
+        <v>-1744725.546290438</v>
       </c>
       <c r="G9">
-        <v>-1123801.028338873</v>
+        <v>-1744725.546290438</v>
       </c>
       <c r="H9">
-        <v>-1024826.206789318</v>
+        <v>-2248733.802715405</v>
       </c>
       <c r="I9">
-        <v>-23139.09751300172</v>
+        <v>-358614.4647506431</v>
       </c>
       <c r="J9">
-        <v>-1001687.109276317</v>
+        <v>-1890119.337964762</v>
       </c>
       <c r="K9">
         <v>0</v>
       </c>
       <c r="L9">
-        <v>1406883.63529421</v>
+        <v>1431927.432095618</v>
       </c>
       <c r="M9">
         <v>0</v>
       </c>
       <c r="N9">
-        <v>1406883.63529421</v>
+        <v>1431927.432095618</v>
       </c>
       <c r="O9">
-        <v>675304.1449412209</v>
+        <v>687325.1674058971</v>
       </c>
       <c r="P9">
-        <v>377297.5415280868</v>
+        <v>0</v>
       </c>
       <c r="Q9">
         <v>0</v>
       </c>
       <c r="R9">
-        <v>377297.5415280868</v>
+        <v>0</v>
       </c>
       <c r="S9">
-        <v>181102.8199334816</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:19">
@@ -967,58 +967,58 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0.3467129848896737</v>
+        <v>0.5160107829338383</v>
       </c>
       <c r="C10">
-        <v>0.3343490320185892</v>
+        <v>0.3445286318531346</v>
       </c>
       <c r="D10">
-        <v>-3337668.180831301</v>
+        <v>-2221915.918403574</v>
       </c>
       <c r="E10">
         <v>0</v>
       </c>
       <c r="F10">
-        <v>-3337668.180831301</v>
+        <v>-2221915.918403574</v>
       </c>
       <c r="G10">
-        <v>-3337668.180831301</v>
+        <v>-2221915.918403574</v>
       </c>
       <c r="H10">
-        <v>-4351840.46296475</v>
+        <v>-2997777.902377266</v>
       </c>
       <c r="I10">
-        <v>-884923.2702307812</v>
+        <v>-590702.3279542439</v>
       </c>
       <c r="J10">
-        <v>-3466917.192733969</v>
+        <v>-2407075.574423022</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>970833.4310281919</v>
+        <v>1000391.452399452</v>
       </c>
       <c r="M10">
         <v>0</v>
       </c>
       <c r="N10">
-        <v>970833.4310281919</v>
+        <v>1000391.452399452</v>
       </c>
       <c r="O10">
-        <v>466000.0468935322</v>
+        <v>480187.897151737</v>
       </c>
       <c r="P10">
-        <v>260357.7563709554</v>
+        <v>0</v>
       </c>
       <c r="Q10">
         <v>0</v>
       </c>
       <c r="R10">
-        <v>260357.7563709554</v>
+        <v>0</v>
       </c>
       <c r="S10">
-        <v>124971.7230580586</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:19">
@@ -1026,58 +1026,58 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0.4276591538736274</v>
+        <v>0.4445391346994594</v>
       </c>
       <c r="C11">
-        <v>0.2700794309404495</v>
+        <v>0.45465360696859</v>
       </c>
       <c r="D11">
-        <v>-3069157.842085347</v>
+        <v>-2236407.210642167</v>
       </c>
       <c r="E11">
         <v>0</v>
       </c>
       <c r="F11">
-        <v>-3069157.842085347</v>
+        <v>-2236407.210642167</v>
       </c>
       <c r="G11">
-        <v>-3069157.842085347</v>
+        <v>-2236407.210642167</v>
       </c>
       <c r="H11">
-        <v>-4045996.177542837</v>
+        <v>-2966336.771248278</v>
       </c>
       <c r="I11">
-        <v>-841345.0909323925</v>
+        <v>-543562.2965954929</v>
       </c>
       <c r="J11">
-        <v>-3204651.086610445</v>
+        <v>-2422774.474652785</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>784216.8377370393</v>
+        <v>1320156.121038564</v>
       </c>
       <c r="M11">
         <v>0</v>
       </c>
       <c r="N11">
-        <v>784216.8377370393</v>
+        <v>1320156.121038564</v>
       </c>
       <c r="O11">
-        <v>376424.0821137789</v>
+        <v>633674.9380985106</v>
       </c>
       <c r="P11">
-        <v>210310.9862680575</v>
+        <v>0</v>
       </c>
       <c r="Q11">
         <v>0</v>
       </c>
       <c r="R11">
-        <v>210310.9862680575</v>
+        <v>0</v>
       </c>
       <c r="S11">
-        <v>100949.2734086676</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:19">
@@ -1085,58 +1085,58 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>0.3070714433698677</v>
+        <v>0.3913670061184192</v>
       </c>
       <c r="C12">
-        <v>0.290192657341922</v>
+        <v>0.3826027136110881</v>
       </c>
       <c r="D12">
-        <v>-3949426.68903621</v>
+        <v>-3062267.420674835</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
       <c r="F12">
-        <v>-3949426.68903621</v>
+        <v>-3062267.420674835</v>
       </c>
       <c r="G12">
-        <v>-3949426.68903621</v>
+        <v>-3062267.420674835</v>
       </c>
       <c r="H12">
-        <v>-5274343.968946022</v>
+        <v>-4175164.481002862</v>
       </c>
       <c r="I12">
-        <v>-1125024.980329387</v>
+        <v>-857708.1116520369</v>
       </c>
       <c r="J12">
-        <v>-4149318.988616633</v>
+        <v>-3317456.369350824</v>
       </c>
       <c r="K12">
         <v>0</v>
       </c>
       <c r="L12">
-        <v>842618.6595652619</v>
+        <v>1110945.358307775</v>
       </c>
       <c r="M12">
         <v>0</v>
       </c>
       <c r="N12">
-        <v>842618.6595652619</v>
+        <v>1110945.358307775</v>
       </c>
       <c r="O12">
-        <v>404456.9565913258</v>
+        <v>533253.771987732</v>
       </c>
       <c r="P12">
-        <v>225973.1656009927</v>
+        <v>0</v>
       </c>
       <c r="Q12">
         <v>0</v>
       </c>
       <c r="R12">
-        <v>225973.1656009927</v>
+        <v>0</v>
       </c>
       <c r="S12">
-        <v>108467.1194884765</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -1144,58 +1144,58 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>0.491958970463221</v>
+        <v>0.5752409098045101</v>
       </c>
       <c r="C13">
-        <v>0.3655469159831034</v>
+        <v>0.5700569717931837</v>
       </c>
       <c r="D13">
-        <v>-1925452.458684279</v>
+        <v>-532995.906594994</v>
       </c>
       <c r="E13">
         <v>0</v>
       </c>
       <c r="F13">
-        <v>-1925452.458684279</v>
+        <v>-532995.906594994</v>
       </c>
       <c r="G13">
-        <v>-1925452.458684279</v>
+        <v>-532995.906594994</v>
       </c>
       <c r="H13">
-        <v>-2306047.206227333</v>
+        <v>-488717.460066537</v>
       </c>
       <c r="I13">
-        <v>-382923.206320744</v>
+        <v>88694.76742391619</v>
       </c>
       <c r="J13">
-        <v>-1923123.999906589</v>
+        <v>-577412.227490453</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13">
-        <v>1061421.247440368</v>
+        <v>1655247.399599912</v>
       </c>
       <c r="M13">
         <v>0</v>
       </c>
       <c r="N13">
-        <v>1061421.247440368</v>
+        <v>1655247.399599912</v>
       </c>
       <c r="O13">
-        <v>509482.1987713766</v>
+        <v>794518.751807958</v>
       </c>
       <c r="P13">
-        <v>284651.5640230461</v>
+        <v>0</v>
       </c>
       <c r="Q13">
         <v>0</v>
       </c>
       <c r="R13">
-        <v>284651.5640230461</v>
+        <v>0</v>
       </c>
       <c r="S13">
-        <v>136632.7507310621</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:19">
@@ -1203,58 +1203,58 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>0.407037062532454</v>
+        <v>0.386708424313029</v>
       </c>
       <c r="C14">
-        <v>0.5630012211207192</v>
+        <v>0.3963616530678007</v>
       </c>
       <c r="D14">
-        <v>-1381463.901534106</v>
+        <v>-3028376.474733957</v>
       </c>
       <c r="E14">
         <v>0</v>
       </c>
       <c r="F14">
-        <v>-1381463.901534106</v>
+        <v>-3028376.474733957</v>
       </c>
       <c r="G14">
-        <v>-1381463.901534106</v>
+        <v>-3028376.474733957</v>
       </c>
       <c r="H14">
-        <v>-1298413.53468013</v>
+        <v>-4120451.586719099</v>
       </c>
       <c r="I14">
-        <v>-52539.45815295089</v>
+        <v>-839710.4087958848</v>
       </c>
       <c r="J14">
-        <v>-1245874.076527179</v>
+        <v>-3280741.177923216</v>
       </c>
       <c r="K14">
         <v>0</v>
       </c>
       <c r="L14">
-        <v>1634759.950922486</v>
+        <v>1150896.538424626</v>
       </c>
       <c r="M14">
         <v>0</v>
       </c>
       <c r="N14">
-        <v>1634759.950922485</v>
+        <v>1150896.538424626</v>
       </c>
       <c r="O14">
-        <v>784684.776442793</v>
+        <v>552430.3384438206</v>
       </c>
       <c r="P14">
-        <v>438409.3289582155</v>
+        <v>0</v>
       </c>
       <c r="Q14">
         <v>0</v>
       </c>
       <c r="R14">
-        <v>438409.3289582155</v>
+        <v>0</v>
       </c>
       <c r="S14">
-        <v>210436.4778999434</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:19">
@@ -1262,58 +1262,58 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0.3398072808900268</v>
+        <v>0.3086713916747138</v>
       </c>
       <c r="C15">
-        <v>0.3023317000812984</v>
+        <v>0.346022001402262</v>
       </c>
       <c r="D15">
-        <v>-3598705.010859956</v>
+        <v>-3947154.900646711</v>
       </c>
       <c r="E15">
         <v>0</v>
       </c>
       <c r="F15">
-        <v>-3598705.010859956</v>
+        <v>-3947154.900646711</v>
       </c>
       <c r="G15">
-        <v>-3598705.010859956</v>
+        <v>-3947154.900646711</v>
       </c>
       <c r="H15">
-        <v>-4761074.425299866</v>
+        <v>-5451191.022441128</v>
       </c>
       <c r="I15">
-        <v>-997109.5962524704</v>
+        <v>-1175106.549148097</v>
       </c>
       <c r="J15">
-        <v>-3763964.829047395</v>
+        <v>-4276084.473293031</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
-        <v>877866.2223917973</v>
+        <v>1004727.678750757</v>
       </c>
       <c r="M15">
         <v>0</v>
       </c>
       <c r="N15">
-        <v>877866.2223917973</v>
+        <v>1004727.678750757</v>
       </c>
       <c r="O15">
-        <v>421375.7867480629</v>
+        <v>482269.2858003636</v>
       </c>
       <c r="P15">
-        <v>235425.8441777306</v>
+        <v>0</v>
       </c>
       <c r="Q15">
         <v>0</v>
       </c>
       <c r="R15">
-        <v>235425.8441777306</v>
+        <v>0</v>
       </c>
       <c r="S15">
-        <v>113004.4052053107</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:19">
@@ -1321,58 +1321,58 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>0.4683024327291097</v>
+        <v>0.344784598808699</v>
       </c>
       <c r="C16">
-        <v>0.531768375522468</v>
+        <v>0.5331005753838244</v>
       </c>
       <c r="D16">
-        <v>-1067679.137180448</v>
+        <v>-2654999.46347141</v>
       </c>
       <c r="E16">
         <v>0</v>
       </c>
       <c r="F16">
-        <v>-1067679.137180448</v>
+        <v>-2654999.46347141</v>
       </c>
       <c r="G16">
-        <v>-1067679.137180448</v>
+        <v>-2654999.46347141</v>
       </c>
       <c r="H16">
-        <v>-889045.9496918081</v>
+        <v>-3524695.22705815</v>
       </c>
       <c r="I16">
-        <v>30803.02672342329</v>
+        <v>-648445.8112835408</v>
       </c>
       <c r="J16">
-        <v>-919848.9764152311</v>
+        <v>-2876249.415774608</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
       <c r="L16">
-        <v>1544070.618072142</v>
+        <v>1547938.863642968</v>
       </c>
       <c r="M16">
         <v>0</v>
       </c>
       <c r="N16">
-        <v>1544070.618072142</v>
+        <v>1547938.863642968</v>
       </c>
       <c r="O16">
-        <v>741153.8966746284</v>
+        <v>743010.6545486248</v>
       </c>
       <c r="P16">
-        <v>414088.296664666</v>
+        <v>0</v>
       </c>
       <c r="Q16">
         <v>0</v>
       </c>
       <c r="R16">
-        <v>414088.296664666</v>
+        <v>0</v>
       </c>
       <c r="S16">
-        <v>198762.3823990397</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:19">
@@ -1380,58 +1380,58 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0.352969618493466</v>
+        <v>0.5174019413933307</v>
       </c>
       <c r="C17">
-        <v>0.4326959043739886</v>
+        <v>0.3390526731520805</v>
       </c>
       <c r="D17">
-        <v>-2660859.791509783</v>
+        <v>-2239273.834868472</v>
       </c>
       <c r="E17">
         <v>0</v>
       </c>
       <c r="F17">
-        <v>-2660859.791509783</v>
+        <v>-2239273.834868472</v>
       </c>
       <c r="G17">
-        <v>-2660859.791509783</v>
+        <v>-2239273.834868472</v>
       </c>
       <c r="H17">
-        <v>-3272633.718287089</v>
+        <v>-3025057.620095644</v>
       </c>
       <c r="I17">
-        <v>-582720.763799594</v>
+        <v>-599177.6361690817</v>
       </c>
       <c r="J17">
-        <v>-2689912.954487495</v>
+        <v>-2425879.983926562</v>
       </c>
       <c r="K17">
         <v>0</v>
       </c>
       <c r="L17">
-        <v>1256398.58114466</v>
+        <v>984491.1707631727</v>
       </c>
       <c r="M17">
         <v>0</v>
       </c>
       <c r="N17">
-        <v>1256398.581144659</v>
+        <v>984491.1707631727</v>
       </c>
       <c r="O17">
-        <v>603071.3189494367</v>
+        <v>472555.761966323</v>
       </c>
       <c r="P17">
-        <v>336940.514448535</v>
+        <v>0</v>
       </c>
       <c r="Q17">
         <v>0</v>
       </c>
       <c r="R17">
-        <v>336940.514448535</v>
+        <v>0</v>
       </c>
       <c r="S17">
-        <v>161731.4469352968</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:19">
@@ -1439,58 +1439,58 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0.3848249279142985</v>
+        <v>0.5779434757922117</v>
       </c>
       <c r="C18">
-        <v>0.3645135666526405</v>
+        <v>0.5180519784968147</v>
       </c>
       <c r="D18">
-        <v>-2827544.684172722</v>
+        <v>-785689.7041265869</v>
       </c>
       <c r="E18">
         <v>0</v>
       </c>
       <c r="F18">
-        <v>-2827544.684172722</v>
+        <v>-785689.7041265869</v>
       </c>
       <c r="G18">
-        <v>-2827544.684172722</v>
+        <v>-785689.7041265869</v>
       </c>
       <c r="H18">
-        <v>-3590479.581227965</v>
+        <v>-872751.606921935</v>
       </c>
       <c r="I18">
-        <v>-689628.8389785311</v>
+        <v>-21587.76536675355</v>
       </c>
       <c r="J18">
-        <v>-2900850.742249433</v>
+        <v>-851163.8415551813</v>
       </c>
       <c r="K18">
         <v>0</v>
       </c>
       <c r="L18">
-        <v>1058420.759986023</v>
+        <v>1504242.966395198</v>
       </c>
       <c r="M18">
         <v>0</v>
       </c>
       <c r="N18">
-        <v>1058420.759986023</v>
+        <v>1504242.966395198</v>
       </c>
       <c r="O18">
-        <v>508041.9647932911</v>
+        <v>722036.6238696952</v>
       </c>
       <c r="P18">
-        <v>283846.8943890338</v>
+        <v>0</v>
       </c>
       <c r="Q18">
         <v>0</v>
       </c>
       <c r="R18">
-        <v>283846.8943890337</v>
+        <v>0</v>
       </c>
       <c r="S18">
-        <v>136246.5093067363</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:19">
@@ -1498,58 +1498,58 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>0.3051651044829288</v>
+        <v>0.5354723691847816</v>
       </c>
       <c r="C19">
-        <v>0.4096254725664755</v>
+        <v>0.5893501048511529</v>
       </c>
       <c r="D19">
-        <v>-3206955.172481899</v>
+        <v>-763293.2664984402</v>
       </c>
       <c r="E19">
         <v>0</v>
       </c>
       <c r="F19">
-        <v>-3206955.172481899</v>
+        <v>-763293.2664984402</v>
       </c>
       <c r="G19">
-        <v>-3206955.172481899</v>
+        <v>-763293.2664984402</v>
       </c>
       <c r="H19">
-        <v>-4076763.247691954</v>
+        <v>-807191.3660601664</v>
       </c>
       <c r="I19">
-        <v>-784973.3981741692</v>
+        <v>19709.66823529205</v>
       </c>
       <c r="J19">
-        <v>-3291789.849517783</v>
+        <v>-826901.0342954585</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
-        <v>1189410.062195561</v>
+        <v>1711267.955271539</v>
       </c>
       <c r="M19">
         <v>0</v>
       </c>
       <c r="N19">
-        <v>1189410.062195561</v>
+        <v>1711267.955271539</v>
       </c>
       <c r="O19">
-        <v>570916.8298538695</v>
+        <v>821408.6185303386</v>
       </c>
       <c r="P19">
-        <v>318975.5578053248</v>
+        <v>0</v>
       </c>
       <c r="Q19">
         <v>0</v>
       </c>
       <c r="R19">
-        <v>318975.5578053248</v>
+        <v>0</v>
       </c>
       <c r="S19">
-        <v>153108.2677465559</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:19">
@@ -1557,58 +1557,58 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>0.533319049537044</v>
+        <v>0.3476537348303897</v>
       </c>
       <c r="C20">
-        <v>0.243044035624014</v>
+        <v>0.4947783044710695</v>
       </c>
       <c r="D20">
-        <v>-2357626.417146617</v>
+        <v>-2833872.45860434</v>
       </c>
       <c r="E20">
         <v>0</v>
       </c>
       <c r="F20">
-        <v>-2357626.417146617</v>
+        <v>-2833872.45860434</v>
       </c>
       <c r="G20">
-        <v>-2357626.417146617</v>
+        <v>-2833872.45860434</v>
       </c>
       <c r="H20">
-        <v>-3065871.159610982</v>
+        <v>-3797253.059520672</v>
       </c>
       <c r="I20">
-        <v>-620006.5686167397</v>
+        <v>-727224.5656383124</v>
       </c>
       <c r="J20">
-        <v>-2445864.590994242</v>
+        <v>-3070028.493882359</v>
       </c>
       <c r="K20">
         <v>0</v>
       </c>
       <c r="L20">
-        <v>705715.4422468342</v>
+        <v>1436664.3026538</v>
       </c>
       <c r="M20">
         <v>0</v>
       </c>
       <c r="N20">
-        <v>705715.4422468342</v>
+        <v>1436664.3026538</v>
       </c>
       <c r="O20">
-        <v>338743.4122784804</v>
+        <v>689598.8652738243</v>
       </c>
       <c r="P20">
-        <v>189258.5105821173</v>
+        <v>0</v>
       </c>
       <c r="Q20">
         <v>0</v>
       </c>
       <c r="R20">
-        <v>189258.5105821173</v>
+        <v>0</v>
       </c>
       <c r="S20">
-        <v>90844.0850794163</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:19">
@@ -1616,58 +1616,58 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>0.5125242500923018</v>
+        <v>0.5894698208136384</v>
       </c>
       <c r="C21">
-        <v>0.2616404202269187</v>
+        <v>0.3409154809448693</v>
       </c>
       <c r="D21">
-        <v>-2413361.234176673</v>
+        <v>-1626999.868301982</v>
       </c>
       <c r="E21">
         <v>0</v>
       </c>
       <c r="F21">
-        <v>-2413361.234176673</v>
+        <v>-1626999.868301982</v>
       </c>
       <c r="G21">
-        <v>-2413361.234176673</v>
+        <v>-1626999.868301982</v>
       </c>
       <c r="H21">
-        <v>-3123131.479234727</v>
+        <v>-2153229.242228498</v>
       </c>
       <c r="I21">
-        <v>-625168.7164987884</v>
+        <v>-390646.0559203024</v>
       </c>
       <c r="J21">
-        <v>-2497962.762735938</v>
+        <v>-1762583.186308196</v>
       </c>
       <c r="K21">
         <v>0</v>
       </c>
       <c r="L21">
-        <v>759712.8824659943</v>
+        <v>989900.1174255891</v>
       </c>
       <c r="M21">
         <v>0</v>
       </c>
       <c r="N21">
-        <v>759712.8824659943</v>
+        <v>989900.1174255894</v>
       </c>
       <c r="O21">
-        <v>364662.1835836772</v>
+        <v>475152.0563642829</v>
       </c>
       <c r="P21">
-        <v>203739.5244573256</v>
+        <v>0</v>
       </c>
       <c r="Q21">
         <v>0</v>
       </c>
       <c r="R21">
-        <v>203739.5244573256</v>
+        <v>0</v>
       </c>
       <c r="S21">
-        <v>97794.97173951629</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:19">
@@ -1675,58 +1675,58 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0.5072192823199134</v>
+        <v>0.3924347186545817</v>
       </c>
       <c r="C22">
-        <v>0.4633485986088892</v>
+        <v>0.2127731770273897</v>
       </c>
       <c r="D22">
-        <v>-1176844.573371003</v>
+        <v>-3952322.152525235</v>
       </c>
       <c r="E22">
         <v>0</v>
       </c>
       <c r="F22">
-        <v>-1176844.573371003</v>
+        <v>-3952322.152525235</v>
       </c>
       <c r="G22">
-        <v>-1176844.573371003</v>
+        <v>-3952322.152525235</v>
       </c>
       <c r="H22">
-        <v>-1125352.670121981</v>
+        <v>-5521526.409101821</v>
       </c>
       <c r="I22">
-        <v>-56772.91572494575</v>
+        <v>-1239844.079956746</v>
       </c>
       <c r="J22">
-        <v>-1068579.754397035</v>
+        <v>-4281682.329145076</v>
       </c>
       <c r="K22">
         <v>0</v>
       </c>
       <c r="L22">
-        <v>1345403.355989266</v>
+        <v>617819.385440257</v>
       </c>
       <c r="M22">
         <v>0</v>
       </c>
       <c r="N22">
-        <v>1345403.355989266</v>
+        <v>617819.3854402569</v>
       </c>
       <c r="O22">
-        <v>645793.6108748474</v>
+        <v>296553.3050113234</v>
       </c>
       <c r="P22">
-        <v>360809.7825889013</v>
+        <v>0</v>
       </c>
       <c r="Q22">
         <v>0</v>
       </c>
       <c r="R22">
-        <v>360809.7825889013</v>
+        <v>0</v>
       </c>
       <c r="S22">
-        <v>173188.6956426727</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:19">
@@ -1734,58 +1734,58 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>0.4051684913538617</v>
+        <v>0.3484202269800509</v>
       </c>
       <c r="C23">
-        <v>0.3668482636862165</v>
+        <v>0.2492443660177321</v>
       </c>
       <c r="D23">
-        <v>-2642667.935405116</v>
+        <v>-4127180.565372506</v>
       </c>
       <c r="E23">
         <v>0</v>
       </c>
       <c r="F23">
-        <v>-2642667.935405116</v>
+        <v>-4127180.565372506</v>
       </c>
       <c r="G23">
-        <v>-2642667.935405116</v>
+        <v>-4127180.565372506</v>
       </c>
       <c r="H23">
-        <v>-3324731.298660469</v>
+        <v>-5753019.632758274</v>
       </c>
       <c r="I23">
-        <v>-625203.372204633</v>
+        <v>-1281907.356119556</v>
       </c>
       <c r="J23">
-        <v>-2699527.926455836</v>
+        <v>-4471112.276638718</v>
       </c>
       <c r="K23">
         <v>0</v>
       </c>
       <c r="L23">
-        <v>1065199.909062166</v>
+        <v>723719.0476208345</v>
       </c>
       <c r="M23">
         <v>0</v>
       </c>
       <c r="N23">
-        <v>1065199.909062166</v>
+        <v>723719.0476208347</v>
       </c>
       <c r="O23">
-        <v>511295.9563498397</v>
+        <v>347385.1428580006</v>
       </c>
       <c r="P23">
-        <v>285664.9241222081</v>
+        <v>0</v>
       </c>
       <c r="Q23">
         <v>0</v>
       </c>
       <c r="R23">
-        <v>285664.924122208</v>
+        <v>0</v>
       </c>
       <c r="S23">
-        <v>137119.1635786598</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:19">
@@ -1793,58 +1793,58 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0.4146177695208894</v>
+        <v>0.30230809422865</v>
       </c>
       <c r="C24">
-        <v>0.2901743485880965</v>
+        <v>0.5273749780437678</v>
       </c>
       <c r="D24">
-        <v>-3050566.297544352</v>
+        <v>-3040367.359236895</v>
       </c>
       <c r="E24">
         <v>0</v>
       </c>
       <c r="F24">
-        <v>-3050566.297544352</v>
+        <v>-3040367.359236895</v>
       </c>
       <c r="G24">
-        <v>-3050566.297544352</v>
+        <v>-3040367.359236895</v>
       </c>
       <c r="H24">
-        <v>-3995754.162596117</v>
+        <v>-4075580.009451914</v>
       </c>
       <c r="I24">
-        <v>-820192.445716145</v>
+        <v>-781848.7062924851</v>
       </c>
       <c r="J24">
-        <v>-3175561.716879972</v>
+        <v>-3293731.303159429</v>
       </c>
       <c r="K24">
         <v>0</v>
       </c>
       <c r="L24">
-        <v>842565.4973048931</v>
+        <v>1531313.718127297</v>
       </c>
       <c r="M24">
         <v>0</v>
       </c>
       <c r="N24">
-        <v>842565.4973048931</v>
+        <v>1531313.718127297</v>
       </c>
       <c r="O24">
-        <v>404431.4387063488</v>
+        <v>735030.5847011025</v>
       </c>
       <c r="P24">
-        <v>225958.908565346</v>
+        <v>0</v>
       </c>
       <c r="Q24">
         <v>0</v>
       </c>
       <c r="R24">
-        <v>225958.908565346</v>
+        <v>0</v>
       </c>
       <c r="S24">
-        <v>108460.2761113661</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:19">
@@ -1852,58 +1852,58 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>0.422727857061722</v>
+        <v>0.4833481498812586</v>
       </c>
       <c r="C25">
-        <v>0.5099555116669187</v>
+        <v>0.4003394824232875</v>
       </c>
       <c r="D25">
-        <v>-1587148.885008235</v>
+        <v>-2199511.446047037</v>
       </c>
       <c r="E25">
         <v>0</v>
       </c>
       <c r="F25">
-        <v>-1587148.885008235</v>
+        <v>-2199511.446047037</v>
       </c>
       <c r="G25">
-        <v>-1587148.885008235</v>
+        <v>-2199511.446047037</v>
       </c>
       <c r="H25">
-        <v>-1653811.8511676</v>
+        <v>-2939526.875956819</v>
       </c>
       <c r="I25">
-        <v>-161490.4271164532</v>
+        <v>-556722.8131237589</v>
       </c>
       <c r="J25">
-        <v>-1492321.424051146</v>
+        <v>-2382804.062833059</v>
       </c>
       <c r="K25">
         <v>0</v>
       </c>
       <c r="L25">
-        <v>1480733.639557258</v>
+        <v>1162446.772914364</v>
       </c>
       <c r="M25">
         <v>0</v>
       </c>
       <c r="N25">
-        <v>1480733.639557258</v>
+        <v>1162446.772914365</v>
       </c>
       <c r="O25">
-        <v>710752.1469874837</v>
+        <v>557974.4509988951</v>
       </c>
       <c r="P25">
-        <v>397102.6088067744</v>
+        <v>0</v>
       </c>
       <c r="Q25">
         <v>0</v>
       </c>
       <c r="R25">
-        <v>397102.6088067744</v>
+        <v>0</v>
       </c>
       <c r="S25">
-        <v>190609.2522272518</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:19">
@@ -1911,58 +1911,58 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0.4514005906228594</v>
+        <v>0.3318980347827936</v>
       </c>
       <c r="C26">
-        <v>0.2645228041110123</v>
+        <v>0.2215124189892858</v>
       </c>
       <c r="D26">
-        <v>-2905988.814329171</v>
+        <v>-4412086.044025646</v>
       </c>
       <c r="E26">
         <v>0</v>
       </c>
       <c r="F26">
-        <v>-2905988.814329171</v>
+        <v>-4412086.044025646</v>
       </c>
       <c r="G26">
-        <v>-2905988.814329171</v>
+        <v>-4412086.044025646</v>
       </c>
       <c r="H26">
-        <v>-3820471.417441091</v>
+        <v>-6171400.703036601</v>
       </c>
       <c r="I26">
-        <v>-790112.3390597637</v>
+        <v>-1391640.824360185</v>
       </c>
       <c r="J26">
-        <v>-3030359.078381327</v>
+        <v>-4779759.878676414</v>
       </c>
       <c r="K26">
         <v>0</v>
       </c>
       <c r="L26">
-        <v>768082.3238812733</v>
+        <v>643195.1079516395</v>
       </c>
       <c r="M26">
         <v>0</v>
       </c>
       <c r="N26">
-        <v>768082.3238812733</v>
+        <v>643195.1079516395</v>
       </c>
       <c r="O26">
-        <v>368679.5154630112</v>
+        <v>308733.651816787</v>
       </c>
       <c r="P26">
-        <v>205984.0382115053</v>
+        <v>0</v>
       </c>
       <c r="Q26">
         <v>0</v>
       </c>
       <c r="R26">
-        <v>205984.0382115053</v>
+        <v>0</v>
       </c>
       <c r="S26">
-        <v>98872.33834152254</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(engine): Propagate splitter uncertainty in MC simulation
  This commit fixes a bug where uncertainty defined for a Splitter process's material TC was not being applied during Monte Carlo simulations.

  The run_mc_simulation function has been modified to ensure that when a value is sampled for a ..._material TC, it is correctly propagated to the corresponding ..._WC, ..._DM, and ..._CC parameters used by
  the solver.

  Additionally, this commit adds documentation for a deeper, underlying bug related to inconsistent TC naming conventions between the data loader and the solver, which will need to be addressed in a future
  session.
</commit_message>
<xml_diff>
--- a/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
+++ b/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
@@ -14,15 +14,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>iteration</t>
   </si>
   <si>
-    <t>TC_03_04</t>
+    <t>TC_03_05_material</t>
   </si>
   <si>
-    <t>TC_03_05</t>
+    <t>TC_03_04_material</t>
+  </si>
+  <si>
+    <t>TC_05_06_material</t>
+  </si>
+  <si>
+    <t>TC_05_07_material</t>
+  </si>
+  <si>
+    <t>TC_05_09_material</t>
   </si>
   <si>
     <t>S_0_material_mc</t>
@@ -71,6 +80,18 @@
   </si>
   <si>
     <t>S_10_CC_mc</t>
+  </si>
+  <si>
+    <t>S_11_material_mc</t>
+  </si>
+  <si>
+    <t>S_11_WC_mc</t>
+  </si>
+  <si>
+    <t>S_11_DM_mc</t>
+  </si>
+  <si>
+    <t>S_11_CC_mc</t>
   </si>
 </sst>
 </file>
@@ -428,10 +449,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S26"/>
+  <dimension ref="A1:Z26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:26">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -489,1479 +510,2025 @@
       <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:26">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2">
-        <v>0.3300650954079945</v>
+        <v>0.7141179519131081</v>
       </c>
       <c r="C2">
-        <v>0.3300347479000214</v>
+        <v>0.374916472221994</v>
       </c>
       <c r="D2">
-        <v>-3852952.853344902</v>
+        <v>0.07035854270650752</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>0.3409304218260964</v>
       </c>
       <c r="F2">
-        <v>-3852952.853344902</v>
+        <v>0.5680991632037351</v>
       </c>
       <c r="G2">
-        <v>-3852952.853344902</v>
+        <v>-434413.4397508474</v>
       </c>
       <c r="H2">
-        <v>-5324747.412744758</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>-1150715.1574829</v>
+        <v>-434413.4397508474</v>
       </c>
       <c r="J2">
-        <v>-4174032.255261858</v>
+        <v>-644137.7360914743</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>92851.06920426589</v>
       </c>
       <c r="L2">
-        <v>958306.2487959826</v>
+        <v>828447.6871056301</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>-735596.6179013635</v>
       </c>
       <c r="N2">
-        <v>958306.2487959825</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <v>459986.9994220718</v>
+        <v>259551.7904839946</v>
       </c>
       <c r="P2">
         <v>0</v>
       </c>
       <c r="Q2">
-        <v>0</v>
+        <v>259551.7904839946</v>
       </c>
       <c r="R2">
-        <v>0</v>
+        <v>124584.8594239899</v>
       </c>
       <c r="S2">
+        <v>2204620.606525467</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>2204620.606525467</v>
+      </c>
+      <c r="V2">
+        <v>1140750.799546648</v>
+      </c>
+      <c r="W2">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X2">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:19">
+    <row r="3" spans="1:26">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3">
-        <v>0.535772198783161</v>
+        <v>0.6177241021928185</v>
       </c>
       <c r="C3">
-        <v>0.2552318785963185</v>
+        <v>0.1445432858772167</v>
       </c>
       <c r="D3">
-        <v>-2529416.36917831</v>
+        <v>0.2016764824454824</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>0.2702098473322121</v>
       </c>
       <c r="F3">
-        <v>-2529416.36917831</v>
+        <v>0.6735951032709135</v>
       </c>
       <c r="G3">
-        <v>-2529416.36917831</v>
+        <v>-2612238.988641692</v>
       </c>
       <c r="H3">
-        <v>-3477400.804963621</v>
+        <v>0</v>
       </c>
       <c r="I3">
-        <v>-737199.7421825835</v>
+        <v>-2612238.988641692</v>
       </c>
       <c r="J3">
-        <v>-2740201.062781036</v>
+        <v>-2714920.098999678</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>-2668906.908090111</v>
       </c>
       <c r="L3">
-        <v>741104.7039958478</v>
+        <v>198583.6569247001</v>
       </c>
       <c r="M3">
-        <v>0</v>
+        <v>-2867490.56501481</v>
       </c>
       <c r="N3">
-        <v>741104.7039958478</v>
+        <v>0</v>
       </c>
       <c r="O3">
-        <v>355730.2579180071</v>
+        <v>643557.0430995977</v>
       </c>
       <c r="P3">
         <v>0</v>
       </c>
       <c r="Q3">
-        <v>0</v>
+        <v>643557.0430995976</v>
       </c>
       <c r="R3">
-        <v>0</v>
+        <v>308907.3806671588</v>
       </c>
       <c r="S3">
+        <v>2261170.080690844</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <v>2261170.080690844</v>
+      </c>
+      <c r="V3">
+        <v>1170011.552021317</v>
+      </c>
+      <c r="W3">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X3">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y3">
+        <v>0</v>
+      </c>
+      <c r="Z3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:19">
+    <row r="4" spans="1:26">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.5896335647893132</v>
+        <v>0.8102403433131202</v>
       </c>
       <c r="C4">
-        <v>0.5280671019942949</v>
+        <v>0.1773769037443589</v>
       </c>
       <c r="D4">
-        <v>-634958.2927012753</v>
+        <v>0.3081927605365722</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>0.3914404303325235</v>
       </c>
       <c r="F4">
-        <v>-634958.2927012753</v>
+        <v>0.5352638396254494</v>
       </c>
       <c r="G4">
-        <v>-634958.2927012753</v>
+        <v>-185068.9408502296</v>
       </c>
       <c r="H4">
-        <v>-653605.0703298808</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>34266.40874902662</v>
+        <v>-185068.9408502296</v>
       </c>
       <c r="J4">
-        <v>-687871.4790789078</v>
+        <v>-351269.6840210815</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>759286.019129728</v>
       </c>
       <c r="L4">
-        <v>1533323.405625209</v>
+        <v>1122217.038413074</v>
       </c>
       <c r="M4">
-        <v>0</v>
+        <v>-362931.0192833458</v>
       </c>
       <c r="N4">
-        <v>1533323.405625209</v>
+        <v>0</v>
       </c>
       <c r="O4">
-        <v>735995.2347001006</v>
+        <v>1289951.96783017</v>
       </c>
       <c r="P4">
         <v>0</v>
       </c>
       <c r="Q4">
-        <v>0</v>
+        <v>1289951.96783017</v>
       </c>
       <c r="R4">
-        <v>0</v>
+        <v>619176.9445170942</v>
       </c>
       <c r="S4">
+        <v>2356793.495474354</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>2356793.495474354</v>
+      </c>
+      <c r="V4">
+        <v>1219490.58099655</v>
+      </c>
+      <c r="W4">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X4">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:19">
+    <row r="5" spans="1:26">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5">
-        <v>0.4093599894573831</v>
+        <v>0.6044427041784902</v>
       </c>
       <c r="C5">
-        <v>0.4731179237872294</v>
+        <v>0.3610353065805824</v>
       </c>
       <c r="D5">
-        <v>-2432729.22192007</v>
+        <v>-0.1846131332897333</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>0.3256859196937808</v>
       </c>
       <c r="F5">
-        <v>-2432729.22192007</v>
+        <v>0.6127851720596404</v>
       </c>
       <c r="G5">
-        <v>-2432729.22192007</v>
+        <v>-2107866.959007225</v>
       </c>
       <c r="H5">
-        <v>-3236873.173442998</v>
+        <v>0</v>
       </c>
       <c r="I5">
-        <v>-601416.5196933598</v>
+        <v>-2107866.959007225</v>
       </c>
       <c r="J5">
-        <v>-2635456.653749638</v>
+        <v>-2297015.866613362</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>-2422472.143054044</v>
       </c>
       <c r="L5">
-        <v>1373770.08229458</v>
+        <v>98126.68916577478</v>
       </c>
       <c r="M5">
-        <v>0</v>
+        <v>-2520598.832219819</v>
       </c>
       <c r="N5">
-        <v>1373770.08229458</v>
+        <v>0</v>
       </c>
       <c r="O5">
-        <v>659409.6395013983</v>
+        <v>-576441.150033399</v>
       </c>
       <c r="P5">
         <v>0</v>
       </c>
       <c r="Q5">
-        <v>0</v>
+        <v>-576441.150033399</v>
       </c>
       <c r="R5">
-        <v>0</v>
+        <v>-276691.7519975368</v>
       </c>
       <c r="S5">
+        <v>2012811.707469404</v>
+      </c>
+      <c r="T5">
+        <v>0</v>
+      </c>
+      <c r="U5">
+        <v>2012811.707469404</v>
+      </c>
+      <c r="V5">
+        <v>1041501.906421581</v>
+      </c>
+      <c r="W5">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X5">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y5">
+        <v>0</v>
+      </c>
+      <c r="Z5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:19">
+    <row r="6" spans="1:26">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6">
-        <v>0.5808678480067124</v>
+        <v>0.5887100173938941</v>
       </c>
       <c r="C6">
-        <v>0.4199853283774986</v>
+        <v>0.2385952869318479</v>
       </c>
       <c r="D6">
-        <v>-1280353.300105714</v>
+        <v>0.07506266536843578</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>0.3221149590456617</v>
       </c>
       <c r="F6">
-        <v>-1280353.300105714</v>
+        <v>0.6842810901233787</v>
       </c>
       <c r="G6">
-        <v>-1280353.300105714</v>
+        <v>-2141474.880288031</v>
       </c>
       <c r="H6">
-        <v>-1622755.878132736</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <v>-235706.4741156322</v>
+        <v>-2141474.880288031</v>
       </c>
       <c r="J6">
-        <v>-1387049.404017104</v>
+        <v>-2285010.212392238</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <v>-2184081.683276666</v>
       </c>
       <c r="L6">
-        <v>1219491.484298837</v>
+        <v>264144.3278319714</v>
       </c>
       <c r="M6">
-        <v>0</v>
+        <v>-2448226.011108636</v>
       </c>
       <c r="N6">
-        <v>1219491.484298837</v>
+        <v>0</v>
       </c>
       <c r="O6">
-        <v>585355.9124634417</v>
+        <v>228277.2594646938</v>
       </c>
       <c r="P6">
         <v>0</v>
       </c>
       <c r="Q6">
-        <v>0</v>
+        <v>228277.2594646938</v>
       </c>
       <c r="R6">
-        <v>0</v>
+        <v>109573.084535729</v>
       </c>
       <c r="S6">
+        <v>2189151.038929578</v>
+      </c>
+      <c r="T6">
+        <v>0</v>
+      </c>
+      <c r="U6">
+        <v>2189151.038929578</v>
+      </c>
+      <c r="V6">
+        <v>1132746.283236033</v>
+      </c>
+      <c r="W6">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X6">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y6">
+        <v>0</v>
+      </c>
+      <c r="Z6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:19">
+    <row r="7" spans="1:26">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7">
-        <v>0.3705541202939737</v>
+        <v>0.6964751788088929</v>
       </c>
       <c r="C7">
-        <v>0.4317885854590039</v>
+        <v>0.2123895539991836</v>
       </c>
       <c r="D7">
-        <v>-2975880.071387835</v>
+        <v>-0.07486926793711637</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>0.4708386090452701</v>
       </c>
       <c r="F7">
-        <v>-2975880.071387835</v>
+        <v>0.6368329858912428</v>
       </c>
       <c r="G7">
-        <v>-2975880.071387835</v>
+        <v>-1506699.523575195</v>
       </c>
       <c r="H7">
-        <v>-4029030.597618576</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>-805160.5232699048</v>
+        <v>-1506699.523575195</v>
       </c>
       <c r="J7">
-        <v>-3223870.074348671</v>
+        <v>-1688707.564073909</v>
       </c>
       <c r="K7">
-        <v>0</v>
+        <v>-1399280.976434355</v>
       </c>
       <c r="L7">
-        <v>1253764.042231975</v>
+        <v>424175.3411029846</v>
       </c>
       <c r="M7">
-        <v>0</v>
+        <v>-1823456.317537338</v>
       </c>
       <c r="N7">
-        <v>1253764.042231975</v>
+        <v>0</v>
       </c>
       <c r="O7">
-        <v>601806.740271348</v>
+        <v>-269368.2922749965</v>
       </c>
       <c r="P7">
         <v>0</v>
       </c>
       <c r="Q7">
-        <v>0</v>
+        <v>-269368.2922749965</v>
       </c>
       <c r="R7">
-        <v>0</v>
+        <v>-129296.7802833559</v>
       </c>
       <c r="S7">
+        <v>2410299.196485533</v>
+      </c>
+      <c r="T7">
+        <v>0</v>
+      </c>
+      <c r="U7">
+        <v>2410299.196485533</v>
+      </c>
+      <c r="V7">
+        <v>1247176.374655624</v>
+      </c>
+      <c r="W7">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X7">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y7">
+        <v>0</v>
+      </c>
+      <c r="Z7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:19">
+    <row r="8" spans="1:26">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0.3534558264935208</v>
+        <v>0.6123830520681541</v>
       </c>
       <c r="C8">
-        <v>0.4164929836432453</v>
+        <v>0.1164101283602635</v>
       </c>
       <c r="D8">
-        <v>-3199770.32111614</v>
+        <v>-0.1013501714714783</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>0.4131514059166311</v>
       </c>
       <c r="F8">
-        <v>-3199770.32111614</v>
+        <v>0.5002309783041522</v>
       </c>
       <c r="G8">
-        <v>-3199770.32111614</v>
+        <v>-3812275.953032149</v>
       </c>
       <c r="H8">
-        <v>-4354740.180671622</v>
+        <v>0</v>
       </c>
       <c r="I8">
-        <v>-888322.3356382377</v>
+        <v>-3812275.953032149</v>
       </c>
       <c r="J8">
-        <v>-3466417.845033383</v>
+        <v>-3936672.676231652</v>
       </c>
       <c r="K8">
-        <v>0</v>
+        <v>-4736695.579572173</v>
       </c>
       <c r="L8">
-        <v>1209350.928484397</v>
+        <v>-477403.2629380559</v>
       </c>
       <c r="M8">
-        <v>0</v>
+        <v>-4259292.316634117</v>
       </c>
       <c r="N8">
-        <v>1209350.928484397</v>
+        <v>0</v>
       </c>
       <c r="O8">
-        <v>580488.4456725108</v>
+        <v>-320615.7799684128</v>
       </c>
       <c r="P8">
         <v>0</v>
       </c>
       <c r="Q8">
-        <v>0</v>
+        <v>-320615.7799684129</v>
       </c>
       <c r="R8">
-        <v>0</v>
+        <v>-153895.5743745515</v>
       </c>
       <c r="S8">
+        <v>1664690.527306251</v>
+      </c>
+      <c r="T8">
+        <v>0</v>
+      </c>
+      <c r="U8">
+        <v>1664690.527306252</v>
+      </c>
+      <c r="V8">
+        <v>861371.3599525866</v>
+      </c>
+      <c r="W8">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X8">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y8">
+        <v>0</v>
+      </c>
+      <c r="Z8">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:19">
+    <row r="9" spans="1:26">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0.4789835713222546</v>
+        <v>0.6179192900934228</v>
       </c>
       <c r="C9">
-        <v>0.4931469555338494</v>
+        <v>0.3573044668541085</v>
       </c>
       <c r="D9">
-        <v>-1744725.546290438</v>
+        <v>0.1142304910926777</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>0.3906353697813118</v>
       </c>
       <c r="F9">
-        <v>-1744725.546290438</v>
+        <v>0.4760089254042782</v>
       </c>
       <c r="G9">
-        <v>-1744725.546290438</v>
+        <v>-1103564.424055048</v>
       </c>
       <c r="H9">
-        <v>-2248733.802715405</v>
+        <v>0</v>
       </c>
       <c r="I9">
-        <v>-358614.4647506431</v>
+        <v>-1103564.424055048</v>
       </c>
       <c r="J9">
-        <v>-1890119.337964762</v>
+        <v>-1307983.134662195</v>
       </c>
       <c r="K9">
-        <v>0</v>
+        <v>-982708.4126058645</v>
       </c>
       <c r="L9">
-        <v>1431927.432095618</v>
+        <v>514028.7151682488</v>
       </c>
       <c r="M9">
-        <v>0</v>
+        <v>-1496737.127774113</v>
       </c>
       <c r="N9">
-        <v>1431927.432095618</v>
+        <v>0</v>
       </c>
       <c r="O9">
-        <v>687325.1674058971</v>
+        <v>364628.8601584958</v>
       </c>
       <c r="P9">
         <v>0</v>
       </c>
       <c r="Q9">
-        <v>0</v>
+        <v>364628.8601584957</v>
       </c>
       <c r="R9">
-        <v>0</v>
+        <v>175021.8528643792</v>
       </c>
       <c r="S9">
+        <v>1598404.197223871</v>
+      </c>
+      <c r="T9">
+        <v>0</v>
+      </c>
+      <c r="U9">
+        <v>1598404.197223871</v>
+      </c>
+      <c r="V9">
+        <v>827072.4044694201</v>
+      </c>
+      <c r="W9">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X9">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y9">
+        <v>0</v>
+      </c>
+      <c r="Z9">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:19">
+    <row r="10" spans="1:26">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0.5160107829338383</v>
+        <v>0.8138550452656408</v>
       </c>
       <c r="C10">
-        <v>0.3445286318531346</v>
+        <v>0.3352445567359655</v>
       </c>
       <c r="D10">
-        <v>-2221915.918403574</v>
+        <v>0.244333117682454</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>0.3236842350196596</v>
       </c>
       <c r="F10">
-        <v>-2221915.918403574</v>
+        <v>0.541328059176166</v>
       </c>
       <c r="G10">
-        <v>-2221915.918403574</v>
+        <v>460692.7511133614</v>
       </c>
       <c r="H10">
-        <v>-2997777.902377266</v>
+        <v>0</v>
       </c>
       <c r="I10">
-        <v>-590702.3279542439</v>
+        <v>460692.7511133614</v>
       </c>
       <c r="J10">
-        <v>-2407075.574423022</v>
+        <v>258317.1443522025</v>
       </c>
       <c r="K10">
-        <v>0</v>
+        <v>1556931.030423219</v>
       </c>
       <c r="L10">
-        <v>1000391.452399452</v>
+        <v>1292739.37854013</v>
       </c>
       <c r="M10">
-        <v>0</v>
+        <v>264191.6518830899</v>
       </c>
       <c r="N10">
-        <v>1000391.452399452</v>
+        <v>0</v>
       </c>
       <c r="O10">
-        <v>480187.897151737</v>
+        <v>1027227.504948739</v>
       </c>
       <c r="P10">
         <v>0</v>
       </c>
       <c r="Q10">
-        <v>0</v>
+        <v>1027227.504948739</v>
       </c>
       <c r="R10">
-        <v>0</v>
+        <v>493069.2023424371</v>
       </c>
       <c r="S10">
+        <v>2394127.97364834</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+      <c r="U10">
+        <v>2394127.97364834</v>
+      </c>
+      <c r="V10">
+        <v>1238808.796430794</v>
+      </c>
+      <c r="W10">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X10">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y10">
+        <v>0</v>
+      </c>
+      <c r="Z10">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:19">
+    <row r="11" spans="1:26">
       <c r="A11">
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0.4445391346994594</v>
+        <v>0.6427484954260548</v>
       </c>
       <c r="C11">
-        <v>0.45465360696859</v>
+        <v>0.3963787674379488</v>
       </c>
       <c r="D11">
-        <v>-2236407.210642167</v>
+        <v>0.0756309022106509</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>0.4534701178075405</v>
       </c>
       <c r="F11">
-        <v>-2236407.210642167</v>
+        <v>0.5871522425730369</v>
       </c>
       <c r="G11">
-        <v>-2236407.210642167</v>
+        <v>4256.847531574487</v>
       </c>
       <c r="H11">
-        <v>-2966336.771248278</v>
+        <v>0</v>
       </c>
       <c r="I11">
-        <v>-543562.2965954929</v>
+        <v>4256.847531574487</v>
       </c>
       <c r="J11">
-        <v>-2422774.474652785</v>
+        <v>-230055.6903586425</v>
       </c>
       <c r="K11">
-        <v>0</v>
+        <v>616933.0482691182</v>
       </c>
       <c r="L11">
-        <v>1320156.121038564</v>
+        <v>940522.819655643</v>
       </c>
       <c r="M11">
-        <v>0</v>
+        <v>-323589.7713865239</v>
       </c>
       <c r="N11">
-        <v>1320156.121038564</v>
+        <v>0</v>
       </c>
       <c r="O11">
-        <v>633674.9380985106</v>
+        <v>251117.8547800418</v>
       </c>
       <c r="P11">
         <v>0</v>
       </c>
       <c r="Q11">
-        <v>0</v>
+        <v>251117.8547800418</v>
       </c>
       <c r="R11">
-        <v>0</v>
+        <v>120536.5702863632</v>
       </c>
       <c r="S11">
+        <v>2050838.939159638</v>
+      </c>
+      <c r="T11">
+        <v>0</v>
+      </c>
+      <c r="U11">
+        <v>2050838.939159638</v>
+      </c>
+      <c r="V11">
+        <v>1061178.577694081</v>
+      </c>
+      <c r="W11">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X11">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y11">
+        <v>0</v>
+      </c>
+      <c r="Z11">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:19">
+    <row r="12" spans="1:26">
       <c r="A12">
         <v>10</v>
       </c>
       <c r="B12">
-        <v>0.3913670061184192</v>
+        <v>0.5254224560371819</v>
       </c>
       <c r="C12">
-        <v>0.3826027136110881</v>
+        <v>0.2508611022124017</v>
       </c>
       <c r="D12">
-        <v>-3062267.420674835</v>
+        <v>0.1261928241121761</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>0.4211961554644648</v>
       </c>
       <c r="F12">
-        <v>-3062267.420674835</v>
+        <v>0.8184149956952312</v>
       </c>
       <c r="G12">
-        <v>-3062267.420674835</v>
+        <v>-1478524.938687313</v>
       </c>
       <c r="H12">
-        <v>-4175164.481002862</v>
+        <v>0</v>
       </c>
       <c r="I12">
-        <v>-857708.1116520369</v>
+        <v>-1478524.938687313</v>
       </c>
       <c r="J12">
-        <v>-3317456.369350824</v>
+        <v>-1636985.426943052</v>
       </c>
       <c r="K12">
-        <v>0</v>
+        <v>-1221180.615218635</v>
       </c>
       <c r="L12">
-        <v>1110945.358307775</v>
+        <v>528428.0314906929</v>
       </c>
       <c r="M12">
-        <v>0</v>
+        <v>-1749608.646709326</v>
       </c>
       <c r="N12">
-        <v>1110945.358307775</v>
+        <v>0</v>
       </c>
       <c r="O12">
-        <v>533253.771987732</v>
+        <v>342515.7390067143</v>
       </c>
       <c r="P12">
         <v>0</v>
       </c>
       <c r="Q12">
-        <v>0</v>
+        <v>342515.7390067142</v>
       </c>
       <c r="R12">
-        <v>0</v>
+        <v>164407.5547122335</v>
       </c>
       <c r="S12">
+        <v>2336802.295350139</v>
+      </c>
+      <c r="T12">
+        <v>0</v>
+      </c>
+      <c r="U12">
+        <v>2336802.295350139</v>
+      </c>
+      <c r="V12">
+        <v>1209146.407736945</v>
+      </c>
+      <c r="W12">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X12">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y12">
+        <v>0</v>
+      </c>
+      <c r="Z12">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:19">
+    <row r="13" spans="1:26">
       <c r="A13">
         <v>11</v>
       </c>
       <c r="B13">
-        <v>0.5752409098045101</v>
+        <v>0.6882821311920075</v>
       </c>
       <c r="C13">
-        <v>0.5700569717931837</v>
+        <v>0.3369440738919695</v>
       </c>
       <c r="D13">
-        <v>-532995.906594994</v>
+        <v>0.06260921038024125</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>0.4519542059537509</v>
       </c>
       <c r="F13">
-        <v>-532995.906594994</v>
+        <v>0.5165762246018797</v>
       </c>
       <c r="G13">
-        <v>-532995.906594994</v>
+        <v>-495850.1466884732</v>
       </c>
       <c r="H13">
-        <v>-488717.460066537</v>
+        <v>0</v>
       </c>
       <c r="I13">
-        <v>88694.76742391619</v>
+        <v>-495850.1466884732</v>
       </c>
       <c r="J13">
-        <v>-577412.227490453</v>
+        <v>-716594.5820794145</v>
       </c>
       <c r="K13">
-        <v>0</v>
+        <v>-96317.43367610761</v>
       </c>
       <c r="L13">
-        <v>1655247.399599912</v>
+        <v>750044.9232714865</v>
       </c>
       <c r="M13">
-        <v>0</v>
+        <v>-846362.3569475936</v>
       </c>
       <c r="N13">
-        <v>1655247.399599912</v>
+        <v>0</v>
       </c>
       <c r="O13">
-        <v>794518.751807958</v>
+        <v>222608.6132099074</v>
       </c>
       <c r="P13">
         <v>0</v>
       </c>
       <c r="Q13">
-        <v>0</v>
+        <v>222608.6132099074</v>
       </c>
       <c r="R13">
-        <v>0</v>
+        <v>106852.1343336134</v>
       </c>
       <c r="S13">
+        <v>1932149.250401899</v>
+      </c>
+      <c r="T13">
+        <v>0</v>
+      </c>
+      <c r="U13">
+        <v>1932149.250401899</v>
+      </c>
+      <c r="V13">
+        <v>999764.2205264227</v>
+      </c>
+      <c r="W13">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X13">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y13">
+        <v>0</v>
+      </c>
+      <c r="Z13">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:19">
+    <row r="14" spans="1:26">
       <c r="A14">
         <v>12</v>
       </c>
       <c r="B14">
-        <v>0.386708424313029</v>
+        <v>0.6362147722545036</v>
       </c>
       <c r="C14">
-        <v>0.3963616530678007</v>
+        <v>0.1600828673581693</v>
       </c>
       <c r="D14">
-        <v>-3028376.474733957</v>
+        <v>0.1418184838874653</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>0.07463464304140394</v>
       </c>
       <c r="F14">
-        <v>-3028376.474733957</v>
+        <v>0.5404204305804412</v>
       </c>
       <c r="G14">
-        <v>-3028376.474733957</v>
+        <v>-4118725.111540099</v>
       </c>
       <c r="H14">
-        <v>-4120451.586719099</v>
+        <v>0</v>
       </c>
       <c r="I14">
-        <v>-839710.4087958848</v>
+        <v>-4118725.111540099</v>
       </c>
       <c r="J14">
-        <v>-3280741.177923216</v>
+        <v>-4186228.538582548</v>
       </c>
       <c r="K14">
-        <v>0</v>
+        <v>-4855079.498544795</v>
       </c>
       <c r="L14">
-        <v>1150896.538424626</v>
+        <v>-398217.8916208389</v>
       </c>
       <c r="M14">
-        <v>0</v>
+        <v>-4456861.606923957</v>
       </c>
       <c r="N14">
-        <v>1150896.538424626</v>
+        <v>0</v>
       </c>
       <c r="O14">
-        <v>552430.3384438206</v>
+        <v>466094.3407023191</v>
       </c>
       <c r="P14">
         <v>0</v>
       </c>
       <c r="Q14">
-        <v>0</v>
+        <v>466094.3407023191</v>
       </c>
       <c r="R14">
-        <v>0</v>
+        <v>223725.2835221589</v>
       </c>
       <c r="S14">
+        <v>1868423.280797676</v>
+      </c>
+      <c r="T14">
+        <v>0</v>
+      </c>
+      <c r="U14">
+        <v>1868423.280797676</v>
+      </c>
+      <c r="V14">
+        <v>966790.0885770387</v>
+      </c>
+      <c r="W14">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X14">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y14">
+        <v>0</v>
+      </c>
+      <c r="Z14">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:19">
+    <row r="15" spans="1:26">
       <c r="A15">
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0.3086713916747138</v>
+        <v>0.7142450004253041</v>
       </c>
       <c r="C15">
-        <v>0.346022001402262</v>
+        <v>0.2622900613890503</v>
       </c>
       <c r="D15">
-        <v>-3947154.900646711</v>
+        <v>0.1353447938348827</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>0.5939559175622413</v>
       </c>
       <c r="F15">
-        <v>-3947154.900646711</v>
+        <v>0.5559141205633831</v>
       </c>
       <c r="G15">
-        <v>-3947154.900646711</v>
+        <v>384086.1212140897</v>
       </c>
       <c r="H15">
-        <v>-5451191.022441128</v>
+        <v>0</v>
       </c>
       <c r="I15">
-        <v>-1175106.549148097</v>
+        <v>384086.1212140897</v>
       </c>
       <c r="J15">
-        <v>-4276084.473293031</v>
+        <v>150509.3831051205</v>
       </c>
       <c r="K15">
-        <v>0</v>
+        <v>1226520.734728328</v>
       </c>
       <c r="L15">
-        <v>1004727.678750757</v>
+        <v>1128760.129812818</v>
       </c>
       <c r="M15">
-        <v>0</v>
+        <v>97760.60491551121</v>
       </c>
       <c r="N15">
-        <v>1004727.678750757</v>
+        <v>0</v>
       </c>
       <c r="O15">
-        <v>482269.2858003636</v>
+        <v>499374.0917304266</v>
       </c>
       <c r="P15">
         <v>0</v>
       </c>
       <c r="Q15">
-        <v>0</v>
+        <v>499374.0917304265</v>
       </c>
       <c r="R15">
-        <v>0</v>
+        <v>239699.5640145827</v>
       </c>
       <c r="S15">
+        <v>2157717.961180991</v>
+      </c>
+      <c r="T15">
+        <v>0</v>
+      </c>
+      <c r="U15">
+        <v>2157717.961180992</v>
+      </c>
+      <c r="V15">
+        <v>1116481.666790111</v>
+      </c>
+      <c r="W15">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X15">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y15">
+        <v>0</v>
+      </c>
+      <c r="Z15">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:19">
+    <row r="16" spans="1:26">
       <c r="A16">
         <v>14</v>
       </c>
       <c r="B16">
-        <v>0.344784598808699</v>
+        <v>0.6780465418980448</v>
       </c>
       <c r="C16">
-        <v>0.5331005753838244</v>
+        <v>0.07892074904412297</v>
       </c>
       <c r="D16">
-        <v>-2654999.46347141</v>
+        <v>0.05964668648771772</v>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>0.5110603062864235</v>
       </c>
       <c r="F16">
-        <v>-2654999.46347141</v>
+        <v>0.6867643358631997</v>
       </c>
       <c r="G16">
-        <v>-2654999.46347141</v>
+        <v>-1840181.173702325</v>
       </c>
       <c r="H16">
-        <v>-3524695.22705815</v>
+        <v>0</v>
       </c>
       <c r="I16">
-        <v>-648445.8112835408</v>
+        <v>-1840181.173702325</v>
       </c>
       <c r="J16">
-        <v>-2876249.415774608</v>
+        <v>-1981871.691407186</v>
       </c>
       <c r="K16">
-        <v>0</v>
+        <v>-1667653.207210434</v>
       </c>
       <c r="L16">
-        <v>1547938.863642968</v>
+        <v>423705.0149766456</v>
       </c>
       <c r="M16">
-        <v>0</v>
+        <v>-2091358.222187079</v>
       </c>
       <c r="N16">
-        <v>1547938.863642968</v>
+        <v>0</v>
       </c>
       <c r="O16">
-        <v>743010.6545486248</v>
+        <v>208921.4689550902</v>
       </c>
       <c r="P16">
         <v>0</v>
       </c>
       <c r="Q16">
-        <v>0</v>
+        <v>208921.4689550902</v>
       </c>
       <c r="R16">
-        <v>0</v>
+        <v>100282.3050917402</v>
       </c>
       <c r="S16">
+        <v>2530503.843818405</v>
+      </c>
+      <c r="T16">
+        <v>0</v>
+      </c>
+      <c r="U16">
+        <v>2530503.843818405</v>
+      </c>
+      <c r="V16">
+        <v>1309374.626431155</v>
+      </c>
+      <c r="W16">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X16">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y16">
+        <v>0</v>
+      </c>
+      <c r="Z16">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:19">
+    <row r="17" spans="1:26">
       <c r="A17">
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0.5174019413933307</v>
+        <v>0.7097125435755307</v>
       </c>
       <c r="C17">
-        <v>0.3390526731520805</v>
+        <v>0.2235076219758375</v>
       </c>
       <c r="D17">
-        <v>-2239273.834868472</v>
+        <v>0.1168051118687917</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>0.1674700882488548</v>
       </c>
       <c r="F17">
-        <v>-2239273.834868472</v>
+        <v>0.4694144994317876</v>
       </c>
       <c r="G17">
-        <v>-2239273.834868472</v>
+        <v>-3047166.171590806</v>
       </c>
       <c r="H17">
-        <v>-3025057.620095644</v>
+        <v>0</v>
       </c>
       <c r="I17">
-        <v>-599177.6361690817</v>
+        <v>-3047166.171590806</v>
       </c>
       <c r="J17">
-        <v>-2425879.983926562</v>
+        <v>-3161766.717345882</v>
       </c>
       <c r="K17">
-        <v>0</v>
+        <v>-3465766.044967825</v>
       </c>
       <c r="L17">
-        <v>984491.1707631727</v>
+        <v>-67116.95283861135</v>
       </c>
       <c r="M17">
-        <v>0</v>
+        <v>-3398649.092129212</v>
       </c>
       <c r="N17">
-        <v>984491.1707631727</v>
+        <v>0</v>
       </c>
       <c r="O17">
-        <v>472555.761966323</v>
+        <v>428234.422090029</v>
       </c>
       <c r="P17">
         <v>0</v>
       </c>
       <c r="Q17">
-        <v>0</v>
+        <v>428234.422090029</v>
       </c>
       <c r="R17">
-        <v>0</v>
+        <v>205552.5225894745</v>
       </c>
       <c r="S17">
+        <v>1810417.517988091</v>
+      </c>
+      <c r="T17">
+        <v>0</v>
+      </c>
+      <c r="U17">
+        <v>1810417.517988092</v>
+      </c>
+      <c r="V17">
+        <v>936775.7994483376</v>
+      </c>
+      <c r="W17">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X17">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y17">
+        <v>0</v>
+      </c>
+      <c r="Z17">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:19">
+    <row r="18" spans="1:26">
       <c r="A18">
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0.5779434757922117</v>
+        <v>0.5683946983950449</v>
       </c>
       <c r="C18">
-        <v>0.5180519784968147</v>
+        <v>0.3200476205441926</v>
       </c>
       <c r="D18">
-        <v>-785689.7041265869</v>
+        <v>0.1537223367781242</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>0.3932938930368052</v>
       </c>
       <c r="F18">
-        <v>-785689.7041265869</v>
+        <v>0.4669042689686214</v>
       </c>
       <c r="G18">
-        <v>-785689.7041265869</v>
+        <v>-1643623.716202915</v>
       </c>
       <c r="H18">
-        <v>-872751.606921935</v>
+        <v>0</v>
       </c>
       <c r="I18">
-        <v>-21587.76536675355</v>
+        <v>-1643623.716202915</v>
       </c>
       <c r="J18">
-        <v>-851163.8415551813</v>
+        <v>-1829254.996020293</v>
       </c>
       <c r="K18">
-        <v>0</v>
+        <v>-1730902.061786955</v>
       </c>
       <c r="L18">
-        <v>1504242.966395198</v>
+        <v>323943.5892243154</v>
       </c>
       <c r="M18">
-        <v>0</v>
+        <v>-2054845.65101127</v>
       </c>
       <c r="N18">
-        <v>1504242.966395198</v>
+        <v>0</v>
       </c>
       <c r="O18">
-        <v>722036.6238696952</v>
+        <v>451361.2161027352</v>
       </c>
       <c r="P18">
         <v>0</v>
       </c>
       <c r="Q18">
-        <v>0</v>
+        <v>451361.2161027352</v>
       </c>
       <c r="R18">
-        <v>0</v>
+        <v>216653.3837148313</v>
       </c>
       <c r="S18">
+        <v>1442173.879267625</v>
+      </c>
+      <c r="T18">
+        <v>0</v>
+      </c>
+      <c r="U18">
+        <v>1442173.879267625</v>
+      </c>
+      <c r="V18">
+        <v>746233.1618376032</v>
+      </c>
+      <c r="W18">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X18">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y18">
+        <v>0</v>
+      </c>
+      <c r="Z18">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:19">
+    <row r="19" spans="1:26">
       <c r="A19">
         <v>17</v>
       </c>
       <c r="B19">
-        <v>0.5354723691847816</v>
+        <v>0.6351630365280596</v>
       </c>
       <c r="C19">
-        <v>0.5893501048511529</v>
+        <v>0.1606756796910299</v>
       </c>
       <c r="D19">
-        <v>-763293.2664984402</v>
+        <v>0.1086813004205811</v>
       </c>
       <c r="E19">
-        <v>0</v>
+        <v>0.3333399296385667</v>
       </c>
       <c r="F19">
-        <v>-763293.2664984402</v>
+        <v>0.6195483612853996</v>
       </c>
       <c r="G19">
-        <v>-763293.2664984402</v>
+        <v>-2533145.806286952</v>
       </c>
       <c r="H19">
-        <v>-807191.3660601664</v>
+        <v>0</v>
       </c>
       <c r="I19">
-        <v>19709.66823529205</v>
+        <v>-2533145.806286952</v>
       </c>
       <c r="J19">
-        <v>-826901.0342954585</v>
+        <v>-2657367.194674403</v>
       </c>
       <c r="K19">
-        <v>0</v>
+        <v>-2686399.435611576</v>
       </c>
       <c r="L19">
-        <v>1711267.955271539</v>
+        <v>149853.237318019</v>
       </c>
       <c r="M19">
-        <v>0</v>
+        <v>-2836252.672929594</v>
       </c>
       <c r="N19">
-        <v>1711267.955271539</v>
+        <v>0</v>
       </c>
       <c r="O19">
-        <v>821408.6185303386</v>
+        <v>356596.671704758</v>
       </c>
       <c r="P19">
         <v>0</v>
       </c>
       <c r="Q19">
-        <v>0</v>
+        <v>356596.671704758</v>
       </c>
       <c r="R19">
-        <v>0</v>
+        <v>171166.4024068427</v>
       </c>
       <c r="S19">
+        <v>2138455.370531241</v>
+      </c>
+      <c r="T19">
+        <v>0</v>
+      </c>
+      <c r="U19">
+        <v>2138455.370531241</v>
+      </c>
+      <c r="V19">
+        <v>1106514.502544253</v>
+      </c>
+      <c r="W19">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X19">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y19">
+        <v>0</v>
+      </c>
+      <c r="Z19">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:19">
+    <row r="20" spans="1:26">
       <c r="A20">
         <v>18</v>
       </c>
       <c r="B20">
-        <v>0.3476537348303897</v>
+        <v>0.7457619464381012</v>
       </c>
       <c r="C20">
-        <v>0.4947783044710695</v>
+        <v>0.310949715259784</v>
       </c>
       <c r="D20">
-        <v>-2833872.45860434</v>
+        <v>0.2669035037321189</v>
       </c>
       <c r="E20">
-        <v>0</v>
+        <v>0.4320807574704697</v>
       </c>
       <c r="F20">
-        <v>-2833872.45860434</v>
+        <v>0.5557140615725582</v>
       </c>
       <c r="G20">
-        <v>-2833872.45860434</v>
+        <v>617666.4597114507</v>
       </c>
       <c r="H20">
-        <v>-3797253.059520672</v>
+        <v>0</v>
       </c>
       <c r="I20">
-        <v>-727224.5656383124</v>
+        <v>617666.4597114507</v>
       </c>
       <c r="J20">
-        <v>-3070028.493882359</v>
+        <v>402909.8983927293</v>
       </c>
       <c r="K20">
-        <v>0</v>
+        <v>1714397.909637007</v>
       </c>
       <c r="L20">
-        <v>1436664.3026538</v>
+        <v>1317020.663511372</v>
       </c>
       <c r="M20">
-        <v>0</v>
+        <v>397377.2461256354</v>
       </c>
       <c r="N20">
-        <v>1436664.3026538</v>
+        <v>0</v>
       </c>
       <c r="O20">
-        <v>689598.8652738243</v>
+        <v>1028233.4708773</v>
       </c>
       <c r="P20">
         <v>0</v>
       </c>
       <c r="Q20">
-        <v>0</v>
+        <v>1028233.4708773</v>
       </c>
       <c r="R20">
-        <v>0</v>
+        <v>493552.065988114</v>
       </c>
       <c r="S20">
+        <v>2252119.170180423</v>
+      </c>
+      <c r="T20">
+        <v>0</v>
+      </c>
+      <c r="U20">
+        <v>2252119.170180423</v>
+      </c>
+      <c r="V20">
+        <v>1165328.282087784</v>
+      </c>
+      <c r="W20">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X20">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y20">
+        <v>0</v>
+      </c>
+      <c r="Z20">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:19">
+    <row r="21" spans="1:26">
       <c r="A21">
         <v>19</v>
       </c>
       <c r="B21">
-        <v>0.5894698208136384</v>
+        <v>0.7086600720627274</v>
       </c>
       <c r="C21">
-        <v>0.3409154809448693</v>
+        <v>0.06153079875539469</v>
       </c>
       <c r="D21">
-        <v>-1626999.868301982</v>
+        <v>0.1573991775603775</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>0.2634078471567534</v>
       </c>
       <c r="F21">
-        <v>-1626999.868301982</v>
+        <v>0.7073829014592595</v>
       </c>
       <c r="G21">
-        <v>-1626999.868301982</v>
+        <v>-2768309.341268966</v>
       </c>
       <c r="H21">
-        <v>-2153229.242228498</v>
+        <v>0</v>
       </c>
       <c r="I21">
-        <v>-390646.0559203024</v>
+        <v>-2768309.341268966</v>
       </c>
       <c r="J21">
-        <v>-1762583.186308196</v>
+        <v>-2847770.30138173</v>
       </c>
       <c r="K21">
-        <v>0</v>
+        <v>-2728269.817436323</v>
       </c>
       <c r="L21">
-        <v>989900.1174255891</v>
+        <v>223812.1346805051</v>
       </c>
       <c r="M21">
-        <v>0</v>
+        <v>-2952081.952116827</v>
       </c>
       <c r="N21">
-        <v>989900.1174255894</v>
+        <v>0</v>
       </c>
       <c r="O21">
-        <v>475152.0563642829</v>
+        <v>576205.8531964117</v>
       </c>
       <c r="P21">
         <v>0</v>
       </c>
       <c r="Q21">
-        <v>0</v>
+        <v>576205.8531964117</v>
       </c>
       <c r="R21">
-        <v>0</v>
+        <v>276578.8095157906</v>
       </c>
       <c r="S21">
+        <v>2724157.945605551</v>
+      </c>
+      <c r="T21">
+        <v>0</v>
+      </c>
+      <c r="U21">
+        <v>2724157.945605551</v>
+      </c>
+      <c r="V21">
+        <v>1409578.294488734</v>
+      </c>
+      <c r="W21">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X21">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y21">
+        <v>0</v>
+      </c>
+      <c r="Z21">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:19">
+    <row r="22" spans="1:26">
       <c r="A22">
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0.3924347186545817</v>
+        <v>0.6562918516087181</v>
       </c>
       <c r="C22">
-        <v>0.2127731770273897</v>
+        <v>0.1356517054263593</v>
       </c>
       <c r="D22">
-        <v>-3952322.152525235</v>
+        <v>-0.01965174861438668</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>0.382360731142212</v>
       </c>
       <c r="F22">
-        <v>-3952322.152525235</v>
+        <v>0.7081164691966496</v>
       </c>
       <c r="G22">
-        <v>-3952322.152525235</v>
+        <v>-2497210.727842766</v>
       </c>
       <c r="H22">
-        <v>-5521526.409101821</v>
+        <v>0</v>
       </c>
       <c r="I22">
-        <v>-1239844.079956746</v>
+        <v>-2497210.727842766</v>
       </c>
       <c r="J22">
-        <v>-4281682.329145076</v>
+        <v>-2625382.559819886</v>
       </c>
       <c r="K22">
-        <v>0</v>
+        <v>-2615649.691032325</v>
       </c>
       <c r="L22">
-        <v>617819.385440257</v>
+        <v>159719.5585179308</v>
       </c>
       <c r="M22">
-        <v>0</v>
+        <v>-2775369.249550255</v>
       </c>
       <c r="N22">
-        <v>617819.3854402569</v>
+        <v>0</v>
       </c>
       <c r="O22">
-        <v>296553.3050113234</v>
+        <v>-66624.72891336159</v>
       </c>
       <c r="P22">
         <v>0</v>
       </c>
       <c r="Q22">
-        <v>0</v>
+        <v>-66624.72891336157</v>
       </c>
       <c r="R22">
-        <v>0</v>
+        <v>-31979.86987627595</v>
       </c>
       <c r="S22">
+        <v>2525465.671176634</v>
+      </c>
+      <c r="T22">
+        <v>0</v>
+      </c>
+      <c r="U22">
+        <v>2525465.671176634</v>
+      </c>
+      <c r="V22">
+        <v>1306767.692860662</v>
+      </c>
+      <c r="W22">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X22">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y22">
+        <v>0</v>
+      </c>
+      <c r="Z22">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:19">
+    <row r="23" spans="1:26">
       <c r="A23">
         <v>21</v>
       </c>
       <c r="B23">
-        <v>0.3484202269800509</v>
+        <v>0.5814487403122754</v>
       </c>
       <c r="C23">
-        <v>0.2492443660177321</v>
+        <v>0.2989125792846405</v>
       </c>
       <c r="D23">
-        <v>-4127180.565372506</v>
+        <v>0.2306927903605783</v>
       </c>
       <c r="E23">
-        <v>0</v>
+        <v>0.3933300579551955</v>
       </c>
       <c r="F23">
-        <v>-4127180.565372506</v>
+        <v>0.5093236064060696</v>
       </c>
       <c r="G23">
-        <v>-4127180.565372506</v>
+        <v>-1337640.561049753</v>
       </c>
       <c r="H23">
-        <v>-5753019.632758274</v>
+        <v>0</v>
       </c>
       <c r="I23">
-        <v>-1281907.356119556</v>
+        <v>-1337640.561049753</v>
       </c>
       <c r="J23">
-        <v>-4471112.276638718</v>
+        <v>-1517277.648816775</v>
       </c>
       <c r="K23">
-        <v>0</v>
+        <v>-1199432.17193344</v>
       </c>
       <c r="L23">
-        <v>723719.0476208345</v>
+        <v>498406.9580739055</v>
       </c>
       <c r="M23">
-        <v>0</v>
+        <v>-1697839.130007345</v>
       </c>
       <c r="N23">
-        <v>723719.0476208347</v>
+        <v>0</v>
       </c>
       <c r="O23">
-        <v>347385.1428580006</v>
+        <v>692919.365236494</v>
       </c>
       <c r="P23">
         <v>0</v>
       </c>
       <c r="Q23">
-        <v>0</v>
+        <v>692919.365236494</v>
       </c>
       <c r="R23">
-        <v>0</v>
+        <v>332601.2952912854</v>
       </c>
       <c r="S23">
+        <v>1609329.608915363</v>
+      </c>
+      <c r="T23">
+        <v>0</v>
+      </c>
+      <c r="U23">
+        <v>1609329.608915363</v>
+      </c>
+      <c r="V23">
+        <v>832725.609417952</v>
+      </c>
+      <c r="W23">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X23">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y23">
+        <v>0</v>
+      </c>
+      <c r="Z23">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:19">
+    <row r="24" spans="1:26">
       <c r="A24">
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0.30230809422865</v>
+        <v>0.5556401613864939</v>
       </c>
       <c r="C24">
-        <v>0.5273749780437678</v>
+        <v>0.1975806157043141</v>
       </c>
       <c r="D24">
-        <v>-3040367.359236895</v>
+        <v>0.1045672769036568</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>0.3749870748209161</v>
       </c>
       <c r="F24">
-        <v>-3040367.359236895</v>
+        <v>0.6304929757736745</v>
       </c>
       <c r="G24">
-        <v>-3040367.359236895</v>
+        <v>-2544338.919835958</v>
       </c>
       <c r="H24">
-        <v>-4075580.009451914</v>
+        <v>0</v>
       </c>
       <c r="I24">
-        <v>-781848.7062924851</v>
+        <v>-2544338.919835958</v>
       </c>
       <c r="J24">
-        <v>-3293731.303159429</v>
+        <v>-2680842.804023526</v>
       </c>
       <c r="K24">
-        <v>0</v>
+        <v>-2800754.692791896</v>
       </c>
       <c r="L24">
-        <v>1531313.718127297</v>
+        <v>91516.33708231343</v>
       </c>
       <c r="M24">
-        <v>0</v>
+        <v>-2892271.02987421</v>
       </c>
       <c r="N24">
-        <v>1531313.718127297</v>
+        <v>0</v>
       </c>
       <c r="O24">
-        <v>735030.5847011025</v>
+        <v>300141.9294282658</v>
       </c>
       <c r="P24">
         <v>0</v>
       </c>
       <c r="Q24">
-        <v>0</v>
+        <v>300141.9294282658</v>
       </c>
       <c r="R24">
-        <v>0</v>
+        <v>144068.1261159377</v>
       </c>
       <c r="S24">
+        <v>1903766.33784806</v>
+      </c>
+      <c r="T24">
+        <v>0</v>
+      </c>
+      <c r="U24">
+        <v>1903766.33784806</v>
+      </c>
+      <c r="V24">
+        <v>985077.8703701104</v>
+      </c>
+      <c r="W24">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X24">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y24">
+        <v>0</v>
+      </c>
+      <c r="Z24">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:19">
+    <row r="25" spans="1:26">
       <c r="A25">
         <v>23</v>
       </c>
       <c r="B25">
-        <v>0.4833481498812586</v>
+        <v>0.6316254619238113</v>
       </c>
       <c r="C25">
-        <v>0.4003394824232875</v>
+        <v>0.3251274850995381</v>
       </c>
       <c r="D25">
-        <v>-2199511.446047037</v>
+        <v>0.2082341538473999</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>0.2986982571562277</v>
       </c>
       <c r="F25">
-        <v>-2199511.446047037</v>
+        <v>0.4886048085270118</v>
       </c>
       <c r="G25">
-        <v>-2199511.446047037</v>
+        <v>-1404331.829432959</v>
       </c>
       <c r="H25">
-        <v>-2939526.875956819</v>
+        <v>0</v>
       </c>
       <c r="I25">
-        <v>-556722.8131237589</v>
+        <v>-1404331.829432959</v>
       </c>
       <c r="J25">
-        <v>-2382804.062833059</v>
+        <v>-1578981.494132987</v>
       </c>
       <c r="K25">
-        <v>0</v>
+        <v>-1267235.556809016</v>
       </c>
       <c r="L25">
-        <v>1162446.772914364</v>
+        <v>487176.9615119733</v>
       </c>
       <c r="M25">
-        <v>0</v>
+        <v>-1754412.518320988</v>
       </c>
       <c r="N25">
-        <v>1162446.772914365</v>
+        <v>0</v>
       </c>
       <c r="O25">
-        <v>557974.4509988951</v>
+        <v>679436.4378181199</v>
       </c>
       <c r="P25">
         <v>0</v>
       </c>
       <c r="Q25">
-        <v>0</v>
+        <v>679436.4378181198</v>
       </c>
       <c r="R25">
-        <v>0</v>
+        <v>326129.4901308983</v>
       </c>
       <c r="S25">
+        <v>1677092.92821482</v>
+      </c>
+      <c r="T25">
+        <v>0</v>
+      </c>
+      <c r="U25">
+        <v>1677092.92821482</v>
+      </c>
+      <c r="V25">
+        <v>867788.8127836408</v>
+      </c>
+      <c r="W25">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X25">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y25">
+        <v>0</v>
+      </c>
+      <c r="Z25">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:19">
+    <row r="26" spans="1:26">
       <c r="A26">
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0.3318980347827936</v>
+        <v>0.5247748294947608</v>
       </c>
       <c r="C26">
-        <v>0.2215124189892858</v>
+        <v>0.2185058233638709</v>
       </c>
       <c r="D26">
-        <v>-4412086.044025646</v>
+        <v>0.1316055816870273</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>0.3381094703391625</v>
       </c>
       <c r="F26">
-        <v>-4412086.044025646</v>
+        <v>0.536414824958495</v>
       </c>
       <c r="G26">
-        <v>-4412086.044025646</v>
+        <v>-2947824.745261272</v>
       </c>
       <c r="H26">
-        <v>-6171400.703036601</v>
+        <v>0</v>
       </c>
       <c r="I26">
-        <v>-1391640.824360185</v>
+        <v>-2947824.745261272</v>
       </c>
       <c r="J26">
-        <v>-4779759.878676414</v>
+        <v>-3081804.177393634</v>
       </c>
       <c r="K26">
-        <v>0</v>
+        <v>-3454183.663459043</v>
       </c>
       <c r="L26">
-        <v>643195.1079516395</v>
+        <v>-100889.9441920754</v>
       </c>
       <c r="M26">
-        <v>0</v>
+        <v>-3353293.719266967</v>
       </c>
       <c r="N26">
-        <v>643195.1079516395</v>
+        <v>0</v>
       </c>
       <c r="O26">
-        <v>308733.651816787</v>
+        <v>356766.8945017974</v>
       </c>
       <c r="P26">
         <v>0</v>
       </c>
       <c r="Q26">
-        <v>0</v>
+        <v>356766.8945017974</v>
       </c>
       <c r="R26">
-        <v>0</v>
+        <v>171248.1093494162</v>
       </c>
       <c r="S26">
+        <v>1529725.584548512</v>
+      </c>
+      <c r="T26">
+        <v>0</v>
+      </c>
+      <c r="U26">
+        <v>1529725.584548512</v>
+      </c>
+      <c r="V26">
+        <v>791535.5950568272</v>
+      </c>
+      <c r="W26">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="X26">
+        <v>-617770.0976527601</v>
+      </c>
+      <c r="Y26">
+        <v>0</v>
+      </c>
+      <c r="Z26">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor Project. Flatten project structure
</commit_message>
<xml_diff>
--- a/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
+++ b/biodym_mfa_tool/data/02_output/mc_results_detailed.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>iteration</t>
   </si>
@@ -92,6 +92,18 @@
   </si>
   <si>
     <t>S_11_CC_mc</t>
+  </si>
+  <si>
+    <t>S_12_material_mc</t>
+  </si>
+  <si>
+    <t>S_12_WC_mc</t>
+  </si>
+  <si>
+    <t>S_12_DM_mc</t>
+  </si>
+  <si>
+    <t>S_12_CC_mc</t>
   </si>
 </sst>
 </file>
@@ -449,10 +461,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z26"/>
+  <dimension ref="A1:AD26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:26">
+    <row r="1" spans="1:30">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -531,73 +543,85 @@
       <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="2" spans="1:26">
+    <row r="2" spans="1:30">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2">
-        <v>0.7141179519131081</v>
+        <v>0.6431403559272725</v>
       </c>
       <c r="C2">
-        <v>0.374916472221994</v>
+        <v>0.12744463843634</v>
       </c>
       <c r="D2">
-        <v>0.07035854270650752</v>
+        <v>0.03945485230663937</v>
       </c>
       <c r="E2">
-        <v>0.3409304218260964</v>
+        <v>0.4330484284520055</v>
       </c>
       <c r="F2">
-        <v>0.5680991632037351</v>
+        <v>0.5206701024032627</v>
       </c>
       <c r="G2">
-        <v>-434413.4397508474</v>
+        <v>-4748474.064369355</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2">
-        <v>-434413.4397508474</v>
+        <v>-4748474.064369355</v>
       </c>
       <c r="J2">
-        <v>-644137.7360914743</v>
+        <v>-4808146.935979391</v>
       </c>
       <c r="K2">
-        <v>92851.06920426589</v>
+        <v>-5798794.149884361</v>
       </c>
       <c r="L2">
-        <v>828447.6871056301</v>
+        <v>-672220.8576691156</v>
       </c>
       <c r="M2">
-        <v>-735596.6179013635</v>
+        <v>-5126573.292215247</v>
       </c>
       <c r="N2">
         <v>0</v>
       </c>
       <c r="O2">
-        <v>259551.7904839946</v>
+        <v>131082.1108858116</v>
       </c>
       <c r="P2">
         <v>0</v>
       </c>
       <c r="Q2">
-        <v>259551.7904839946</v>
+        <v>131082.1108858116</v>
       </c>
       <c r="R2">
-        <v>124584.8594239899</v>
+        <v>62919.41322098392</v>
       </c>
       <c r="S2">
-        <v>2204620.606525467</v>
+        <v>1819735.067723746</v>
       </c>
       <c r="T2">
         <v>0</v>
       </c>
       <c r="U2">
-        <v>2204620.606525467</v>
+        <v>1819735.067723746</v>
       </c>
       <c r="V2">
-        <v>1140750.799546648</v>
+        <v>941597.0382044769</v>
       </c>
       <c r="W2">
         <v>-617770.0976527601</v>
@@ -611,73 +635,85 @@
       <c r="Z2">
         <v>0</v>
       </c>
+      <c r="AA2">
+        <v>3181176.525180651</v>
+      </c>
+      <c r="AB2">
+        <v>445364.7125130642</v>
+      </c>
+      <c r="AC2">
+        <v>2735811.812667588</v>
+      </c>
+      <c r="AD2">
+        <v>1313189.669255731</v>
+      </c>
     </row>
-    <row r="3" spans="1:26">
+    <row r="3" spans="1:30">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3">
-        <v>0.6177241021928185</v>
+        <v>0.7814234870689233</v>
       </c>
       <c r="C3">
-        <v>0.1445432858772167</v>
+        <v>0.3679853523912332</v>
       </c>
       <c r="D3">
-        <v>0.2016764824454824</v>
+        <v>0.2090806584875583</v>
       </c>
       <c r="E3">
-        <v>0.2702098473322121</v>
+        <v>0.4125590807057733</v>
       </c>
       <c r="F3">
-        <v>0.6735951032709135</v>
+        <v>0.6008557123869054</v>
       </c>
       <c r="G3">
-        <v>-2612238.988641692</v>
+        <v>-990306.9614693365</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>-2612238.988641692</v>
+        <v>-990306.9614693365</v>
       </c>
       <c r="J3">
-        <v>-2714920.098999678</v>
+        <v>-1136171.42098981</v>
       </c>
       <c r="K3">
-        <v>-2668906.908090111</v>
+        <v>-360128.2234143842</v>
       </c>
       <c r="L3">
-        <v>198583.6569247001</v>
+        <v>817590.7230088059</v>
       </c>
       <c r="M3">
-        <v>-2867490.56501481</v>
+        <v>-1177718.946423189</v>
       </c>
       <c r="N3">
         <v>0</v>
       </c>
       <c r="O3">
-        <v>643557.0430995977</v>
+        <v>843990.508480077</v>
       </c>
       <c r="P3">
         <v>0</v>
       </c>
       <c r="Q3">
-        <v>643557.0430995976</v>
+        <v>843990.5084800771</v>
       </c>
       <c r="R3">
-        <v>308907.3806671588</v>
+        <v>405115.4440433583</v>
       </c>
       <c r="S3">
-        <v>2261170.080690844</v>
+        <v>2551504.960970229</v>
       </c>
       <c r="T3">
         <v>0</v>
       </c>
       <c r="U3">
-        <v>2261170.080690844</v>
+        <v>2551504.96097023</v>
       </c>
       <c r="V3">
-        <v>1170011.552021317</v>
+        <v>1320241.367452902</v>
       </c>
       <c r="W3">
         <v>-617770.0976527601</v>
@@ -691,73 +727,85 @@
       <c r="Z3">
         <v>0</v>
       </c>
+      <c r="AA3">
+        <v>3865168.824158765</v>
+      </c>
+      <c r="AB3">
+        <v>541123.6341523586</v>
+      </c>
+      <c r="AC3">
+        <v>3324045.190006407</v>
+      </c>
+      <c r="AD3">
+        <v>1595541.690201041</v>
+      </c>
     </row>
-    <row r="4" spans="1:26">
+    <row r="4" spans="1:30">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.8102403433131202</v>
+        <v>0.6291394656067194</v>
       </c>
       <c r="C4">
-        <v>0.1773769037443589</v>
+        <v>0.1525463467182081</v>
       </c>
       <c r="D4">
-        <v>0.3081927605365722</v>
+        <v>-0.1120990661786276</v>
       </c>
       <c r="E4">
-        <v>0.3914404303325235</v>
+        <v>0.3382481729904302</v>
       </c>
       <c r="F4">
-        <v>0.5352638396254494</v>
+        <v>0.5196844865374735</v>
       </c>
       <c r="G4">
-        <v>-185068.9408502296</v>
+        <v>-5148370.645360963</v>
       </c>
       <c r="H4">
         <v>0</v>
       </c>
       <c r="I4">
-        <v>-185068.9408502296</v>
+        <v>-5148370.645360963</v>
       </c>
       <c r="J4">
-        <v>-351269.6840210815</v>
+        <v>-5216462.091139037</v>
       </c>
       <c r="K4">
-        <v>759286.019129728</v>
+        <v>-6479576.113041029</v>
       </c>
       <c r="L4">
-        <v>1122217.038413074</v>
+        <v>-898890.3600189651</v>
       </c>
       <c r="M4">
-        <v>-362931.0192833458</v>
+        <v>-5580685.753022062</v>
       </c>
       <c r="N4">
         <v>0</v>
       </c>
       <c r="O4">
-        <v>1289951.96783017</v>
+        <v>-364322.6453516384</v>
       </c>
       <c r="P4">
         <v>0</v>
       </c>
       <c r="Q4">
-        <v>1289951.96783017</v>
+        <v>-364322.6453516384</v>
       </c>
       <c r="R4">
-        <v>619176.9445170942</v>
+        <v>-174874.8697570975</v>
       </c>
       <c r="S4">
-        <v>2356793.495474354</v>
+        <v>1776750.489687006</v>
       </c>
       <c r="T4">
         <v>0</v>
       </c>
       <c r="U4">
-        <v>2356793.495474354</v>
+        <v>1776750.489687006</v>
       </c>
       <c r="V4">
-        <v>1219490.58099655</v>
+        <v>919355.2558232143</v>
       </c>
       <c r="W4">
         <v>-617770.0976527601</v>
@@ -771,73 +819,85 @@
       <c r="Z4">
         <v>0</v>
       </c>
+      <c r="AA4">
+        <v>3111923.673592514</v>
+      </c>
+      <c r="AB4">
+        <v>435669.3133127608</v>
+      </c>
+      <c r="AC4">
+        <v>2676254.360279754</v>
+      </c>
+      <c r="AD4">
+        <v>1284602.092127525</v>
+      </c>
     </row>
-    <row r="5" spans="1:26">
+    <row r="5" spans="1:30">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5">
-        <v>0.6044427041784902</v>
+        <v>0.6182626299841631</v>
       </c>
       <c r="C5">
-        <v>0.3610353065805824</v>
+        <v>0.2365963502391236</v>
       </c>
       <c r="D5">
-        <v>-0.1846131332897333</v>
+        <v>-0.1080869601270106</v>
       </c>
       <c r="E5">
-        <v>0.3256859196937808</v>
+        <v>0.4252991628973815</v>
       </c>
       <c r="F5">
-        <v>0.6127851720596404</v>
+        <v>0.5624744769282723</v>
       </c>
       <c r="G5">
-        <v>-2107866.959007225</v>
+        <v>-4288101.676740206</v>
       </c>
       <c r="H5">
         <v>0</v>
       </c>
       <c r="I5">
-        <v>-2107866.959007225</v>
+        <v>-4288101.676740206</v>
       </c>
       <c r="J5">
-        <v>-2297015.866613362</v>
+        <v>-4384839.718194245</v>
       </c>
       <c r="K5">
-        <v>-2422472.143054044</v>
+        <v>-5293489.223176964</v>
       </c>
       <c r="L5">
-        <v>98126.68916577478</v>
+        <v>-593898.0197997396</v>
       </c>
       <c r="M5">
-        <v>-2520598.832219819</v>
+        <v>-4699591.203377223</v>
       </c>
       <c r="N5">
         <v>0</v>
       </c>
       <c r="O5">
-        <v>-576441.150033399</v>
+        <v>-345210.1388804268</v>
       </c>
       <c r="P5">
         <v>0</v>
       </c>
       <c r="Q5">
-        <v>-576441.150033399</v>
+        <v>-345210.1388804268</v>
       </c>
       <c r="R5">
-        <v>-276691.7519975368</v>
+        <v>-165700.8666515292</v>
       </c>
       <c r="S5">
-        <v>2012811.707469404</v>
+        <v>1889798.846559763</v>
       </c>
       <c r="T5">
         <v>0</v>
       </c>
       <c r="U5">
-        <v>2012811.707469404</v>
+        <v>1889798.846559763</v>
       </c>
       <c r="V5">
-        <v>1041501.906421581</v>
+        <v>977850.5829141082</v>
       </c>
       <c r="W5">
         <v>-617770.0976527601</v>
@@ -851,73 +911,85 @@
       <c r="Z5">
         <v>0</v>
       </c>
+      <c r="AA5">
+        <v>3058123.389048348</v>
+      </c>
+      <c r="AB5">
+        <v>428137.2734936961</v>
+      </c>
+      <c r="AC5">
+        <v>2629986.115554652</v>
+      </c>
+      <c r="AD5">
+        <v>1262393.334673423</v>
+      </c>
     </row>
-    <row r="6" spans="1:26">
+    <row r="6" spans="1:30">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6">
-        <v>0.5887100173938941</v>
+        <v>0.585220431616184</v>
       </c>
       <c r="C6">
-        <v>0.2385952869318479</v>
+        <v>0.104111339391327</v>
       </c>
       <c r="D6">
-        <v>0.07506266536843578</v>
+        <v>-0.04589048135038606</v>
       </c>
       <c r="E6">
-        <v>0.3221149590456617</v>
+        <v>0.5052433611027169</v>
       </c>
       <c r="F6">
-        <v>0.6842810901233787</v>
+        <v>0.5188194137405856</v>
       </c>
       <c r="G6">
-        <v>-2141474.880288031</v>
+        <v>-5476504.265870244</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6">
-        <v>-2141474.880288031</v>
+        <v>-5476504.265870244</v>
       </c>
       <c r="J6">
-        <v>-2285010.212392238</v>
+        <v>-5526688.913592145</v>
       </c>
       <c r="K6">
-        <v>-2184081.683276666</v>
+        <v>-6898373.857331268</v>
       </c>
       <c r="L6">
-        <v>264144.3278319714</v>
+        <v>-989627.7615287148</v>
       </c>
       <c r="M6">
-        <v>-2448226.011108636</v>
+        <v>-5908746.095802553</v>
       </c>
       <c r="N6">
         <v>0</v>
       </c>
       <c r="O6">
-        <v>228277.2594646938</v>
+        <v>-138732.8588993075</v>
       </c>
       <c r="P6">
         <v>0</v>
       </c>
       <c r="Q6">
-        <v>228277.2594646938</v>
+        <v>-138732.8588993074</v>
       </c>
       <c r="R6">
-        <v>109573.084535729</v>
+        <v>-66591.77226721644</v>
       </c>
       <c r="S6">
-        <v>2189151.038929578</v>
+        <v>1649967.769645117</v>
       </c>
       <c r="T6">
         <v>0</v>
       </c>
       <c r="U6">
-        <v>2189151.038929578</v>
+        <v>1649967.769645117</v>
       </c>
       <c r="V6">
-        <v>1132746.283236033</v>
+        <v>853753.2702351268</v>
       </c>
       <c r="W6">
         <v>-617770.0976527601</v>
@@ -931,73 +1003,85 @@
       <c r="Z6">
         <v>0</v>
       </c>
+      <c r="AA6">
+        <v>2894686.178461513</v>
+      </c>
+      <c r="AB6">
+        <v>405256.0640635437</v>
+      </c>
+      <c r="AC6">
+        <v>2489430.11439797</v>
+      </c>
+      <c r="AD6">
+        <v>1194926.454160586</v>
+      </c>
     </row>
-    <row r="7" spans="1:26">
+    <row r="7" spans="1:30">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7">
-        <v>0.6964751788088929</v>
+        <v>0.5814572526496374</v>
       </c>
       <c r="C7">
-        <v>0.2123895539991836</v>
+        <v>0.1043039093023103</v>
       </c>
       <c r="D7">
-        <v>-0.07486926793711637</v>
+        <v>0.1425387313609233</v>
       </c>
       <c r="E7">
-        <v>0.4708386090452701</v>
+        <v>0.2655206365401057</v>
       </c>
       <c r="F7">
-        <v>0.6368329858912428</v>
+        <v>0.5912345526269167</v>
       </c>
       <c r="G7">
-        <v>-1506699.523575195</v>
+        <v>-4610385.924707288</v>
       </c>
       <c r="H7">
         <v>0</v>
       </c>
       <c r="I7">
-        <v>-1506699.523575195</v>
+        <v>-4610385.924707288</v>
       </c>
       <c r="J7">
-        <v>-1688707.564073909</v>
+        <v>-4659961.499498062</v>
       </c>
       <c r="K7">
-        <v>-1399280.976434355</v>
+        <v>-5517269.024062592</v>
       </c>
       <c r="L7">
-        <v>424175.3411029846</v>
+        <v>-565105.1307685947</v>
       </c>
       <c r="M7">
-        <v>-1823456.317537338</v>
+        <v>-4952163.893293994</v>
       </c>
       <c r="N7">
         <v>0</v>
       </c>
       <c r="O7">
-        <v>-269368.2922749965</v>
+        <v>428142.0890998264</v>
       </c>
       <c r="P7">
         <v>0</v>
       </c>
       <c r="Q7">
-        <v>-269368.2922749965</v>
+        <v>428142.0890998265</v>
       </c>
       <c r="R7">
-        <v>-129296.7802833559</v>
+        <v>205508.2027541801</v>
       </c>
       <c r="S7">
-        <v>2410299.196485533</v>
+        <v>1868174.160990658</v>
       </c>
       <c r="T7">
         <v>0</v>
       </c>
       <c r="U7">
-        <v>2410299.196485533</v>
+        <v>1868174.160990658</v>
       </c>
       <c r="V7">
-        <v>1247176.374655624</v>
+        <v>966661.1849379281</v>
       </c>
       <c r="W7">
         <v>-617770.0976527601</v>
@@ -1011,73 +1095,85 @@
       <c r="Z7">
         <v>0</v>
       </c>
+      <c r="AA7">
+        <v>2876072.299736438</v>
+      </c>
+      <c r="AB7">
+        <v>402650.1210479561</v>
+      </c>
+      <c r="AC7">
+        <v>2473422.178688482</v>
+      </c>
+      <c r="AD7">
+        <v>1187242.645024858</v>
+      </c>
     </row>
-    <row r="8" spans="1:26">
+    <row r="8" spans="1:30">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0.6123830520681541</v>
+        <v>0.6078630886732733</v>
       </c>
       <c r="C8">
-        <v>0.1164101283602635</v>
+        <v>0.1252909838836148</v>
       </c>
       <c r="D8">
-        <v>-0.1013501714714783</v>
+        <v>0.1304382030945319</v>
       </c>
       <c r="E8">
-        <v>0.4131514059166311</v>
+        <v>0.5780111060793798</v>
       </c>
       <c r="F8">
-        <v>0.5002309783041522</v>
+        <v>0.7121521222863875</v>
       </c>
       <c r="G8">
-        <v>-3812275.953032149</v>
+        <v>-3935206.05115747</v>
       </c>
       <c r="H8">
         <v>0</v>
       </c>
       <c r="I8">
-        <v>-3812275.953032149</v>
+        <v>-3935206.05115747</v>
       </c>
       <c r="J8">
-        <v>-3936672.676231652</v>
+        <v>-3991668.843745939</v>
       </c>
       <c r="K8">
-        <v>-4736695.579572173</v>
+        <v>-4453792.117262071</v>
       </c>
       <c r="L8">
-        <v>-477403.2629380559</v>
+        <v>-256493.6463975731</v>
       </c>
       <c r="M8">
-        <v>-4259292.316634117</v>
+        <v>-4197298.470864496</v>
       </c>
       <c r="N8">
         <v>0</v>
       </c>
       <c r="O8">
-        <v>-320615.7799684128</v>
+        <v>409588.5642912443</v>
       </c>
       <c r="P8">
         <v>0</v>
       </c>
       <c r="Q8">
-        <v>-320615.7799684129</v>
+        <v>409588.5642912442</v>
       </c>
       <c r="R8">
-        <v>-153895.5743745515</v>
+        <v>196602.510846656</v>
       </c>
       <c r="S8">
-        <v>1664690.527306251</v>
+        <v>2352438.657093657</v>
       </c>
       <c r="T8">
         <v>0</v>
       </c>
       <c r="U8">
-        <v>1664690.527306252</v>
+        <v>2352438.657093657</v>
       </c>
       <c r="V8">
-        <v>861371.3599525866</v>
+        <v>1217237.229399467</v>
       </c>
       <c r="W8">
         <v>-617770.0976527601</v>
@@ -1091,73 +1187,85 @@
       <c r="Z8">
         <v>0</v>
       </c>
+      <c r="AA8">
+        <v>3006683.953805398</v>
+      </c>
+      <c r="AB8">
+        <v>420935.7525760508</v>
+      </c>
+      <c r="AC8">
+        <v>2585748.201229347</v>
+      </c>
+      <c r="AD8">
+        <v>1241159.135810612</v>
+      </c>
     </row>
-    <row r="9" spans="1:26">
+    <row r="9" spans="1:30">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0.6179192900934228</v>
+        <v>0.6266324226597151</v>
       </c>
       <c r="C9">
-        <v>0.3573044668541085</v>
+        <v>0.252185812690386</v>
       </c>
       <c r="D9">
-        <v>0.1142304910926777</v>
+        <v>0.002307329147430259</v>
       </c>
       <c r="E9">
-        <v>0.3906353697813118</v>
+        <v>0.3416252598998789</v>
       </c>
       <c r="F9">
-        <v>0.4760089254042782</v>
+        <v>0.4292378602133771</v>
       </c>
       <c r="G9">
-        <v>-1103564.424055048</v>
+        <v>-4180388.516179044</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
       <c r="I9">
-        <v>-1103564.424055048</v>
+        <v>-4180388.516179044</v>
       </c>
       <c r="J9">
-        <v>-1307983.134662195</v>
+        <v>-4283913.420140602</v>
       </c>
       <c r="K9">
-        <v>-982708.4126058645</v>
+        <v>-5207818.268187582</v>
       </c>
       <c r="L9">
-        <v>514028.7151682488</v>
+        <v>-577386.5913296803</v>
       </c>
       <c r="M9">
-        <v>-1496737.127774113</v>
+        <v>-4630431.676857902</v>
       </c>
       <c r="N9">
         <v>0</v>
       </c>
       <c r="O9">
-        <v>364628.8601584958</v>
+        <v>7468.951806306268</v>
       </c>
       <c r="P9">
         <v>0</v>
       </c>
       <c r="Q9">
-        <v>364628.8601584957</v>
+        <v>7468.951806306268</v>
       </c>
       <c r="R9">
-        <v>175021.8528643792</v>
+        <v>3585.096866787375</v>
       </c>
       <c r="S9">
-        <v>1598404.197223871</v>
+        <v>1461674.415453607</v>
       </c>
       <c r="T9">
         <v>0</v>
       </c>
       <c r="U9">
-        <v>1598404.197223871</v>
+        <v>1461674.415453607</v>
       </c>
       <c r="V9">
-        <v>827072.4044694201</v>
+        <v>756323.4477488862</v>
       </c>
       <c r="W9">
         <v>-617770.0976527601</v>
@@ -1171,73 +1279,85 @@
       <c r="Z9">
         <v>0</v>
       </c>
+      <c r="AA9">
+        <v>3099523.042692701</v>
+      </c>
+      <c r="AB9">
+        <v>433933.2249907325</v>
+      </c>
+      <c r="AC9">
+        <v>2665589.817701968</v>
+      </c>
+      <c r="AD9">
+        <v>1279483.111693402</v>
+      </c>
     </row>
-    <row r="10" spans="1:26">
+    <row r="10" spans="1:30">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0.8138550452656408</v>
+        <v>0.5281023984675571</v>
       </c>
       <c r="C10">
-        <v>0.3352445567359655</v>
+        <v>0.4276110578215772</v>
       </c>
       <c r="D10">
-        <v>0.244333117682454</v>
+        <v>-0.04353964428230009</v>
       </c>
       <c r="E10">
-        <v>0.3236842350196596</v>
+        <v>0.2858720439795592</v>
       </c>
       <c r="F10">
-        <v>0.541328059176166</v>
+        <v>0.3723934569855348</v>
       </c>
       <c r="G10">
-        <v>460692.7511133614</v>
+        <v>-3273129.763743097</v>
       </c>
       <c r="H10">
         <v>0</v>
       </c>
       <c r="I10">
-        <v>460692.7511133614</v>
+        <v>-3273129.763743097</v>
       </c>
       <c r="J10">
-        <v>258317.1443522025</v>
+        <v>-3435704.621982186</v>
       </c>
       <c r="K10">
-        <v>1556931.030423219</v>
+        <v>-4180468.038052973</v>
       </c>
       <c r="L10">
-        <v>1292739.37854013</v>
+        <v>-379231.0641330704</v>
       </c>
       <c r="M10">
-        <v>264191.6518830899</v>
+        <v>-3801236.973919902</v>
       </c>
       <c r="N10">
         <v>0</v>
       </c>
       <c r="O10">
-        <v>1027227.504948739</v>
+        <v>-118779.1626266762</v>
       </c>
       <c r="P10">
         <v>0</v>
       </c>
       <c r="Q10">
-        <v>1027227.504948739</v>
+        <v>-118779.1626266762</v>
       </c>
       <c r="R10">
-        <v>493069.2023424371</v>
+        <v>-57013.99805699366</v>
       </c>
       <c r="S10">
-        <v>2394127.97364834</v>
+        <v>1068710.17381395</v>
       </c>
       <c r="T10">
         <v>0</v>
       </c>
       <c r="U10">
-        <v>2394127.97364834</v>
+        <v>1068710.17381395</v>
       </c>
       <c r="V10">
-        <v>1238808.796430794</v>
+        <v>552989.4720449344</v>
       </c>
       <c r="W10">
         <v>-617770.0976527601</v>
@@ -1251,73 +1371,85 @@
       <c r="Z10">
         <v>0</v>
       </c>
+      <c r="AA10">
+        <v>2612162.240191576</v>
+      </c>
+      <c r="AB10">
+        <v>365702.7127956497</v>
+      </c>
+      <c r="AC10">
+        <v>2246459.527395926</v>
+      </c>
+      <c r="AD10">
+        <v>1078300.572472849</v>
+      </c>
     </row>
-    <row r="11" spans="1:26">
+    <row r="11" spans="1:30">
       <c r="A11">
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0.6427484954260548</v>
+        <v>0.6216556385927545</v>
       </c>
       <c r="C11">
-        <v>0.3963787674379488</v>
+        <v>0.2690404980999423</v>
       </c>
       <c r="D11">
-        <v>0.0756309022106509</v>
+        <v>0.1033330267451521</v>
       </c>
       <c r="E11">
-        <v>0.4534701178075405</v>
+        <v>0.3889268779913954</v>
       </c>
       <c r="F11">
-        <v>0.5871522425730369</v>
+        <v>0.5181585515848035</v>
       </c>
       <c r="G11">
-        <v>4256.847531574487</v>
+        <v>-3374270.720843185</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>4256.847531574487</v>
+        <v>-3374270.720843185</v>
       </c>
       <c r="J11">
-        <v>-230055.6903586425</v>
+        <v>-3482771.218850451</v>
       </c>
       <c r="K11">
-        <v>616933.0482691182</v>
+        <v>-3947178.983040337</v>
       </c>
       <c r="L11">
-        <v>940522.819655643</v>
+        <v>-202198.8693850906</v>
       </c>
       <c r="M11">
-        <v>-323589.7713865239</v>
+        <v>-3744980.113655246</v>
       </c>
       <c r="N11">
         <v>0</v>
       </c>
       <c r="O11">
-        <v>251117.8547800418</v>
+        <v>331838.1171530579</v>
       </c>
       <c r="P11">
         <v>0</v>
       </c>
       <c r="Q11">
-        <v>251117.8547800418</v>
+        <v>331838.1171530579</v>
       </c>
       <c r="R11">
-        <v>120536.5702863632</v>
+        <v>159282.296222821</v>
       </c>
       <c r="S11">
-        <v>2050838.939159638</v>
+        <v>1750460.476600892</v>
       </c>
       <c r="T11">
         <v>0</v>
       </c>
       <c r="U11">
-        <v>2050838.939159638</v>
+        <v>1750460.476600892</v>
       </c>
       <c r="V11">
-        <v>1061178.577694081</v>
+        <v>905751.8478902084</v>
       </c>
       <c r="W11">
         <v>-617770.0976527601</v>
@@ -1331,73 +1463,85 @@
       <c r="Z11">
         <v>0</v>
       </c>
+      <c r="AA11">
+        <v>3074906.287580387</v>
+      </c>
+      <c r="AB11">
+        <v>430486.8792828414</v>
+      </c>
+      <c r="AC11">
+        <v>2644419.408297545</v>
+      </c>
+      <c r="AD11">
+        <v>1269321.315185661</v>
+      </c>
     </row>
-    <row r="12" spans="1:26">
+    <row r="12" spans="1:30">
       <c r="A12">
         <v>10</v>
       </c>
       <c r="B12">
-        <v>0.5254224560371819</v>
+        <v>0.7116747879062296</v>
       </c>
       <c r="C12">
-        <v>0.2508611022124017</v>
+        <v>0.3696427189128711</v>
       </c>
       <c r="D12">
-        <v>0.1261928241121761</v>
+        <v>0.1083587252299568</v>
       </c>
       <c r="E12">
-        <v>0.4211961554644648</v>
+        <v>0.3155691527788931</v>
       </c>
       <c r="F12">
-        <v>0.8184149956952312</v>
+        <v>0.7738408561036993</v>
       </c>
       <c r="G12">
-        <v>-1478524.938687313</v>
+        <v>-1087853.945499251</v>
       </c>
       <c r="H12">
         <v>0</v>
       </c>
       <c r="I12">
-        <v>-1478524.938687313</v>
+        <v>-1087853.945499251</v>
       </c>
       <c r="J12">
-        <v>-1636985.426943052</v>
+        <v>-1231000.783240833</v>
       </c>
       <c r="K12">
-        <v>-1221180.615218635</v>
+        <v>-452995.9547933342</v>
       </c>
       <c r="L12">
-        <v>528428.0314906929</v>
+        <v>790322.0627346016</v>
       </c>
       <c r="M12">
-        <v>-1749608.646709326</v>
+        <v>-1243318.017527935</v>
       </c>
       <c r="N12">
         <v>0</v>
       </c>
       <c r="O12">
-        <v>342515.7390067143</v>
+        <v>398366.4088260234</v>
       </c>
       <c r="P12">
         <v>0</v>
       </c>
       <c r="Q12">
-        <v>342515.7390067142</v>
+        <v>398366.4088260234</v>
       </c>
       <c r="R12">
-        <v>164407.5547122335</v>
+        <v>191215.8762237099</v>
       </c>
       <c r="S12">
-        <v>2336802.295350139</v>
+        <v>2992767.630514105</v>
       </c>
       <c r="T12">
         <v>0</v>
       </c>
       <c r="U12">
-        <v>2336802.295350139</v>
+        <v>2992767.630514105</v>
       </c>
       <c r="V12">
-        <v>1209146.407736945</v>
+        <v>1548566.704521028</v>
       </c>
       <c r="W12">
         <v>-617770.0976527601</v>
@@ -1411,73 +1555,85 @@
       <c r="Z12">
         <v>0</v>
       </c>
+      <c r="AA12">
+        <v>3520169.599038861</v>
+      </c>
+      <c r="AB12">
+        <v>492823.7427453483</v>
+      </c>
+      <c r="AC12">
+        <v>3027345.856293513</v>
+      </c>
+      <c r="AD12">
+        <v>1453126.010108292</v>
+      </c>
     </row>
-    <row r="13" spans="1:26">
+    <row r="13" spans="1:30">
       <c r="A13">
         <v>11</v>
       </c>
       <c r="B13">
-        <v>0.6882821311920075</v>
+        <v>0.6782299012020115</v>
       </c>
       <c r="C13">
-        <v>0.3369440738919695</v>
+        <v>0.2918116465963552</v>
       </c>
       <c r="D13">
-        <v>0.06260921038024125</v>
+        <v>0.08998311622921418</v>
       </c>
       <c r="E13">
-        <v>0.4519542059537509</v>
+        <v>0.2203160368436593</v>
       </c>
       <c r="F13">
-        <v>0.5165762246018797</v>
+        <v>0.6373340413476649</v>
       </c>
       <c r="G13">
-        <v>-495850.1466884732</v>
+        <v>-2541547.883460356</v>
       </c>
       <c r="H13">
         <v>0</v>
       </c>
       <c r="I13">
-        <v>-495850.1466884732</v>
+        <v>-2541547.883460356</v>
       </c>
       <c r="J13">
-        <v>-716594.5820794145</v>
+        <v>-2658199.830306392</v>
       </c>
       <c r="K13">
-        <v>-96317.43367610761</v>
+        <v>-2633373.049152795</v>
       </c>
       <c r="L13">
-        <v>750044.9232714865</v>
+        <v>179790.9990401718</v>
       </c>
       <c r="M13">
-        <v>-846362.3569475936</v>
+        <v>-2813164.048192965</v>
       </c>
       <c r="N13">
         <v>0</v>
       </c>
       <c r="O13">
-        <v>222608.6132099074</v>
+        <v>315264.5975896546</v>
       </c>
       <c r="P13">
         <v>0</v>
       </c>
       <c r="Q13">
-        <v>222608.6132099074</v>
+        <v>315264.5975896546</v>
       </c>
       <c r="R13">
-        <v>106852.1343336134</v>
+        <v>151327.0068329192</v>
       </c>
       <c r="S13">
-        <v>1932149.250401899</v>
+        <v>2349004.292728174</v>
       </c>
       <c r="T13">
         <v>0</v>
       </c>
       <c r="U13">
-        <v>1932149.250401899</v>
+        <v>2349004.292728174</v>
       </c>
       <c r="V13">
-        <v>999764.2205264227</v>
+        <v>1215460.16450029</v>
       </c>
       <c r="W13">
         <v>-617770.0976527601</v>
@@ -1491,73 +1647,85 @@
       <c r="Z13">
         <v>0</v>
       </c>
+      <c r="AA13">
+        <v>3354740.564007483</v>
+      </c>
+      <c r="AB13">
+        <v>469663.6778935936</v>
+      </c>
+      <c r="AC13">
+        <v>2885076.88611389</v>
+      </c>
+      <c r="AD13">
+        <v>1384836.90446496</v>
+      </c>
     </row>
-    <row r="14" spans="1:26">
+    <row r="14" spans="1:30">
       <c r="A14">
         <v>12</v>
       </c>
       <c r="B14">
-        <v>0.6362147722545036</v>
+        <v>0.6019787902140284</v>
       </c>
       <c r="C14">
-        <v>0.1600828673581693</v>
+        <v>0.2574102387781348</v>
       </c>
       <c r="D14">
-        <v>0.1418184838874653</v>
+        <v>0.09154612569059632</v>
       </c>
       <c r="E14">
-        <v>0.07463464304140394</v>
+        <v>0.3720911463722949</v>
       </c>
       <c r="F14">
-        <v>0.5404204305804412</v>
+        <v>0.4896619547870266</v>
       </c>
       <c r="G14">
-        <v>-4118725.111540099</v>
+        <v>-3695801.62608428</v>
       </c>
       <c r="H14">
         <v>0</v>
       </c>
       <c r="I14">
-        <v>-4118725.111540099</v>
+        <v>-3695801.62608428</v>
       </c>
       <c r="J14">
-        <v>-4186228.538582548</v>
+        <v>-3800022.067455609</v>
       </c>
       <c r="K14">
-        <v>-4855079.498544795</v>
+        <v>-4439532.802335742</v>
       </c>
       <c r="L14">
-        <v>-398217.8916208389</v>
+        <v>-343552.5409720289</v>
       </c>
       <c r="M14">
-        <v>-4456861.606923957</v>
+        <v>-4095980.261363711</v>
       </c>
       <c r="N14">
         <v>0</v>
       </c>
       <c r="O14">
-        <v>466094.3407023191</v>
+        <v>284680.9470586713</v>
       </c>
       <c r="P14">
         <v>0</v>
       </c>
       <c r="Q14">
-        <v>466094.3407023191</v>
+        <v>284680.9470586712</v>
       </c>
       <c r="R14">
-        <v>223725.2835221589</v>
+        <v>136646.8545790284</v>
       </c>
       <c r="S14">
-        <v>1868423.280797676</v>
+        <v>1601833.285638678</v>
       </c>
       <c r="T14">
         <v>0</v>
       </c>
       <c r="U14">
-        <v>1868423.280797676</v>
+        <v>1601833.285638678</v>
       </c>
       <c r="V14">
-        <v>966790.0885770387</v>
+        <v>828846.739400033</v>
       </c>
       <c r="W14">
         <v>-617770.0976527601</v>
@@ -1571,73 +1739,85 @@
       <c r="Z14">
         <v>0</v>
       </c>
+      <c r="AA14">
+        <v>2977578.34419283</v>
+      </c>
+      <c r="AB14">
+        <v>416860.9672395525</v>
+      </c>
+      <c r="AC14">
+        <v>2560717.376953277</v>
+      </c>
+      <c r="AD14">
+        <v>1229144.340165645</v>
+      </c>
     </row>
-    <row r="15" spans="1:26">
+    <row r="15" spans="1:30">
       <c r="A15">
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0.7142450004253041</v>
+        <v>0.5534754533811409</v>
       </c>
       <c r="C15">
-        <v>0.2622900613890503</v>
+        <v>0.4227602976753032</v>
       </c>
       <c r="D15">
-        <v>0.1353447938348827</v>
+        <v>0.2133993382939711</v>
       </c>
       <c r="E15">
-        <v>0.5939559175622413</v>
+        <v>0.4322485730669088</v>
       </c>
       <c r="F15">
-        <v>0.5559141205633831</v>
+        <v>0.7178592785326956</v>
       </c>
       <c r="G15">
-        <v>384086.1212140897</v>
+        <v>-1355820.646828732</v>
       </c>
       <c r="H15">
         <v>0</v>
       </c>
       <c r="I15">
-        <v>384086.1212140897</v>
+        <v>-1355820.646828732</v>
       </c>
       <c r="J15">
-        <v>150509.3831051205</v>
+        <v>-1514697.650216857</v>
       </c>
       <c r="K15">
-        <v>1226520.734728328</v>
+        <v>-1049116.567049311</v>
       </c>
       <c r="L15">
-        <v>1128760.129812818</v>
+        <v>582287.7749032034</v>
       </c>
       <c r="M15">
-        <v>97760.60491551121</v>
+        <v>-1631404.341952513</v>
       </c>
       <c r="N15">
         <v>0</v>
       </c>
       <c r="O15">
-        <v>499374.0917304266</v>
+        <v>610138.8454543438</v>
       </c>
       <c r="P15">
         <v>0</v>
       </c>
       <c r="Q15">
-        <v>499374.0917304265</v>
+        <v>610138.8454543439</v>
       </c>
       <c r="R15">
-        <v>239699.5640145827</v>
+        <v>292866.6457985094</v>
       </c>
       <c r="S15">
-        <v>2157717.961180991</v>
+        <v>2159123.304203005</v>
       </c>
       <c r="T15">
         <v>0</v>
       </c>
       <c r="U15">
-        <v>2157717.961180992</v>
+        <v>2159123.304203005</v>
       </c>
       <c r="V15">
-        <v>1116481.666790111</v>
+        <v>1117208.842328276</v>
       </c>
       <c r="W15">
         <v>-617770.0976527601</v>
@@ -1651,73 +1831,85 @@
       <c r="Z15">
         <v>0</v>
       </c>
+      <c r="AA15">
+        <v>2737665.430777146</v>
+      </c>
+      <c r="AB15">
+        <v>383273.1594376953</v>
+      </c>
+      <c r="AC15">
+        <v>2354392.27133945</v>
+      </c>
+      <c r="AD15">
+        <v>1130108.289533205</v>
+      </c>
     </row>
-    <row r="16" spans="1:26">
+    <row r="16" spans="1:30">
       <c r="A16">
         <v>14</v>
       </c>
       <c r="B16">
-        <v>0.6780465418980448</v>
+        <v>0.5986305883946125</v>
       </c>
       <c r="C16">
-        <v>0.07892074904412297</v>
+        <v>0.2245433466074488</v>
       </c>
       <c r="D16">
-        <v>0.05964668648771772</v>
+        <v>0.02069703390006317</v>
       </c>
       <c r="E16">
-        <v>0.5110603062864235</v>
+        <v>0.3420409272884719</v>
       </c>
       <c r="F16">
-        <v>0.6867643358631997</v>
+        <v>0.7065505762884741</v>
       </c>
       <c r="G16">
-        <v>-1840181.173702325</v>
+        <v>-3526407.367319969</v>
       </c>
       <c r="H16">
         <v>0</v>
       </c>
       <c r="I16">
-        <v>-1840181.173702325</v>
+        <v>-3526407.367319969</v>
       </c>
       <c r="J16">
-        <v>-1981871.691407186</v>
+        <v>-3617290.73437062</v>
       </c>
       <c r="K16">
-        <v>-1667653.207210434</v>
+        <v>-4025600.920760069</v>
       </c>
       <c r="L16">
-        <v>423705.0149766456</v>
+        <v>-195250.2898850153</v>
       </c>
       <c r="M16">
-        <v>-2091358.222187079</v>
+        <v>-3830350.630875053</v>
       </c>
       <c r="N16">
         <v>0</v>
       </c>
       <c r="O16">
-        <v>208921.4689550902</v>
+        <v>64003.5787441314</v>
       </c>
       <c r="P16">
         <v>0</v>
       </c>
       <c r="Q16">
-        <v>208921.4689550902</v>
+        <v>64003.57874413138</v>
       </c>
       <c r="R16">
-        <v>100282.3050917402</v>
+        <v>30721.71779512956</v>
       </c>
       <c r="S16">
-        <v>2530503.843818405</v>
+        <v>2298486.310002937</v>
       </c>
       <c r="T16">
         <v>0</v>
       </c>
       <c r="U16">
-        <v>2530503.843818405</v>
+        <v>2298486.310002937</v>
       </c>
       <c r="V16">
-        <v>1309374.626431155</v>
+        <v>1189320.324831405</v>
       </c>
       <c r="W16">
         <v>-617770.0976527601</v>
@@ -1731,73 +1923,85 @@
       <c r="Z16">
         <v>0</v>
       </c>
+      <c r="AA16">
+        <v>2961017.074275106</v>
+      </c>
+      <c r="AB16">
+        <v>414542.3894563407</v>
+      </c>
+      <c r="AC16">
+        <v>2546474.684818765</v>
+      </c>
+      <c r="AD16">
+        <v>1222307.847945372</v>
+      </c>
     </row>
-    <row r="17" spans="1:26">
+    <row r="17" spans="1:30">
       <c r="A17">
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0.7097125435755307</v>
+        <v>0.514106832061633</v>
       </c>
       <c r="C17">
-        <v>0.2235076219758375</v>
+        <v>0.2270406410814022</v>
       </c>
       <c r="D17">
-        <v>0.1168051118687917</v>
+        <v>0.1840074204814704</v>
       </c>
       <c r="E17">
-        <v>0.1674700882488548</v>
+        <v>0.4415684088239745</v>
       </c>
       <c r="F17">
-        <v>0.4694144994317876</v>
+        <v>0.6754322962648835</v>
       </c>
       <c r="G17">
-        <v>-3047166.171590806</v>
+        <v>-3505831.28120247</v>
       </c>
       <c r="H17">
         <v>0</v>
       </c>
       <c r="I17">
-        <v>-3047166.171590806</v>
+        <v>-3505831.28120247</v>
       </c>
       <c r="J17">
-        <v>-3161766.717345882</v>
+        <v>-3596017.372137852</v>
       </c>
       <c r="K17">
-        <v>-3465766.044967825</v>
+        <v>-4029809.0413043</v>
       </c>
       <c r="L17">
-        <v>-67116.95283861135</v>
+        <v>-191110.0786400994</v>
       </c>
       <c r="M17">
-        <v>-3398649.092129212</v>
+        <v>-3838698.962664199</v>
       </c>
       <c r="N17">
         <v>0</v>
       </c>
       <c r="O17">
-        <v>428234.422090029</v>
+        <v>488681.5641778562</v>
       </c>
       <c r="P17">
         <v>0</v>
       </c>
       <c r="Q17">
-        <v>428234.422090029</v>
+        <v>488681.5641778562</v>
       </c>
       <c r="R17">
-        <v>205552.5225894745</v>
+        <v>234567.150789692</v>
       </c>
       <c r="S17">
-        <v>1810417.517988091</v>
+        <v>1887013.296339266</v>
       </c>
       <c r="T17">
         <v>0</v>
       </c>
       <c r="U17">
-        <v>1810417.517988092</v>
+        <v>1887013.296339266</v>
       </c>
       <c r="V17">
-        <v>936775.7994483376</v>
+        <v>976409.2380261023</v>
       </c>
       <c r="W17">
         <v>-617770.0976527601</v>
@@ -1811,73 +2015,85 @@
       <c r="Z17">
         <v>0</v>
       </c>
+      <c r="AA17">
+        <v>2542935.722376594</v>
+      </c>
+      <c r="AB17">
+        <v>356011.0003235794</v>
+      </c>
+      <c r="AC17">
+        <v>2186924.722053014</v>
+      </c>
+      <c r="AD17">
+        <v>1049723.865926198</v>
+      </c>
     </row>
-    <row r="18" spans="1:26">
+    <row r="18" spans="1:30">
       <c r="A18">
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0.5683946983950449</v>
+        <v>0.6166432745103166</v>
       </c>
       <c r="C18">
-        <v>0.3200476205441926</v>
+        <v>0.2891019034364413</v>
       </c>
       <c r="D18">
-        <v>0.1537223367781242</v>
+        <v>0.1020711615467172</v>
       </c>
       <c r="E18">
-        <v>0.3932938930368052</v>
+        <v>0.4443948529900326</v>
       </c>
       <c r="F18">
-        <v>0.4669042689686214</v>
+        <v>0.770404296273668</v>
       </c>
       <c r="G18">
-        <v>-1643623.716202915</v>
+        <v>-2364809.726280488</v>
       </c>
       <c r="H18">
         <v>0</v>
       </c>
       <c r="I18">
-        <v>-1643623.716202915</v>
+        <v>-2364809.726280488</v>
       </c>
       <c r="J18">
-        <v>-1829254.996020293</v>
+        <v>-2478011.116883099</v>
       </c>
       <c r="K18">
-        <v>-1730902.061786955</v>
+        <v>-2313035.920120178</v>
       </c>
       <c r="L18">
-        <v>323943.5892243154</v>
+        <v>283330.8195519277</v>
       </c>
       <c r="M18">
-        <v>-2054845.65101127</v>
+        <v>-2596366.739672104</v>
       </c>
       <c r="N18">
         <v>0</v>
       </c>
       <c r="O18">
-        <v>451361.2161027352</v>
+        <v>325142.9179570713</v>
       </c>
       <c r="P18">
         <v>0</v>
       </c>
       <c r="Q18">
-        <v>451361.2161027352</v>
+        <v>325142.9179570713</v>
       </c>
       <c r="R18">
-        <v>216653.3837148313</v>
+        <v>156068.6006089623</v>
       </c>
       <c r="S18">
-        <v>1442173.879267625</v>
+        <v>2581620.834551708</v>
       </c>
       <c r="T18">
         <v>0</v>
       </c>
       <c r="U18">
-        <v>1442173.879267625</v>
+        <v>2581620.834551708</v>
       </c>
       <c r="V18">
-        <v>746233.1618376032</v>
+        <v>1335824.414606426</v>
       </c>
       <c r="W18">
         <v>-617770.0976527601</v>
@@ -1891,73 +2107,85 @@
       <c r="Z18">
         <v>0</v>
       </c>
+      <c r="AA18">
+        <v>3050113.542407802</v>
+      </c>
+      <c r="AB18">
+        <v>427015.8949665685</v>
+      </c>
+      <c r="AC18">
+        <v>2623097.647441233</v>
+      </c>
+      <c r="AD18">
+        <v>1259086.869981059</v>
+      </c>
     </row>
-    <row r="19" spans="1:26">
+    <row r="19" spans="1:30">
       <c r="A19">
         <v>17</v>
       </c>
       <c r="B19">
-        <v>0.6351630365280596</v>
+        <v>0.5013877584211551</v>
       </c>
       <c r="C19">
-        <v>0.1606756796910299</v>
+        <v>0.1527931497081637</v>
       </c>
       <c r="D19">
-        <v>0.1086813004205811</v>
+        <v>0.1661330769516401</v>
       </c>
       <c r="E19">
-        <v>0.3333399296385667</v>
+        <v>0.5339104723906027</v>
       </c>
       <c r="F19">
-        <v>0.6195483612853996</v>
+        <v>0.5745155891019531</v>
       </c>
       <c r="G19">
-        <v>-2533145.806286952</v>
+        <v>-4556142.161215737</v>
       </c>
       <c r="H19">
         <v>0</v>
       </c>
       <c r="I19">
-        <v>-2533145.806286952</v>
+        <v>-4556142.161215737</v>
       </c>
       <c r="J19">
-        <v>-2657367.194674403</v>
+        <v>-4620898.61314629</v>
       </c>
       <c r="K19">
-        <v>-2686399.435611576</v>
+        <v>-5553289.299342522</v>
       </c>
       <c r="L19">
-        <v>149853.237318019</v>
+        <v>-604645.7674735889</v>
       </c>
       <c r="M19">
-        <v>-2836252.672929594</v>
+        <v>-4948643.531868935</v>
       </c>
       <c r="N19">
         <v>0</v>
       </c>
       <c r="O19">
-        <v>356596.671704758</v>
+        <v>430295.7709798953</v>
       </c>
       <c r="P19">
         <v>0</v>
       </c>
       <c r="Q19">
-        <v>356596.671704758</v>
+        <v>430295.7709798953</v>
       </c>
       <c r="R19">
-        <v>171166.4024068427</v>
+        <v>206541.9700565439</v>
       </c>
       <c r="S19">
-        <v>2138455.370531241</v>
+        <v>1565363.870608092</v>
       </c>
       <c r="T19">
         <v>0</v>
       </c>
       <c r="U19">
-        <v>2138455.370531241</v>
+        <v>1565363.870608092</v>
       </c>
       <c r="V19">
-        <v>1106514.502544253</v>
+        <v>809976.1390654448</v>
       </c>
       <c r="W19">
         <v>-617770.0976527601</v>
@@ -1971,73 +2199,85 @@
       <c r="Z19">
         <v>0</v>
       </c>
+      <c r="AA19">
+        <v>2480023.143319422</v>
+      </c>
+      <c r="AB19">
+        <v>347203.239275594</v>
+      </c>
+      <c r="AC19">
+        <v>2132819.904043829</v>
+      </c>
+      <c r="AD19">
+        <v>1023753.553298098</v>
+      </c>
     </row>
-    <row r="20" spans="1:26">
+    <row r="20" spans="1:30">
       <c r="A20">
         <v>18</v>
       </c>
       <c r="B20">
-        <v>0.7457619464381012</v>
+        <v>0.6668828778365229</v>
       </c>
       <c r="C20">
-        <v>0.310949715259784</v>
+        <v>0.3514103502017392</v>
       </c>
       <c r="D20">
-        <v>0.2669035037321189</v>
+        <v>0.07346827451908697</v>
       </c>
       <c r="E20">
-        <v>0.4320807574704697</v>
+        <v>0.472388776738255</v>
       </c>
       <c r="F20">
-        <v>0.5557140615725582</v>
+        <v>0.6576759467987514</v>
       </c>
       <c r="G20">
-        <v>617666.4597114507</v>
+        <v>-2067115.510571464</v>
       </c>
       <c r="H20">
         <v>0</v>
       </c>
       <c r="I20">
-        <v>617666.4597114507</v>
+        <v>-2067115.510571464</v>
       </c>
       <c r="J20">
-        <v>402909.8983927293</v>
+        <v>-2204084.891086744</v>
       </c>
       <c r="K20">
-        <v>1714397.909637007</v>
+        <v>-2009116.460968387</v>
       </c>
       <c r="L20">
-        <v>1317020.663511372</v>
+        <v>329722.7045865532</v>
       </c>
       <c r="M20">
-        <v>397377.2461256354</v>
+        <v>-2338839.165554939</v>
       </c>
       <c r="N20">
         <v>0</v>
       </c>
       <c r="O20">
-        <v>1028233.4708773</v>
+        <v>253096.7975093344</v>
       </c>
       <c r="P20">
         <v>0</v>
       </c>
       <c r="Q20">
-        <v>1028233.4708773</v>
+        <v>253096.7975093343</v>
       </c>
       <c r="R20">
-        <v>493552.065988114</v>
+        <v>121486.4627963601</v>
       </c>
       <c r="S20">
-        <v>2252119.170180423</v>
+        <v>2383423.888561921</v>
       </c>
       <c r="T20">
         <v>0</v>
       </c>
       <c r="U20">
-        <v>2252119.170180423</v>
+        <v>2383423.888561921</v>
       </c>
       <c r="V20">
-        <v>1165328.282087784</v>
+        <v>1233270.11390891</v>
       </c>
       <c r="W20">
         <v>-617770.0976527601</v>
@@ -2051,73 +2291,85 @@
       <c r="Z20">
         <v>0</v>
       </c>
+      <c r="AA20">
+        <v>3298614.581508803</v>
+      </c>
+      <c r="AB20">
+        <v>461806.0403616375</v>
+      </c>
+      <c r="AC20">
+        <v>2836808.541147166</v>
+      </c>
+      <c r="AD20">
+        <v>1361668.098895484</v>
+      </c>
     </row>
-    <row r="21" spans="1:26">
+    <row r="21" spans="1:30">
       <c r="A21">
         <v>19</v>
       </c>
       <c r="B21">
-        <v>0.7086600720627274</v>
+        <v>0.6725899095934567</v>
       </c>
       <c r="C21">
-        <v>0.06153079875539469</v>
+        <v>0.4757049603979319</v>
       </c>
       <c r="D21">
-        <v>0.1573991775603775</v>
+        <v>-0.05972017671732135</v>
       </c>
       <c r="E21">
-        <v>0.2634078471567534</v>
+        <v>0.5213342475293615</v>
       </c>
       <c r="F21">
-        <v>0.7073829014592595</v>
+        <v>0.6359507072286577</v>
       </c>
       <c r="G21">
-        <v>-2768309.341268966</v>
+        <v>-1564725.106301096</v>
       </c>
       <c r="H21">
         <v>0</v>
       </c>
       <c r="I21">
-        <v>-2768309.341268966</v>
+        <v>-1564725.106301096</v>
       </c>
       <c r="J21">
-        <v>-2847770.30138173</v>
+        <v>-1745313.42882504</v>
       </c>
       <c r="K21">
-        <v>-2728269.817436323</v>
+        <v>-1490079.715107991</v>
       </c>
       <c r="L21">
-        <v>223812.1346805051</v>
+        <v>399978.2611806736</v>
       </c>
       <c r="M21">
-        <v>-2952081.952116827</v>
+        <v>-1890057.976288664</v>
       </c>
       <c r="N21">
         <v>0</v>
       </c>
       <c r="O21">
-        <v>576205.8531964117</v>
+        <v>-207495.4962018969</v>
       </c>
       <c r="P21">
         <v>0</v>
       </c>
       <c r="Q21">
-        <v>576205.8531964117</v>
+        <v>-207495.4962018968</v>
       </c>
       <c r="R21">
-        <v>276578.8095157906</v>
+        <v>-99597.83817025315</v>
       </c>
       <c r="S21">
-        <v>2724157.945605551</v>
+        <v>2324414.437782574</v>
       </c>
       <c r="T21">
         <v>0</v>
       </c>
       <c r="U21">
-        <v>2724157.945605551</v>
+        <v>2324414.437782574</v>
       </c>
       <c r="V21">
-        <v>1409578.294488734</v>
+        <v>1202736.480158912</v>
       </c>
       <c r="W21">
         <v>-617770.0976527601</v>
@@ -2131,73 +2383,85 @@
       <c r="Z21">
         <v>0</v>
       </c>
+      <c r="AA21">
+        <v>3326843.373694364</v>
+      </c>
+      <c r="AB21">
+        <v>465758.0712586338</v>
+      </c>
+      <c r="AC21">
+        <v>2861085.30243573</v>
+      </c>
+      <c r="AD21">
+        <v>1373320.944306676</v>
+      </c>
     </row>
-    <row r="22" spans="1:26">
+    <row r="22" spans="1:30">
       <c r="A22">
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0.6562918516087181</v>
+        <v>0.6757328595849195</v>
       </c>
       <c r="C22">
-        <v>0.1356517054263593</v>
+        <v>0.2150933573247609</v>
       </c>
       <c r="D22">
-        <v>-0.01965174861438668</v>
+        <v>0.04537561180386183</v>
       </c>
       <c r="E22">
-        <v>0.382360731142212</v>
+        <v>0.4188482188540914</v>
       </c>
       <c r="F22">
-        <v>0.7081164691966496</v>
+        <v>0.7359175241845073</v>
       </c>
       <c r="G22">
-        <v>-2497210.727842766</v>
+        <v>-3030240.815548166</v>
       </c>
       <c r="H22">
         <v>0</v>
       </c>
       <c r="I22">
-        <v>-2497210.727842766</v>
+        <v>-3030240.815548166</v>
       </c>
       <c r="J22">
-        <v>-2625382.559819886</v>
+        <v>-3119189.15604203</v>
       </c>
       <c r="K22">
-        <v>-2615649.691032325</v>
+        <v>-3197385.540766086</v>
       </c>
       <c r="L22">
-        <v>159719.5585179308</v>
+        <v>59920.59943236323</v>
       </c>
       <c r="M22">
-        <v>-2775369.249550255</v>
+        <v>-3257306.14019845</v>
       </c>
       <c r="N22">
         <v>0</v>
       </c>
       <c r="O22">
-        <v>-66624.72891336159</v>
+        <v>158392.5588156202</v>
       </c>
       <c r="P22">
         <v>0</v>
       </c>
       <c r="Q22">
-        <v>-66624.72891336157</v>
+        <v>158392.5588156202</v>
       </c>
       <c r="R22">
-        <v>-31979.86987627595</v>
+        <v>76028.4282264158</v>
       </c>
       <c r="S22">
-        <v>2525465.671176634</v>
+        <v>2702364.612782164</v>
       </c>
       <c r="T22">
         <v>0</v>
       </c>
       <c r="U22">
-        <v>2525465.671176634</v>
+        <v>2702364.612782164</v>
       </c>
       <c r="V22">
-        <v>1306767.692860662</v>
+        <v>1398301.632295938</v>
       </c>
       <c r="W22">
         <v>-617770.0976527601</v>
@@ -2211,73 +2475,85 @@
       <c r="Z22">
         <v>0</v>
       </c>
+      <c r="AA22">
+        <v>3342389.402862823</v>
+      </c>
+      <c r="AB22">
+        <v>467934.5153372712</v>
+      </c>
+      <c r="AC22">
+        <v>2874454.887525551</v>
+      </c>
+      <c r="AD22">
+        <v>1379738.34514576</v>
+      </c>
     </row>
-    <row r="23" spans="1:26">
+    <row r="23" spans="1:30">
       <c r="A23">
         <v>21</v>
       </c>
       <c r="B23">
-        <v>0.5814487403122754</v>
+        <v>0.7039513767871206</v>
       </c>
       <c r="C23">
-        <v>0.2989125792846405</v>
+        <v>0.2234308689498467</v>
       </c>
       <c r="D23">
-        <v>0.2306927903605783</v>
+        <v>0.06437621299672391</v>
       </c>
       <c r="E23">
-        <v>0.3933300579551955</v>
+        <v>0.3033583848977927</v>
       </c>
       <c r="F23">
-        <v>0.5093236064060696</v>
+        <v>0.5537408594018681</v>
       </c>
       <c r="G23">
-        <v>-1337640.561049753</v>
+        <v>-3444279.962111221</v>
       </c>
       <c r="H23">
         <v>0</v>
       </c>
       <c r="I23">
-        <v>-1337640.561049753</v>
+        <v>-3444279.962111221</v>
       </c>
       <c r="J23">
-        <v>-1517277.648816775</v>
+        <v>-3538504.850082232</v>
       </c>
       <c r="K23">
-        <v>-1199432.17193344</v>
+        <v>-3934852.232656742</v>
       </c>
       <c r="L23">
-        <v>498406.9580739055</v>
+        <v>-172458.8816928371</v>
       </c>
       <c r="M23">
-        <v>-1697839.130007345</v>
+        <v>-3762393.350963905</v>
       </c>
       <c r="N23">
         <v>0</v>
       </c>
       <c r="O23">
-        <v>692919.365236494</v>
+        <v>234102.1114050286</v>
       </c>
       <c r="P23">
         <v>0</v>
       </c>
       <c r="Q23">
-        <v>692919.365236494</v>
+        <v>234102.1114050287</v>
       </c>
       <c r="R23">
-        <v>332601.2952912854</v>
+        <v>112369.0134669028</v>
       </c>
       <c r="S23">
-        <v>1609329.608915363</v>
+        <v>2118307.457531363</v>
       </c>
       <c r="T23">
         <v>0</v>
       </c>
       <c r="U23">
-        <v>1609329.608915363</v>
+        <v>2118307.457531363</v>
       </c>
       <c r="V23">
-        <v>832725.609417952</v>
+        <v>1096089.240349127</v>
       </c>
       <c r="W23">
         <v>-617770.0976527601</v>
@@ -2291,73 +2567,85 @@
       <c r="Z23">
         <v>0</v>
       </c>
+      <c r="AA23">
+        <v>3481967.153927163</v>
+      </c>
+      <c r="AB23">
+        <v>487475.4004418664</v>
+      </c>
+      <c r="AC23">
+        <v>2994491.753485297</v>
+      </c>
+      <c r="AD23">
+        <v>1437356.040770253</v>
+      </c>
     </row>
-    <row r="24" spans="1:26">
+    <row r="24" spans="1:30">
       <c r="A24">
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0.5556401613864939</v>
+        <v>0.834037206843414</v>
       </c>
       <c r="C24">
-        <v>0.1975806157043141</v>
+        <v>0.3393437396082378</v>
       </c>
       <c r="D24">
-        <v>0.1045672769036568</v>
+        <v>0.04719031678777415</v>
       </c>
       <c r="E24">
-        <v>0.3749870748209161</v>
+        <v>0.4458376114694318</v>
       </c>
       <c r="F24">
-        <v>0.6304929757736745</v>
+        <v>0.5898474515346852</v>
       </c>
       <c r="G24">
-        <v>-2544338.919835958</v>
+        <v>-1803949.181727477</v>
       </c>
       <c r="H24">
         <v>0</v>
       </c>
       <c r="I24">
-        <v>-2544338.919835958</v>
+        <v>-1803949.181727477</v>
       </c>
       <c r="J24">
-        <v>-2680842.804023526</v>
+        <v>-1941157.612894339</v>
       </c>
       <c r="K24">
-        <v>-2800754.692791896</v>
+        <v>-1569945.621050389</v>
       </c>
       <c r="L24">
-        <v>91516.33708231343</v>
+        <v>461678.3336767687</v>
       </c>
       <c r="M24">
-        <v>-2892271.02987421</v>
+        <v>-2031623.954727158</v>
       </c>
       <c r="N24">
         <v>0</v>
       </c>
       <c r="O24">
-        <v>300141.9294282658</v>
+        <v>203317.8744159263</v>
       </c>
       <c r="P24">
         <v>0</v>
       </c>
       <c r="Q24">
-        <v>300141.9294282658</v>
+        <v>203317.8744159262</v>
       </c>
       <c r="R24">
-        <v>144068.1261159377</v>
+        <v>97592.57971312126</v>
       </c>
       <c r="S24">
-        <v>1903766.33784806</v>
+        <v>2673405.853677068</v>
       </c>
       <c r="T24">
         <v>0</v>
       </c>
       <c r="U24">
-        <v>1903766.33784806</v>
+        <v>2673405.853677068</v>
       </c>
       <c r="V24">
-        <v>985077.8703701104</v>
+        <v>1383317.318212491</v>
       </c>
       <c r="W24">
         <v>-617770.0976527601</v>
@@ -2371,73 +2659,85 @@
       <c r="Z24">
         <v>0</v>
       </c>
+      <c r="AA24">
+        <v>4125412.997466356</v>
+      </c>
+      <c r="AB24">
+        <v>577557.8183326136</v>
+      </c>
+      <c r="AC24">
+        <v>3547855.179133743</v>
+      </c>
+      <c r="AD24">
+        <v>1702970.484914695</v>
+      </c>
     </row>
-    <row r="25" spans="1:26">
+    <row r="25" spans="1:30">
       <c r="A25">
         <v>23</v>
       </c>
       <c r="B25">
-        <v>0.6316254619238113</v>
+        <v>0.7846492802747165</v>
       </c>
       <c r="C25">
-        <v>0.3251274850995381</v>
+        <v>0.2675141549413244</v>
       </c>
       <c r="D25">
-        <v>0.2082341538473999</v>
+        <v>0.1820713772985778</v>
       </c>
       <c r="E25">
-        <v>0.2986982571562277</v>
+        <v>0.6199131944313446</v>
       </c>
       <c r="F25">
-        <v>0.4886048085270118</v>
+        <v>0.5369633030372837</v>
       </c>
       <c r="G25">
-        <v>-1404331.829432959</v>
+        <v>-2249939.891560697</v>
       </c>
       <c r="H25">
         <v>0</v>
       </c>
       <c r="I25">
-        <v>-1404331.829432959</v>
+        <v>-2249939.891560697</v>
       </c>
       <c r="J25">
-        <v>-1578981.494132987</v>
+        <v>-2361582.687940916</v>
       </c>
       <c r="K25">
-        <v>-1267235.556809016</v>
+        <v>-2152672.211569066</v>
       </c>
       <c r="L25">
-        <v>487176.9615119733</v>
+        <v>338780.3929281814</v>
       </c>
       <c r="M25">
-        <v>-1754412.518320988</v>
+        <v>-2491452.604497246</v>
       </c>
       <c r="N25">
         <v>0</v>
       </c>
       <c r="O25">
-        <v>679436.4378181199</v>
+        <v>737996.8378959532</v>
       </c>
       <c r="P25">
         <v>0</v>
       </c>
       <c r="Q25">
-        <v>679436.4378181198</v>
+        <v>737996.8378959532</v>
       </c>
       <c r="R25">
-        <v>326129.4901308983</v>
+        <v>354238.4821663795</v>
       </c>
       <c r="S25">
-        <v>1677092.92821482</v>
+        <v>2289601.754093513</v>
       </c>
       <c r="T25">
         <v>0</v>
       </c>
       <c r="U25">
-        <v>1677092.92821482</v>
+        <v>2289601.754093513</v>
       </c>
       <c r="V25">
-        <v>867788.8127836408</v>
+        <v>1184723.132812381</v>
       </c>
       <c r="W25">
         <v>-617770.0976527601</v>
@@ -2451,73 +2751,85 @@
       <c r="Z25">
         <v>0</v>
       </c>
+      <c r="AA25">
+        <v>3881124.622184472</v>
+      </c>
+      <c r="AB25">
+        <v>543357.4458708805</v>
+      </c>
+      <c r="AC25">
+        <v>3337767.17631359</v>
+      </c>
+      <c r="AD25">
+        <v>1602128.243624354</v>
+      </c>
     </row>
-    <row r="26" spans="1:26">
+    <row r="26" spans="1:30">
       <c r="A26">
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0.5247748294947608</v>
+        <v>0.5189335541587072</v>
       </c>
       <c r="C26">
-        <v>0.2185058233638709</v>
+        <v>0.2519278409879759</v>
       </c>
       <c r="D26">
-        <v>0.1316055816870273</v>
+        <v>0.07626335872218765</v>
       </c>
       <c r="E26">
-        <v>0.3381094703391625</v>
+        <v>0.3582469543209711</v>
       </c>
       <c r="F26">
-        <v>0.536414824958495</v>
+        <v>0.5021841896047309</v>
       </c>
       <c r="G26">
-        <v>-2947824.745261272</v>
+        <v>-4088311.31783057</v>
       </c>
       <c r="H26">
         <v>0</v>
       </c>
       <c r="I26">
-        <v>-2947824.745261272</v>
+        <v>-4088311.31783057</v>
       </c>
       <c r="J26">
-        <v>-3081804.177393634</v>
+        <v>-4188522.202036331</v>
       </c>
       <c r="K26">
-        <v>-3454183.663459043</v>
+        <v>-5048282.237125005</v>
       </c>
       <c r="L26">
-        <v>-100889.9441920754</v>
+        <v>-520955.8564460425</v>
       </c>
       <c r="M26">
-        <v>-3353293.719266967</v>
+        <v>-4527326.38067896</v>
       </c>
       <c r="N26">
         <v>0</v>
       </c>
       <c r="O26">
-        <v>356766.8945017974</v>
+        <v>204439.5535887314</v>
       </c>
       <c r="P26">
         <v>0</v>
       </c>
       <c r="Q26">
-        <v>356766.8945017974</v>
+        <v>204439.5535887314</v>
       </c>
       <c r="R26">
-        <v>171248.1093494162</v>
+        <v>98130.98571603181</v>
       </c>
       <c r="S26">
-        <v>1529725.584548512</v>
+        <v>1416167.262853925</v>
       </c>
       <c r="T26">
         <v>0</v>
       </c>
       <c r="U26">
-        <v>1529725.584548512</v>
+        <v>1416167.262853925</v>
       </c>
       <c r="V26">
-        <v>791535.5950568272</v>
+        <v>732776.3936392026</v>
       </c>
       <c r="W26">
         <v>-617770.0976527601</v>
@@ -2530,6 +2842,18 @@
       </c>
       <c r="Z26">
         <v>0</v>
+      </c>
+      <c r="AA26">
+        <v>2566810.223311379</v>
+      </c>
+      <c r="AB26">
+        <v>359353.4304468528</v>
+      </c>
+      <c r="AC26">
+        <v>2207456.792864526</v>
+      </c>
+      <c r="AD26">
+        <v>1059579.259909534</v>
       </c>
     </row>
   </sheetData>

</xml_diff>